<commit_message>
add other livestock manure management enteric
</commit_message>
<xml_diff>
--- a/Excel/3_1_Enteric_Feedlot_WIP_v01.xlsx
+++ b/Excel/3_1_Enteric_Feedlot_WIP_v01.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D45E6336-AC6C-4183-85D6-0B29325654B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33B25205-9B25-4383-BECB-E4CCC0C3112C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="480" yWindow="480" windowWidth="37350" windowHeight="19740" firstSheet="1" activeTab="6" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="735" yWindow="780" windowWidth="37665" windowHeight="20295" firstSheet="1" activeTab="1" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -174,10 +174,6 @@
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Unit">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Variable">_xlfn.LAMBDA("")</definedName>
     <definedName name="Common_SourceData.Common_SourceData_WetAndDryZones_Variation">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 1, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VARIATION OF SOURCE DATA:";"Added warm / cool temperate moist / dry - low frost and high temp classes to accommodate climate scenarios excluded by VEERG criteria.";"Fixed typo - Changed 'Fry' to 'Dry'."}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="CommonCropping_InputFunctions.CommonCropping_CalculateFractionResidueRemoved">_xlfn.LAMBDA(_xlpm.TotalResidue,_xlpm.AmountRemoved, (_xlpm.AmountRemoved * 10 ^ 3) / (_xlpm.TotalResidue * 10 ^ 3))</definedName>
-    <definedName name="CommonCropping_InputFunctions.CommonCropping_CalculateHarvestIndex">_xlfn.LAMBDA(_xlpm.CropType,_xlpm.CropTypeArray,_xlpm.ResidueCropRatioArray, 1 / (1 + Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.CropType, _xlpm.CropTypeArray, _xlpm.ResidueCropRatioArray)))</definedName>
-    <definedName name="CommonCropping_InputFunctions.CommonCropping_CalculateResidueCropRatio">_xlfn.LAMBDA(_xlpm.HarvestIndex, (1 - _xlpm.HarvestIndex) / _xlpm.HarvestIndex)</definedName>
-    <definedName name="CommonCropping_InputFunctions.CommonCropping_GetFracWET">_xlfn.LAMBDA(_xlpm.LeachingZone,_xlpm.ProductionSystem,_xlpm.LeachingZoneLookup,_xlpm.LeachingZoneFracWETLookup,_xlpm.ProductionSystemLookup,_xlpm.ProductionSystemFracWETLookup, _xlfn.LET(_xlpm.LeachingZoneFracWET, Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.LeachingZone, _xlpm.LeachingZoneLookup, _xlpm.LeachingZoneFracWETLookup), _xlpm.ProductionSystemFracWET, Common_InputFunctions.Utility_LookupValueInTableNumber(_xlpm.ProductionSystem, _xlpm.ProductionSystemLookup, _xlpm.ProductionSystemFracWETLookup), IF(_xlpm.LeachingZoneFracWET + _xlpm.ProductionSystemFracWET &gt; 0, 1, 0)))</definedName>
     <definedName name="CommonLivestock_InputFunctions.AverageLiveweightEndOfMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass,_xlpm.HeadAtStart,_xlpm.LiveweightAtStart,_xlpm.LiveweightGain, [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart) + [0]!CommonLivestock_InputFunctions.LivestockMovement_ProportionalAverageLiveweightRemainingAtEndOfMonth(_xlpm.Month, _xlpm.LivestockClass, _xlpm.HeadAtStart, _xlpm.LiveweightAtStart, _xlpm.LiveweightGain))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_AverageLiveweightAddedDuringMonth">_xlfn.LAMBDA(_xlpm.Month,_xlpm.LivestockClass, IFERROR([0]!CommonLivestock_InputFunctions.LivestockMovement_TotalLiveweightAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass) / [0]!CommonLivestock_InputFunctions.LivestockMovement_HeadAddedDuringMonth(_xlpm.Month, _xlpm.LivestockClass), 0))</definedName>
     <definedName name="CommonLivestock_InputFunctions.LivestockMovement_GetMovementLiveweightGain">_xlfn.LAMBDA(_xlpm.LivestockClass,_xlpm.MovementDate, _xlfn.LET(_xlpm.ym, TEXT(_xlpm.MovementDate, "yyyymm"), IFERROR(INDEX(_xlfn._xlws.FILTER(#REF!, (TEXT(#REF!, "yyyymm") = _xlpm.ym) * (#REF! = _xlpm.LivestockClass)), 1), "")))</definedName>
@@ -241,145 +237,6 @@
     <definedName name="Input_Cell_Pallets__Wood">#REF!</definedName>
     <definedName name="Input_Cell_Pallets_Plastic">#REF!</definedName>
     <definedName name="Input_Cell_Pallets_Wood">#REF!</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__1_TotalAnnualAtmosphericDepositionEmissions">_xlfn.LAMBDA(_xlpm.MMS_ATMOS,_xlpm.EF_N2O,_xlpm.C_N2O, (_xlpm.MMS_ATMOS * _xlpm.EF_N2O * _xlpm.C_N2O) * 10 ^ -3)</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__1_TotalAnnualAtmosphericDepositionEmissions_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"MMS_ATMOS","mass of N volatilised from MMS","kg N","Calculated from 4.1.1.5 (2)";"EF_N2O","nitrous oxide emission factor for atmospheric deposition","kg N2O-N/kg N","Constant";"C_N2O","factor to convert elemental mass of nitrous oxide to molecular mass","","Constant";"j","production system","","Input";"i","irrigation method","","Input";"r","rainfall zone","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__1_TotalAnnualAtmosphericDepositionEmissions_LatexEquation">_xlfn.LAMBDA("E_{N2O,ad}=(MMS_{ATMOS}\times EF_{N2O}\times C_{N2O})\times10^{-3}")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__1_TotalAnnualAtmosphericDepositionEmissions_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__1_TotalAnnualAtmosphericDepositionEmissions_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.5, Equation (1)")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__1_TotalAnnualAtmosphericDepositionEmissions_Title">_xlfn.LAMBDA("Total annual atmospheric deposition emissions from manure management")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__1_TotalAnnualAtmosphericDepositionEmissions_Unit">_xlfn.LAMBDA("t N2O")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__1_TotalAnnualAtmosphericDepositionEmissions_Variable">_xlfn.LAMBDA("E_N2Oad")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__2_VolatilisedNitrogenFromManureManagement">_xlfn.LAMBDA(_xlpm.MN_jmT,_xlpm.FracGASM_mT, _xlpm.MN_jmT * _xlpm.FracGASM_mT)</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__2_VolatilisedNitrogenFromManureManagement_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"MN_jmT","nitrogen in each treatment stage MMS (excluding MN_ijm13T2)","kg N","Calculated from 4.1.1.3 (2)(6)(8)";"FracGASM_mT","fraction of N volatilised in each MMS","(kg NH3-N + NOx-N)/kg N","Constant"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__2_VolatilisedNitrogenFromManureManagement_LatexEquation">_xlfn.LAMBDA("MMS_{ATMOS}=\sum_{j}\sum_{m}\sum_{T}(MN_{jmT}\times FracGASM_{mT})")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__2_VolatilisedNitrogenFromManureManagement_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__2_VolatilisedNitrogenFromManureManagement_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.5, Equation (2)")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__2_VolatilisedNitrogenFromManureManagement_Title">_xlfn.LAMBDA("Volatilised nitrogen from manure management")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__2_VolatilisedNitrogenFromManureManagement_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_Feedlot_AtmosphericDeposition_Equations.VEERG_4_1_1_5__2_VolatilisedNitrogenFromManureManagement_Variable">_xlfn.LAMBDA("MMS_ATMOS")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1">_xlfn.LAMBDA(_xlpm.MN_jmT23,_xlpm.EF_mT23,_xlpm.FracGASM_mT23,_xlpm.PF, (_xlpm.MN_jmT23 * (1 - _xlpm.EF_mT23 - _xlpm.FracGASM_mT23)) * _xlpm.PF)</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"MN_jmT23","mass of N in secondary and tertiary treatment MMS stages as calculated for manure management","kg N","Calculated from 4.1.1.3 (6)(8)";"EF_mT23","nitrous oxide emission factor for each MMS","kg N2O-N/kg N","Constant";"FracGASM_mT23","fraction of animal waste N volatilised in each MMS for each cattle group","(kg NH3-N + NOx-N)/kg N","Constant";"PF","fraction of manure applied to soil within the feedlot boundary","fraction","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1_LatexEquation">_xlfn.LAMBDA("MNSoil_{scope1}=\sum_{j}\sum_{m}\sum_{T}(MN_{jmT=2,3}\times(1-EF_{mT=2,3}-FracGASM_{mT=2,3}))\times PF")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.9, Equation (1)")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1_Title">_xlfn.LAMBDA("Mass of nitrogen applied to soils for scope 1 emissions")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__1_MassOfNitrogenAppliedToSoilsScope1_Variable">_xlfn.LAMBDA("MNSoil_scope1")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3">_xlfn.LAMBDA(_xlpm.MN_jmT23,_xlpm.EF_mT23,_xlpm.FracGASM_mT23,_xlpm.PF, (_xlpm.MN_jmT23 * (1 - _xlpm.EF_mT23 - _xlpm.FracGASM_mT23)) * (1 - _xlpm.PF))</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"MN_jmT23","mass of N in secondary and tertiary treatment MMS stages as calculated for manure management","kg N","Calculated from 4.1.1.3 (6)(8)";"EF_mT23","nitrous oxide emission factor for each MMS","kg N2O-N/kg N","Constant";"FracGASM_mT23","fraction of animal waste N volatilised in each MMS for each cattle group","(kg NH3-N + NOx-N)/kg N","Constant";"PF","fraction of manure applied to soil within the feedlot boundary","fraction","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3_LatexEquation">_xlfn.LAMBDA("MNSoil_{scope3}=\sum_{j}\sum_{m}\sum_{T}(MN_{jmT=2,3}\times(1-EF_{mT=2,3}-FracGASM_{mT=2,3}))\times(1-PF)")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.9, Equation (2)")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3_Title">_xlfn.LAMBDA("Mass of nitrogen applied to soils for scope 3 emissions")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_Feedlot_ManureAppliedToSoils_Equations.VEERG_4_1_1_9__2_MassOfNitrogenAppliedToSoilsScope3_Variable">_xlfn.LAMBDA("MNSoil_scope3")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__1_TotalAnnualMethaneEmissions">_xlfn.LAMBDA(_xlpm.D_j,_xlpm.M_jmT,_xlpm.N_j, (_xlpm.D_j * _xlpm.M_jmT * _xlpm.N_j) * 10 ^ -3)</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__1_TotalAnnualMethaneEmissions_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"D_j","length of stay of each cattle group","days","Input";"M_jmT","methane production from manure per cattle group, MMS, and treatment stage","kg CH4/head/day","Calculated from 4.1.1.1 (2)(3)(4)";"N_j","numbers of beef cattle in each group","head","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__1_TotalAnnualMethaneEmissions_LatexEquation">_xlfn.LAMBDA("{E}_{CH4}=\sum_{j}\sum_{m}\sum_{T}(D_{j}\times M_{jmT}\times N_{j})\times10^{-3}")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__1_TotalAnnualMethaneEmissions_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__1_TotalAnnualMethaneEmissions_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.1, Equation (1)")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__1_TotalAnnualMethaneEmissions_Title">_xlfn.LAMBDA("Total annual methane emissions from manure management")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__1_TotalAnnualMethaneEmissions_Unit">_xlfn.LAMBDA("t CH4")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__1_TotalAnnualMethaneEmissions_Variable">_xlfn.LAMBDA("E_CH4")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__2_Stage1MethaneProductionDrylot">_xlfn.LAMBDA(_xlpm.VS_j,_xlpm.BO,_xlpm.MMS_m5T1,_xlpm.MCF_im5,_xlpm.rho, _xlfn.LET(_xlpm.MCF_im5, IF(ISNUMBER(_xlpm.MCF_im5), _xlpm.MCF_im5, 0), _xlpm.VS_j * _xlpm.BO * _xlpm.MMS_m5T1 * _xlpm.MCF_im5 * _xlpm.rho))</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__2_Stage1MethaneProductionDrylot_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VS_j","volatile solid production from feedlot cattle in each group","kg/head/day","Calculated from 4.1.1.1 (5)";"BO","emissions potential","m3 CH4/kg VS","Constant";"MMS_m5T1","fraction of manure in primary system drylot MMS","fraction","Input";"MCF_im5","methane conversion factor for state and drylot system","fraction","Constant";"rho","density of methane","kg/m3","Constant";"i","state","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__2_Stage1MethaneProductionDrylot_Arguments_Method2">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VS_j","volatile solid production from feedlot cattle in each group","kg/head/day","Calculated from 4.1.1.1 (5)";"BO","emissions potential","m3 CH4/kg VS","Constant";"MMS_m5T1","fraction of manure in primary system drylot MMS","fraction","Input";"MCF_im5","methane conversion factor for state and drylot system","fraction","Constant";"rho","density of methane","kg/m3","Constant";"i","state","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__2_Stage1MethaneProductionDrylot_LatexEquation">_xlfn.LAMBDA("M_{jm=5,T=1}=VS_{j}\times BO\times MMS_{m=5,T=1}\times MCF_{im=5}\times \rho")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__2_Stage1MethaneProductionDrylot_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__2_Stage1MethaneProductionDrylot_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.1, Equation (2)")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__2_Stage1MethaneProductionDrylot_Title">_xlfn.LAMBDA("Production of methane in treatment stage 1 MMS")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__2_Stage1MethaneProductionDrylot_Unit">_xlfn.LAMBDA("kg CH4/head/day")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__2_Stage1MethaneProductionDrylot_Variable">_xlfn.LAMBDA("M_jm5T1")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__3_Stage2MethaneProduction">_xlfn.LAMBDA(_xlpm.VSL,_xlpm.VS_j,_xlpm.BO,_xlpm.MMS_mT2,_xlpm.MCF_im,_xlpm.rho, (1 - _xlpm.VSL) * _xlpm.VS_j * _xlpm.BO * _xlpm.MMS_mT2 * _xlpm.MCF_im * _xlpm.rho)</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__3_Stage2MethaneProduction_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(7, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VSL","fraction of volatile solids lost during storage in the primary system","fraction","Constant";"VS_j","volatile solid production from feedlot cattle in each group","kg/head/day","Calculated from 4.1.1.1 (5)";"BO","emissions potential","m3 CH4/kg VS","Constant";"MMS_mT2","fraction of manure in each secondary system","fraction","Input";"MCF_im","methane conversion factor for state and MMS","fraction","Constant";"rho","density of methane","kg/m3","Constant";"i","state","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__3_Stage2MethaneProduction_Arguments_Method2">_xlfn.LAMBDA(_xlfn.MAKEARRAY(7, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VSL","fraction of volatile solids lost during storage in the primary system","fraction","Constant";"VS_j","volatile solid production from feedlot cattle in each group","kg/head/day","Calculated from 4.1.1.1 (5)";"BO","emissions potential","m3 CH4/kg VS","Constant";"MMS_mT2","fraction of manure in each secondary system","fraction","Input";"MCF_im","methane conversion factor for mean annual temperature and MMS","fraction","Constant";"rho","density of methane","kg/m3","Constant";"i","Mean annual temperature","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__3_Stage2MethaneProduction_LatexEquation">_xlfn.LAMBDA("M_{jmT=2}=(1-VSL)\times VS_{j}\times BO\times MMS_{mT=2}\times MCF_{im}\times \rho")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__3_Stage2MethaneProduction_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__3_Stage2MethaneProduction_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.1, Equation (3)")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__3_Stage2MethaneProduction_Title">_xlfn.LAMBDA("Production of methane in treatment stage 2 MMS")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__3_Stage2MethaneProduction_Unit">_xlfn.LAMBDA("kg CH4/head/day")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__3_Stage2MethaneProduction_Variable">_xlfn.LAMBDA("M_jmT2")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__4_Stage3MethaneProductionAnaerobicLagoon">_xlfn.LAMBDA(_xlpm.VS_j,_xlpm.BO,_xlpm.MMS_m1T3,_xlpm.MCF_im1,_xlpm.rho, _xlpm.VS_j * _xlpm.BO * _xlpm.MMS_m1T3 * _xlpm.MCF_im1 * _xlpm.rho)</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__4_Stage3MethaneProductionAnaerobicLagoon_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VS_j","volatile solid production from feedlot cattle in each group j","kg/head/day","Calculated from 4.1.1.1 (5)";"BO","emissions potential","m3 CH4/kg VS","Constant";"MMS_m1T3","fraction of manure to tertiary anaerobic lagoon system","fraction","Input";"MCF_im1","methane conversion factor for state and anaerobic lagoon system","fraction","Constant";"rho","density of methane","kg/m3","Constant";"i","state","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__4_Stage3MethaneProductionAnaerobicLagoon_Arguments_Method2">_xlfn.LAMBDA(_xlfn.MAKEARRAY(6, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"VS_j","volatile solid production from feedlot cattle in each group j","kg/head/day","Calculated from 4.1.1.1 (5)";"BO","emissions potential","m3 CH4/kg VS","Constant";"MMS_m1T3","fraction of manure to tertiary anaerobic lagoon system","fraction","Input";"MCF_im1","methane conversion factor for mean annual temperature and anaerobic lagoon system","fraction","Constant";"rho","density of methane","kg/m3","Constant";"i","Mean annual temperature","","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__4_Stage3MethaneProductionAnaerobicLagoon_LatexEquation">_xlfn.LAMBDA("M_{jm=1,T=3}=VS_{j}\times BO\times MMS_{m=1,T=3}\times MCF_{im=1}\times \rho")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__4_Stage3MethaneProductionAnaerobicLagoon_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__4_Stage3MethaneProductionAnaerobicLagoon_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.1, Equation (4)")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__4_Stage3MethaneProductionAnaerobicLagoon_Title">_xlfn.LAMBDA("Production of methane in treatment stage 3 MMS")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__4_Stage3MethaneProductionAnaerobicLagoon_Unit">_xlfn.LAMBDA("kg CH4/head/day")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__4_Stage3MethaneProductionAnaerobicLagoon_Variable">_xlfn.LAMBDA("M_jm1T3")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__5_VolatileSolidProduction">_xlfn.LAMBDA(_xlpm.I_j,_xlpm.DMD_j,_xlpm.A, _xlpm.I_j * (1 - _xlpm.DMD_j) * (1 - _xlpm.A))</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__5_VolatileSolidProduction_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"I_j","dry matter intake for each group j","kg DM/head/day","Input";"DMD_j","dry matter digestibility for each group j","fraction","Input";"A","ash content of manure","fraction","Constant"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__5_VolatileSolidProduction_LatexEquation">_xlfn.LAMBDA("VS_{j}=I_{j}\times(1-DMD_{j})\times(1-A)")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__5_VolatileSolidProduction_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__5_VolatileSolidProduction_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.1, Equation (5)")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__5_VolatileSolidProduction_Title">_xlfn.LAMBDA("Volatile solid production")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__5_VolatileSolidProduction_Unit">_xlfn.LAMBDA("kg/head/day")</definedName>
-    <definedName name="MMS_Feedlot_Methane_Equations.VEERG_4_1_1_1__5_VolatileSolidProduction_Variable">_xlfn.LAMBDA("VS_j")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__1_TotalAnnualDirectNitrousOxideEmissions">_xlfn.LAMBDA(_xlpm.MN_jmT,_xlpm.EF_jm,_xlpm.C_N2O, SUMPRODUCT(_xlpm.MN_jmT, _xlpm.EF_jm, _xlpm.C_N2O) * 10 ^ -3)</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__1_TotalAnnualDirectNitrousOxideEmissions_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"MN_jmT","nitrogen per cattle group, MMS and treatment stage","kg N","Calculated from 4.1.1.3 (2)(6)(8)";"EF_jm","nitrous oxide emission factor for MMS","kg N2O-N/kg N","Constant";"C_N2O","factor to convert elemental mass of nitrous oxide to molecular mass","ratio","Constant"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__1_TotalAnnualDirectNitrousOxideEmissions_LatexEquation">_xlfn.LAMBDA("E_{N2O,dir}=\sum_{j}\sum_{m}\sum_{T}(MN_{jmT}\times EF_{jm}\times C_{N2O})\times10^{-3}")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__1_TotalAnnualDirectNitrousOxideEmissions_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__1_TotalAnnualDirectNitrousOxideEmissions_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.3, Equation (1)")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__1_TotalAnnualDirectNitrousOxideEmissions_Title">_xlfn.LAMBDA("Total annual direct nitrous oxide emissions from manure management systems")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__1_TotalAnnualDirectNitrousOxideEmissions_Unit">_xlfn.LAMBDA("t N2O")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__1_TotalAnnualDirectNitrousOxideEmissions_Variable">_xlfn.LAMBDA("E_N2Odir")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__2_Stage1NitrogenInMMSDrylot">_xlfn.LAMBDA(_xlpm.AE_j,_xlpm.MMS_jm5T1, _xlpm.AE_j * _xlpm.MMS_jm5T1)</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__2_Stage1NitrogenInMMSDrylot_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"AE_j","total nitrogen excreted by each cattle group","kg N","Calculated from 4.1.1.3 (3)";"MMS_jm5T1","fraction of manure in primary system drylot MMS","fraction","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__2_Stage1NitrogenInMMSDrylot_LatexEquation">_xlfn.LAMBDA("MN_{jm=5,T=1}=AE_{j}\times MMS_{jm=5,T=1}")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__2_Stage1NitrogenInMMSDrylot_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__2_Stage1NitrogenInMMSDrylot_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.3, Equation (2)")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__2_Stage1NitrogenInMMSDrylot_Title">_xlfn.LAMBDA("Nitrogen in treatment stage 1 MMS")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__2_Stage1NitrogenInMMSDrylot_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__2_Stage1NitrogenInMMSDrylot_Variable">_xlfn.LAMBDA("MN_jm5T1")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__3_AnnualNitrogenExcretion">_xlfn.LAMBDA(_xlpm.N_j,_xlpm.NE_j,_xlpm.D_j, _xlpm.N_j * _xlpm.NE_j * _xlpm.D_j)</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__3_AnnualNitrogenExcretion_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"N_j","number of cattle in each group","head","Input";"NE_j","nitrogen excretion","kg N/head/day","Calculated from 4.1.1.3 (4)";"D_j","duration of stay of cattle group","days","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__3_AnnualNitrogenExcretion_LatexEquation">_xlfn.LAMBDA("AE_{j}=N_{j}\times NE_{j}\times D_{j}")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__3_AnnualNitrogenExcretion_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__3_AnnualNitrogenExcretion_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.3, Equation (3)")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__3_AnnualNitrogenExcretion_Title">_xlfn.LAMBDA("Annual nitrogen excretion from each feedlot cattle group")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__3_AnnualNitrogenExcretion_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__3_AnnualNitrogenExcretion_Variable">_xlfn.LAMBDA("AE_j")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__4_NitrogenExcretionPerHead">_xlfn.LAMBDA(_xlpm.NI_j,_xlpm.NR_j, _xlpm.NI_j * (1 - _xlpm.NR_j))</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__4_NitrogenExcretionPerHead_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"NI_j","nitrogen intake","kg N/head/day","Calculated from 4.1.1.3 (5)";"NR_j","nitrogen retention expressed as a fraction of intake","fraction","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__4_NitrogenExcretionPerHead_LatexEquation">_xlfn.LAMBDA("NE_{j}=NI_{j}\times(1-NR_{j})")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__4_NitrogenExcretionPerHead_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__4_NitrogenExcretionPerHead_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.3, Equation (4)")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__4_NitrogenExcretionPerHead_Title">_xlfn.LAMBDA("Nitrogen excretion per head per day")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__4_NitrogenExcretionPerHead_Unit">_xlfn.LAMBDA("kg N/head/day")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__4_NitrogenExcretionPerHead_Variable">_xlfn.LAMBDA("NE_j")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__5_NitrogenIntake">_xlfn.LAMBDA(_xlpm.I_j,_xlpm.CP_j, _xlpm.I_j * _xlpm.CP_j / 6.25)</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__5_NitrogenIntake_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(3, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"I_j","dry matter intake","kg DM/head/day","Input";"CP_j","crude protein content of feed","fraction","Input";"6.25","factor for converting crude protein into nitrogen","ratio","Constant"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__5_NitrogenIntake_LatexEquation">_xlfn.LAMBDA("NI_{j}=I_{j}\times CP_{j}\div 6.25")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__5_NitrogenIntake_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__5_NitrogenIntake_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.3, Equation (5)")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__5_NitrogenIntake_Title">_xlfn.LAMBDA("Nitrogen intake of feedlot cattle")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__5_NitrogenIntake_Unit">_xlfn.LAMBDA("kg N/head/day")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__5_NitrogenIntake_Variable">_xlfn.LAMBDA("NI_j")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__6_Stage2NitrogenInMMS">_xlfn.LAMBDA(_xlpm.NT_jmT2,_xlpm.MMS_jmT2, _xlpm.NT_jmT2 * _xlpm.MMS_jmT2)</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__6_Stage2NitrogenInMMS_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"NT_jmT2","nitrogen transferred to secondary treatment MMS","kg N","Calculated from 4.1.1.3 (7)";"MMS_jmT2","fraction of manure in each secondary system","fraction","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__6_Stage2NitrogenInMMS_LatexEquation">_xlfn.LAMBDA("MN_{jm,T=2}=NT_{jm,T=2}\times MMS_{jm,T=2}")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__6_Stage2NitrogenInMMS_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__6_Stage2NitrogenInMMS_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.3, Equation (6)")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__6_Stage2NitrogenInMMS_Title">_xlfn.LAMBDA("Nitrogen in treatment stage 2 MMS")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__6_Stage2NitrogenInMMS_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__6_Stage2NitrogenInMMS_Variable">_xlfn.LAMBDA("MN_jmT2")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__7_NitrogenTransferredToStage2">_xlfn.LAMBDA(_xlpm.MN_jm5T1,_xlpm.FracGASM_m5,_xlpm.EF_m5,_xlpm.MN_jmT3, (_xlpm.MN_jm5T1 * (1 - _xlpm.FracGASM_m5 - _xlpm.EF_m5)) - _xlpm.MN_jmT3)</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__7_NitrogenTransferredToStage2_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(4, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"MN_jm5T1","nitrogen in MMS treatment stage 1","kg N","Calculated from 4.1.1.3 (2)";"FracGASM_m5","fraction of N volatilised from drylot MMS","fraction","Constant";"EF_m5","nitrous oxide emission factor for drylot MMS","kg N2O-N/kg N deposited","Constant";"MN_jmT3","nitrogen in MMS treatment stage 3","kg N","Calculated from 4.1.1.3 (8)"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__7_NitrogenTransferredToStage2_LatexEquation">_xlfn.LAMBDA("NT_{jm,T=2}=(MN_{jm=5,T=1}\times(1-FracGASM_{m=5}-EF_{m=5}))-MN_{jm,T=3}")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__7_NitrogenTransferredToStage2_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__7_NitrogenTransferredToStage2_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.3, Equation (7)")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__7_NitrogenTransferredToStage2_Title">_xlfn.LAMBDA("Nitrogen transferred to treatment stage 2 MMS")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__7_NitrogenTransferredToStage2_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__7_NitrogenTransferredToStage2_Variable">_xlfn.LAMBDA("NT_jmT2")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__8_Stage3NitrogenInMMSAnaerobicLagoon">_xlfn.LAMBDA(_xlpm.AE_j,_xlpm.MMS_jm1T3, _xlpm.AE_j * _xlpm.MMS_jm1T3)</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__8_Stage3NitrogenInMMSAnaerobicLagoon_Arguments">_xlfn.LAMBDA(_xlfn.MAKEARRAY(2, 4, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"AE_j","total nitrogen excreted by each cattle group","kg N","Calculated from 4.1.1.3 (3)";"MMS_jm1T3","fraction of manure to tertiary anaerobic lagoon system","fraction","Input"}, _xlpm.r, _xlpm.c))))</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__8_Stage3NitrogenInMMSAnaerobicLagoon_LatexEquation">_xlfn.LAMBDA("MN_{jm=1,T=3}=AE_{j}\times MMS_{jm=1,T=3}")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__8_Stage3NitrogenInMMSAnaerobicLagoon_NIRReference">_xlfn.LAMBDA("")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__8_Stage3NitrogenInMMSAnaerobicLagoon_Source">_xlfn.LAMBDA("VEERG 2026: 4.1.1.3, Equation (8)")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__8_Stage3NitrogenInMMSAnaerobicLagoon_Title">_xlfn.LAMBDA("Nitrogen in treatment stage 3 MMS")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__8_Stage3NitrogenInMMSAnaerobicLagoon_Unit">_xlfn.LAMBDA("kg N")</definedName>
-    <definedName name="MMS_Feedlot_N2ODirect_Equations.VEERG_4_1_1_3__8_Stage3NitrogenInMMSAnaerobicLagoon_Variable">_xlfn.LAMBDA("MN_jm1T3")</definedName>
     <definedName name="Range_LivestockStartingValues">#REF!</definedName>
     <definedName name="SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data">_xlfn.LAMBDA(_xlfn.MAKEARRAY(10, 7, _xlfn.LAMBDA(_xlpm.r,_xlpm.c, INDEX({"Feedlot type","Characteristic","Unit","2005-2009","2010-2014","2015-2019","2020-2023";"Domestic","Days on feed","days",70,70,70,75;"Domestic","Feed intake","kg DM/day",10,10,10.4,10.4;"Domestic","N retention","per cent of intake",21.1,20.4,20.4,20.4;"Mid-fed","Days on feed","days",115,115,120,150;"Mid-fed","Feed intake","kg DM/day",11.2,10.8,10.8,10.8;"Mid-fed","N retention","per cent of intake",12.5,12.7,12.7,12.7;"Long-fed","Days on feed","days",250,250,250,250;"Long-fed","Feed intake","kg DM/day",9,8.5,8.2,8.2;"Long-fed","N retention","per cent of intake",6.6,7,7,7}, _xlpm.r, _xlpm.c))))</definedName>
     <definedName name="SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Source">_xlfn.LAMBDA("VEERG 2026: Table A.1.1.2: Beef feedlot cattle - Animal characteristics")</definedName>
@@ -782,9 +639,6 @@
     <t>MMS m</t>
   </si>
   <si>
-    <t>Input - MMS - Feedlot</t>
-  </si>
-  <si>
     <t>kg dry matter / head  day</t>
   </si>
   <si>
@@ -933,9 +787,6 @@
   </si>
   <si>
     <t>Scope 1 source</t>
-  </si>
-  <si>
-    <t>4.1.1.1-2 Manure Methane</t>
   </si>
   <si>
     <t>Production system j</t>
@@ -1177,6 +1028,12 @@
   </si>
   <si>
     <t>💡 Below is a diagram that maps the equations used to calculate emissions and how they interact with each other.</t>
+  </si>
+  <si>
+    <t>3.1.1.1-2 Enteric Methane Beef Feedlot</t>
+  </si>
+  <si>
+    <t>Input - Feedlot</t>
   </si>
 </sst>
 </file>
@@ -3366,6 +3223,32 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Times New Roman"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFB2D498"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
         <b val="0"/>
         <i val="0"/>
         <strike val="0"/>
@@ -3483,32 +3366,6 @@
           <bgColor indexed="65"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <name val="Times New Roman"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <numFmt numFmtId="0" formatCode="General"/>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor indexed="64"/>
-          <bgColor rgb="FFB2D498"/>
-        </patternFill>
-      </fill>
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -6016,22 +5873,22 @@
     <tableColumn id="5" xr3:uid="{5034DCA1-F046-43BC-A94F-832832E6D634}" name="QLD" dataDxfId="59" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{186521AB-DFC2-4E3B-A674-A5382DCC5ACD}" name="NT" dataDxfId="4" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{186521AB-DFC2-4E3B-A674-A5382DCC5ACD}" name="NT" dataDxfId="58" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{95F9E197-F85F-424A-B68D-774604116729}" name="SA" dataDxfId="3" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{95F9E197-F85F-424A-B68D-774604116729}" name="SA" dataDxfId="57" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{A6DDF652-660B-4C41-982D-FECC3B1142AF}" name="VIC" dataDxfId="2" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{A6DDF652-660B-4C41-982D-FECC3B1142AF}" name="VIC" dataDxfId="56" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{5163E1D2-D984-4DBA-95A9-1667F628B2D9}" name="WA" dataDxfId="1" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{5163E1D2-D984-4DBA-95A9-1667F628B2D9}" name="WA" dataDxfId="55" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{A0E67108-978C-4849-A310-69F8E4739C6D}" name="TAS" dataDxfId="0" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{A0E67108-978C-4849-A310-69F8E4739C6D}" name="TAS" dataDxfId="54" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{27E929DD-0554-43B8-A58C-34B0A39F2EBA}" name="NIR definition" dataDxfId="58" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{27E929DD-0554-43B8-A58C-34B0A39F2EBA}" name="NIR definition" dataDxfId="53" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_MCF_Data(), Table_SourceData_Feedlot_MCF[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6147,49 +6004,49 @@
     <tableColumn id="1" xr3:uid="{25162FA7-7F7F-4C9C-8231-8FC51C581FD1}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6E2C0A27-43A1-4D92-B3A8-944DC7691E0A}" name="MAT" totalsRowDxfId="39" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{6E2C0A27-43A1-4D92-B3A8-944DC7691E0A}" name="MAT" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{BCEE406F-741C-4AB5-8347-FD3CEB5D1690}" name="MAP" totalsRowDxfId="38" totalsRowCellStyle="Content bold">
+    <tableColumn id="3" xr3:uid="{BCEE406F-741C-4AB5-8347-FD3CEB5D1690}" name="MAP" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{BF112A88-84E8-4D38-B54C-79713ED69470}" name="Frost days per year" totalsRowDxfId="37" totalsRowCellStyle="Content bold">
+    <tableColumn id="4" xr3:uid="{BF112A88-84E8-4D38-B54C-79713ED69470}" name="Frost days per year" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{DEDF2179-1AFD-46AA-97FF-2C7CC2C8F0A0}" name="Elevation" totalsRowDxfId="36" totalsRowCellStyle="Content bold">
+    <tableColumn id="5" xr3:uid="{DEDF2179-1AFD-46AA-97FF-2C7CC2C8F0A0}" name="Elevation" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{517703E3-C0ED-43E3-909F-4C1979577D3C}" name="MAP:PET" totalsRowDxfId="35" totalsRowCellStyle="Content bold">
+    <tableColumn id="6" xr3:uid="{517703E3-C0ED-43E3-909F-4C1979577D3C}" name="MAP:PET" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{666A24A7-650A-4B3E-982A-50311730DB7C}" name="Min temp" totalsRowDxfId="34" totalsRowCellStyle="Content bold">
+    <tableColumn id="7" xr3:uid="{666A24A7-650A-4B3E-982A-50311730DB7C}" name="Min temp" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{5604EDD5-66DF-4ECC-BCE6-DD11FD6DB4D6}" name="Max temp" totalsRowDxfId="33" totalsRowCellStyle="Content bold">
+    <tableColumn id="8" xr3:uid="{5604EDD5-66DF-4ECC-BCE6-DD11FD6DB4D6}" name="Max temp" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{6DA99F2D-CE18-432C-AB0D-72F425C17C5E}" name="Min rainfall" totalsRowDxfId="32" totalsRowCellStyle="Content bold">
+    <tableColumn id="9" xr3:uid="{6DA99F2D-CE18-432C-AB0D-72F425C17C5E}" name="Min rainfall" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{BC2916D3-A7D1-4722-A9DC-991CB2F62BD8}" name="Max rainfall" totalsRowDxfId="31" totalsRowCellStyle="Content bold">
+    <tableColumn id="10" xr3:uid="{BC2916D3-A7D1-4722-A9DC-991CB2F62BD8}" name="Max rainfall" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{1E64F234-4E02-4B45-A3A1-B18E3FFCFC37}" name="Min frost days" totalsRowDxfId="30" totalsRowCellStyle="Content bold">
+    <tableColumn id="11" xr3:uid="{1E64F234-4E02-4B45-A3A1-B18E3FFCFC37}" name="Min frost days" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{70F03B18-1155-4824-8E62-AE5F3FA2A39C}" name="Max frost days" totalsRowDxfId="29" totalsRowCellStyle="Content bold">
+    <tableColumn id="15" xr3:uid="{70F03B18-1155-4824-8E62-AE5F3FA2A39C}" name="Max frost days" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{C3AD9C66-0836-47F7-A64C-E903E6DAF5EE}" name="Min elevation" totalsRowDxfId="28" totalsRowCellStyle="Content bold">
+    <tableColumn id="12" xr3:uid="{C3AD9C66-0836-47F7-A64C-E903E6DAF5EE}" name="Min elevation" totalsRowDxfId="23" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{ED33ED06-8D20-47FE-B0B6-650FCDD420E2}" name="Max elevation" totalsRowDxfId="27" totalsRowCellStyle="Content bold">
+    <tableColumn id="16" xr3:uid="{ED33ED06-8D20-47FE-B0B6-650FCDD420E2}" name="Max elevation" totalsRowDxfId="22" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{3C28BB66-16DC-4BC9-BE53-61187001ECC2}" name="Min MAP:PET" totalsRowDxfId="26" totalsRowCellStyle="Content bold">
+    <tableColumn id="13" xr3:uid="{3C28BB66-16DC-4BC9-BE53-61187001ECC2}" name="Min MAP:PET" totalsRowDxfId="21" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="17" xr3:uid="{FFF015AD-8516-434B-A94C-11CB9D62F62D}" name="Max MAP:PET" totalsRowDxfId="25" totalsRowCellStyle="Content bold">
+    <tableColumn id="17" xr3:uid="{FFF015AD-8516-434B-A94C-11CB9D62F62D}" name="Max MAP:PET" totalsRowDxfId="20" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_ClimateZones_Data(), Table_SourceData_ClimateZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6207,7 +6064,7 @@
     <tableColumn id="1" xr3:uid="{2BBE1D44-5D3C-421E-B886-5F058BD82B23}" name="Climate zone" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{C3E0B2F3-1F7B-4FCF-B0F4-658087312975}" name="Wet or Dry Zone" totalsRowDxfId="24" totalsRowCellStyle="Content bold">
+    <tableColumn id="2" xr3:uid="{C3E0B2F3-1F7B-4FCF-B0F4-658087312975}" name="Wet or Dry Zone" totalsRowDxfId="19" totalsRowCellStyle="Content bold">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_WetAndDryZones_Data(), Table_SourceData_WetDryZones[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6311,7 +6168,7 @@
   </autoFilter>
   <tableColumns count="2">
     <tableColumn id="1" xr3:uid="{F2B173A3-CADE-4DCA-988D-39EE2392D8DB}" name="MMS"/>
-    <tableColumn id="2" xr3:uid="{67006656-167A-4452-9820-88D798B88ADD}" name="Symbol and MMS" dataDxfId="57" dataCellStyle="Content normal"/>
+    <tableColumn id="2" xr3:uid="{67006656-167A-4452-9820-88D798B88ADD}" name="Symbol and MMS" dataDxfId="52" dataCellStyle="Content normal"/>
   </tableColumns>
   <tableStyleInfo name="Equation table" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -6327,7 +6184,7 @@
     <tableColumn id="1" xr3:uid="{ACC4E2B3-A6FC-4D50-BE90-6D711BFC3B97}" name="Is in leaching zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{35F8284C-32FA-4320-AF32-3F44CCB77CF7}" name="FracWET" dataDxfId="23">
+    <tableColumn id="2" xr3:uid="{35F8284C-32FA-4320-AF32-3F44CCB77CF7}" name="FracWET" dataDxfId="18">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWET_Data(),Table_SourceData_FracWET[[#Headers],[Is in leaching zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6375,7 +6232,7 @@
     <tableColumn id="1" xr3:uid="{6328C683-420D-4EA6-AF9D-245995DC8FD1}" name="Irrigation type i">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{9E5FEA9D-8FB5-494C-9D24-0E6BFC0C6057}" name="FracWET" dataDxfId="22" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{9E5FEA9D-8FB5-494C-9D24-0E6BFC0C6057}" name="FracWET" dataDxfId="17" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_FracWETIrrigation_Data(), Table_SourceData_FracWETIrrigation[[#Headers],[Irrigation type i]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6393,7 +6250,7 @@
     <tableColumn id="1" xr3:uid="{FB787692-FEAA-422C-9A68-A116E1C1D839}" name="Climate zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{AFBB6C89-F456-4C86-80FD-B734DEFDFF30}" name="EFPRP" dataDxfId="21" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{AFBB6C89-F456-4C86-80FD-B734DEFDFF30}" name="EFPRP" dataDxfId="16" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_EFPastureRangeAndPaddock_Data(), Table_SourceData_EFPastureRangeAndPaddock[[#Headers],[Climate zone]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6411,7 +6268,7 @@
     <tableColumn id="1" xr3:uid="{E0DBFFCC-335E-4C29-BC47-5C2A3243CFF0}" name="Month">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{AC3827EF-FE9E-4E81-A7C7-95A7165D62C5}" name="Season" dataDxfId="20" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{AC3827EF-FE9E-4E81-A7C7-95A7165D62C5}" name="Season" dataDxfId="15" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MonthsToSeasons_Data(), Table_SourceData_Common_MonthToSeason[[#Headers],[Month]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6443,49 +6300,49 @@
     <tableColumn id="1" xr3:uid="{8C0CBC0D-B831-4C7E-9F24-0EE0037F3E6B}" name="Temperature zone">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{B6E0D171-2FBE-46A9-9B1F-1269E55C1B38}" name="MAT (ºC)" dataDxfId="19" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{B6E0D171-2FBE-46A9-9B1F-1269E55C1B38}" name="MAT (ºC)" dataDxfId="14" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{7FF50BBA-30EE-4E1A-9449-9265A1067683}" name="Anaerobic lagoon" dataDxfId="18" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{7FF50BBA-30EE-4E1A-9449-9265A1067683}" name="Anaerobic lagoon" dataDxfId="13" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{53654E61-5BB1-44D1-A97F-E38B4117F28F}" name="Digester / covered lagoons" dataDxfId="17" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{53654E61-5BB1-44D1-A97F-E38B4117F28F}" name="Digester / covered lagoons" dataDxfId="12" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{5736C277-B619-4577-BE61-C6F2CFEBBDF4}" name="Liquid systems" dataDxfId="16" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{5736C277-B619-4577-BE61-C6F2CFEBBDF4}" name="Liquid systems" dataDxfId="11" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{A4F5FCA7-77C5-40B2-BAC9-EBF849F5559B}" name="Daily spread" dataDxfId="15" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{A4F5FCA7-77C5-40B2-BAC9-EBF849F5559B}" name="Daily spread" dataDxfId="10" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{D7CABD47-531A-49AF-865F-934434068DEC}" name="Composting (passive windrow)" dataDxfId="14" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{D7CABD47-531A-49AF-865F-934434068DEC}" name="Composting (passive windrow)" dataDxfId="9" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{5B3C335A-BC58-40E9-8E75-96ED6CCF795D}" name="Solid storage" dataDxfId="13" dataCellStyle="Content normal">
+    <tableColumn id="8" xr3:uid="{5B3C335A-BC58-40E9-8E75-96ED6CCF795D}" name="Solid storage" dataDxfId="8" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{2D3901FD-AFED-45CA-9E32-1204AF6D4874}" name="Pit storage" dataDxfId="12" dataCellStyle="Content normal">
+    <tableColumn id="9" xr3:uid="{2D3901FD-AFED-45CA-9E32-1204AF6D4874}" name="Pit storage" dataDxfId="7" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="10" xr3:uid="{343A0FE7-0AA0-43C9-9A4F-02E9C242020A}" name="Deep litter" dataDxfId="11" dataCellStyle="Content normal">
+    <tableColumn id="10" xr3:uid="{343A0FE7-0AA0-43C9-9A4F-02E9C242020A}" name="Deep litter" dataDxfId="6" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{FAF69A1E-4587-4DCD-9535-2ECADB3A8A73}" name="Poultry manure with bedding" dataDxfId="10" dataCellStyle="Content normal">
+    <tableColumn id="11" xr3:uid="{FAF69A1E-4587-4DCD-9535-2ECADB3A8A73}" name="Poultry manure with bedding" dataDxfId="5" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{9D86AF5D-FDC1-4EE1-9D47-BA4BE96F619F}" name="Poultry manure without bedding" dataDxfId="9" dataCellStyle="Content normal">
+    <tableColumn id="12" xr3:uid="{9D86AF5D-FDC1-4EE1-9D47-BA4BE96F619F}" name="Poultry manure without bedding" dataDxfId="4" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{C15483D8-6A7E-4D26-B81F-096629F52A98}" name="Direct processing" dataDxfId="8" dataCellStyle="Content normal">
+    <tableColumn id="13" xr3:uid="{C15483D8-6A7E-4D26-B81F-096629F52A98}" name="Direct processing" dataDxfId="3" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{F82A14FE-E6A5-4C72-AE16-87CCAF66B3DB}" name="Direct application" dataDxfId="7" dataCellStyle="Content normal">
+    <tableColumn id="14" xr3:uid="{F82A14FE-E6A5-4C72-AE16-87CCAF66B3DB}" name="Direct application" dataDxfId="2" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{DBBFE03E-A035-4E39-B68B-F044C4B1E37F}" name="Pasture range and paddock" dataDxfId="6" dataCellStyle="Content normal">
+    <tableColumn id="15" xr3:uid="{DBBFE03E-A035-4E39-B68B-F044C4B1E37F}" name="Pasture range and paddock" dataDxfId="1" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{EE478F66-8602-4161-AB22-52FED9A026F5}" name="MAT raw" dataDxfId="5" dataCellStyle="Content normal">
+    <tableColumn id="16" xr3:uid="{EE478F66-8602-4161-AB22-52FED9A026F5}" name="MAT raw" dataDxfId="0" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(Common_SourceData.Common_SourceData_MCFTemperatureZone_Data(),Table_SourceData_Common_MCFTemperatureZone[[#Headers],[Temperature zone]],0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6530,22 +6387,22 @@
     <tableColumn id="1" xr3:uid="{FDCB848C-205F-48EA-BACF-F54BCD324E05}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{3306F917-B06C-4CC9-B1B1-D97D858E6DAA}" name="Nutrient analysis" dataDxfId="56" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{3306F917-B06C-4CC9-B1B1-D97D858E6DAA}" name="Nutrient analysis" dataDxfId="51" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{F162F7C2-B0FA-499A-BD58-855C4DF97FA8}" name="Unit" dataDxfId="55" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{F162F7C2-B0FA-499A-BD58-855C4DF97FA8}" name="Unit" dataDxfId="50" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{D395A9F5-9A85-4032-A7C1-EC470516DD87}" name="2010-2014" dataDxfId="54" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{D395A9F5-9A85-4032-A7C1-EC470516DD87}" name="2010-2014" dataDxfId="49" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{B149E561-7044-4839-B850-C751ABC364C9}" name="2015-2019" dataDxfId="53" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{B149E561-7044-4839-B850-C751ABC364C9}" name="2015-2019" dataDxfId="48" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{ECEB8E53-4880-43AE-9D36-F969D05BCB18}" name="2020-2023" dataDxfId="52" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{ECEB8E53-4880-43AE-9D36-F969D05BCB18}" name="2020-2023" dataDxfId="47" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{3B7FAEA4-08D7-48B2-9062-7D93639222CC}" name="2020-2023 Converted to fraction" dataDxfId="51" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{3B7FAEA4-08D7-48B2-9062-7D93639222CC}" name="2020-2023 Converted to fraction" dataDxfId="46" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DietProperties_Data(), Table_SourceData_Feedlot_DietProperties[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6568,22 +6425,22 @@
     <tableColumn id="1" xr3:uid="{96F6B4E3-E1EE-445F-9BCE-628B89FC3727}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6B651FD0-BCF6-4081-8A93-6B21A1D6CA99}" name="Characteristic" dataDxfId="50" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{6B651FD0-BCF6-4081-8A93-6B21A1D6CA99}" name="Characteristic" dataDxfId="45" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{3F266A2B-76EA-4E95-B049-75B8E4AB351F}" name="Unit" dataDxfId="49" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{3F266A2B-76EA-4E95-B049-75B8E4AB351F}" name="Unit" dataDxfId="44" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{15472767-3F72-4A65-88AC-C3242A8E1662}" name="2005-2009" dataDxfId="48" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{15472767-3F72-4A65-88AC-C3242A8E1662}" name="2005-2009" dataDxfId="43" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{5F74A8B9-7EFB-4457-8ADA-5E1ABA9DA889}" name="2010-2014" dataDxfId="47" dataCellStyle="Content normal">
+    <tableColumn id="5" xr3:uid="{5F74A8B9-7EFB-4457-8ADA-5E1ABA9DA889}" name="2010-2014" dataDxfId="42" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="6" xr3:uid="{E54F2812-2E8B-41EB-98A8-46890B5B4E13}" name="2015-2019" dataDxfId="46" dataCellStyle="Content normal">
+    <tableColumn id="6" xr3:uid="{E54F2812-2E8B-41EB-98A8-46890B5B4E13}" name="2015-2019" dataDxfId="41" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{88EEE0E3-F5D0-41DF-80EF-59472377C29A}" name="2020-2023" dataDxfId="45" dataCellStyle="Content normal">
+    <tableColumn id="7" xr3:uid="{88EEE0E3-F5D0-41DF-80EF-59472377C29A}" name="2020-2023" dataDxfId="40" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_AnimalCharacteristics_Data(), Table_SourceData_Feedlot_AnimalCharacteristics[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6601,7 +6458,7 @@
     <tableColumn id="1" xr3:uid="{9D472457-4D8B-44ED-9567-B889D058C2F1}" name="Feedlot type">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DurationOfStay_Data(), Table_SourceData_Feedlot_LengthOfStay[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{DA3DA009-634B-4C70-926B-C8FB255EB4DC}" name="Length of stay" dataDxfId="44" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{DA3DA009-634B-4C70-926B-C8FB255EB4DC}" name="Length of stay" dataDxfId="39" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_DurationOfStay_Data(), Table_SourceData_Feedlot_LengthOfStay[[#Headers],[Feedlot type]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6621,13 +6478,13 @@
     <tableColumn id="1" xr3:uid="{C80C08D8-3F48-4E18-98E3-9B53ACB6C6D9}" name="Treatment stage T">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{2BCD8589-5CB8-4ED1-AF2B-2866CEF779A8}" name="MMS m" dataDxfId="43" dataCellStyle="Content normal">
+    <tableColumn id="2" xr3:uid="{2BCD8589-5CB8-4ED1-AF2B-2866CEF779A8}" name="MMS m" dataDxfId="38" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{51E876CD-83B6-49C8-85DD-E2F427A3DCD0}" name="EF mT" dataDxfId="42" dataCellStyle="Content normal">
+    <tableColumn id="3" xr3:uid="{51E876CD-83B6-49C8-85DD-E2F427A3DCD0}" name="EF mT" dataDxfId="37" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{BEDEE6BB-8013-495A-8D74-2C8D37558C98}" name="NIR definition" dataDxfId="41" dataCellStyle="Content normal">
+    <tableColumn id="4" xr3:uid="{BEDEE6BB-8013-495A-8D74-2C8D37558C98}" name="NIR definition" dataDxfId="36" dataCellStyle="Content normal">
       <calculatedColumnFormula array="1">Common_InputFunctions.Utility_DisplayArrayInTable(SourceData_Feedlot.SourceData_Feedlot_NitrousOxideEFs_Data(), Table_SourceData_Feedlot_NO2EFs[[#Headers],[Treatment stage T]], 0)</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -6636,7 +6493,7 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}" name="Table_SourceData_Feedlot_FracGASMmT" displayName="Table_SourceData_Feedlot_FracGASMmT" ref="D112:G117" totalsRowShown="0" headerRowDxfId="40" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="12" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}" name="Table_SourceData_Feedlot_FracGASMmT" displayName="Table_SourceData_Feedlot_FracGASMmT" ref="D112:G117" totalsRowShown="0" headerRowDxfId="35" headerRowCellStyle="Content normal" dataCellStyle="Content normal">
   <autoFilter ref="D112:G117" xr:uid="{100A8309-C0D3-4638-A47B-72840A042D9A}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
@@ -6910,7 +6767,7 @@
 
 <file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
 <wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
-  <wetp:taskpane dockstate="right" visibility="0" width="503" row="4">
+  <wetp:taskpane dockstate="right" visibility="0" width="882" row="4">
     <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </wetp:taskpane>
 </wetp:taskpanes>
@@ -6962,7 +6819,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -7360,7 +7217,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="109" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="D1" s="110"/>
       <c r="E1" s="110"/>
@@ -7570,7 +7427,7 @@
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="112" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="E5" s="112"/>
       <c r="F5" s="112"/>
@@ -7637,7 +7494,7 @@
       <c r="A6" s="16"/>
       <c r="C6" s="1"/>
       <c r="D6" s="113" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E6" s="114"/>
       <c r="F6" s="114"/>
@@ -12636,7 +12493,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="102" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -12697,25 +12554,25 @@
       <c r="A6" s="16"/>
       <c r="C6" s="24"/>
       <c r="D6" s="100" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E6" s="100" t="s">
+        <v>139</v>
+      </c>
+      <c r="F6" s="100" t="s">
+        <v>140</v>
+      </c>
+      <c r="G6" s="100" t="s">
+        <v>130</v>
+      </c>
+      <c r="H6" s="100" t="s">
         <v>141</v>
       </c>
-      <c r="F6" s="100" t="s">
-        <v>142</v>
-      </c>
-      <c r="G6" s="100" t="s">
-        <v>132</v>
-      </c>
-      <c r="H6" s="100" t="s">
+      <c r="I6" s="100" t="s">
         <v>143</v>
       </c>
-      <c r="I6" s="100" t="s">
-        <v>145</v>
-      </c>
       <c r="J6" s="100" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="K6" s="24"/>
       <c r="L6" s="24"/>
@@ -12726,7 +12583,7 @@
       </c>
       <c r="C7" s="24"/>
       <c r="D7" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E7" s="98">
         <f>'3.1.1.1-2 Enteric Methane'!E67</f>
@@ -12749,7 +12606,7 @@
         <v>991.7664400000001</v>
       </c>
       <c r="J7" s="52" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="K7" s="24"/>
       <c r="L7" s="24"/>
@@ -12761,7 +12618,7 @@
       </c>
       <c r="C8" s="24"/>
       <c r="D8" s="31" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E8" s="25"/>
       <c r="F8" s="31"/>
@@ -12775,7 +12632,7 @@
         <v>991.7664400000001</v>
       </c>
       <c r="J8" s="93" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="K8" s="24"/>
       <c r="L8" s="24"/>
@@ -14670,7 +14527,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="63" t="s">
-        <v>81</v>
+        <v>183</v>
       </c>
       <c r="N1" s="54"/>
       <c r="O1" s="54"/>
@@ -14719,7 +14576,7 @@
         <v>Results</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14731,13 +14588,13 @@
       </c>
       <c r="D7" s="58"/>
       <c r="E7" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="F7" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="F7" s="39" t="s">
+      <c r="G7" s="39" t="s">
         <v>100</v>
-      </c>
-      <c r="G7" s="39" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="8" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14759,7 +14616,7 @@
         <v>100</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
@@ -14784,7 +14641,7 @@
         <v>250</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -14809,16 +14666,16 @@
     </row>
     <row r="13" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D13" s="58" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E13" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="F13" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="F13" s="39" t="s">
+      <c r="G13" s="39" t="s">
         <v>100</v>
-      </c>
-      <c r="G13" s="39" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="14" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14826,7 +14683,7 @@
         <v>4</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E14" s="50" cm="1">
         <f t="array" ref="E14">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_AnimalCharacteristics[Feedlot type] = E$13) * (Table_SourceData_Feedlot_AnimalCharacteristics[Characteristic] = $D$14), Table_SourceData_Feedlot_AnimalCharacteristics[2020-2023], "Not Found")</f>
@@ -14841,7 +14698,7 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I14" s="2"/>
       <c r="J14" s="2"/>
@@ -14853,7 +14710,7 @@
         <v>Constants - Feedlot</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E15" s="50" cm="1">
         <f t="array" ref="E15">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_DietProperties[Feedlot type] = E$13) * (Table_SourceData_Feedlot_DietProperties[Nutrient analysis] = $D$15), Table_SourceData_Feedlot_DietProperties[2020-2023 Converted to fraction], "Not Found")</f>
@@ -14868,7 +14725,7 @@
         <v>5.5</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -14880,7 +14737,7 @@
         <v>Constants - Livestock</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E16" s="50" cm="1">
         <f t="array" ref="E16">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_DietProperties[Feedlot type] = E$13) * (Table_SourceData_Feedlot_DietProperties[Nutrient analysis] = $D$16), Table_SourceData_Feedlot_DietProperties[2020-2023 Converted to fraction], "Not Found")</f>
@@ -14895,7 +14752,7 @@
         <v>24</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -14915,21 +14772,21 @@
         <v>Acknowledgements</v>
       </c>
       <c r="D18" s="58" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E18" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="F18" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="F18" s="39" t="s">
+      <c r="G18" s="39" t="s">
         <v>100</v>
-      </c>
-      <c r="G18" s="39" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D19" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E19" s="61" cm="1">
         <f t="array" ref="E19">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_AnimalCharacteristics[Feedlot type] = E$18) * (Table_SourceData_Feedlot_AnimalCharacteristics[Characteristic] = $D$19), Table_SourceData_Feedlot_AnimalCharacteristics[2020-2023], "Not Found")</f>
@@ -14944,13 +14801,13 @@
         <v>8.1999999999999993</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I19" s="2"/>
     </row>
     <row r="20" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D20" s="1" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="E20" s="61" cm="1">
         <f t="array" ref="E20">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_DietProperties[Feedlot type] = E$18) * (Table_SourceData_Feedlot_DietProperties[Nutrient analysis] = $D$20), Table_SourceData_Feedlot_DietProperties[2020-2023 Converted to fraction], "Not Found")</f>
@@ -14965,7 +14822,7 @@
         <v>5.5</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -14974,7 +14831,7 @@
     <row r="21" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="17"/>
       <c r="D21" s="1" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E21" s="61" cm="1">
         <f t="array" ref="E21">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_DietProperties[Feedlot type] = E$18) * (Table_SourceData_Feedlot_DietProperties[Nutrient analysis] = $D$21), Table_SourceData_Feedlot_DietProperties[2020-2023 Converted to fraction], "Not Found")</f>
@@ -14989,7 +14846,7 @@
         <v>24</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -15225,7 +15082,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>118</v>
+        <v>182</v>
       </c>
       <c r="K1"/>
     </row>
@@ -15239,7 +15096,7 @@
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
@@ -15249,7 +15106,7 @@
       <c r="J3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
@@ -15411,10 +15268,10 @@
         <v>Constants - Common</v>
       </c>
       <c r="D17" s="86" t="s">
+        <v>108</v>
+      </c>
+      <c r="M17" s="86" t="s">
         <v>109</v>
-      </c>
-      <c r="M17" s="86" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15423,30 +15280,30 @@
         <v>Acknowledgements</v>
       </c>
       <c r="D18" s="85" t="s">
+        <v>112</v>
+      </c>
+      <c r="M18" s="85" t="s">
         <v>113</v>
-      </c>
-      <c r="M18" s="85" t="s">
-        <v>114</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D19" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="E19" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="E19" s="39" t="s">
+      <c r="F19" s="39" t="s">
         <v>100</v>
       </c>
-      <c r="F19" s="39" t="s">
-        <v>101</v>
-      </c>
       <c r="M19" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="N19" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="N19" s="39" t="s">
+      <c r="O19" s="39" t="s">
         <v>100</v>
-      </c>
-      <c r="O19" s="39" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15488,38 +15345,38 @@
     </row>
     <row r="22" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D22" s="86" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="M22" s="86" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="23" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D23" s="85" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M23" s="85" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D24" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="E24" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="E24" s="39" t="s">
+      <c r="F24" s="39" t="s">
         <v>100</v>
       </c>
-      <c r="F24" s="39" t="s">
-        <v>101</v>
-      </c>
       <c r="M24" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="N24" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="N24" s="39" t="s">
+      <c r="O24" s="39" t="s">
         <v>100</v>
-      </c>
-      <c r="O24" s="39" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15560,38 +15417,38 @@
     <row r="26" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D27" s="86" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="M27" s="86" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="28" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D28" s="85" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="M28" s="85" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="29" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D29" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="E29" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="E29" s="39" t="s">
+      <c r="F29" s="39" t="s">
         <v>100</v>
       </c>
-      <c r="F29" s="39" t="s">
-        <v>101</v>
-      </c>
       <c r="M29" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="N29" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="N29" s="39" t="s">
+      <c r="O29" s="39" t="s">
         <v>100</v>
-      </c>
-      <c r="O29" s="39" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15631,38 +15488,38 @@
     <row r="31" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D32" s="86" t="s">
+        <v>169</v>
+      </c>
+      <c r="M32" s="86" t="s">
         <v>171</v>
-      </c>
-      <c r="M32" s="86" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="33" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D33" s="85" t="s">
+        <v>170</v>
+      </c>
+      <c r="M33" s="85" t="s">
         <v>172</v>
-      </c>
-      <c r="M33" s="85" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="34" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D34" s="49" t="s">
+        <v>98</v>
+      </c>
+      <c r="E34" s="49" t="s">
         <v>99</v>
       </c>
-      <c r="E34" s="49" t="s">
+      <c r="F34" s="49" t="s">
         <v>100</v>
       </c>
-      <c r="F34" s="49" t="s">
-        <v>101</v>
-      </c>
       <c r="M34" s="49" t="s">
+        <v>98</v>
+      </c>
+      <c r="N34" s="49" t="s">
         <v>99</v>
       </c>
-      <c r="N34" s="49" t="s">
+      <c r="O34" s="49" t="s">
         <v>100</v>
-      </c>
-      <c r="O34" s="49" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="35" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15825,23 +15682,23 @@
     <row r="51" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="52" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D52" s="86" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="53" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D53" s="85" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="54" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D54" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="E54" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="E54" s="39" t="s">
+      <c r="F54" s="39" t="s">
         <v>100</v>
-      </c>
-      <c r="F54" s="39" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="55" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15865,23 +15722,23 @@
     <row r="56" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="57" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D57" s="86" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
     </row>
     <row r="58" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D58" s="85" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="59" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D59" s="39" t="s">
+        <v>98</v>
+      </c>
+      <c r="E59" s="39" t="s">
         <v>99</v>
       </c>
-      <c r="E59" s="39" t="s">
+      <c r="F59" s="39" t="s">
         <v>100</v>
-      </c>
-      <c r="F59" s="39" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="60" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15905,38 +15762,38 @@
     <row r="61" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="62" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D62" s="86" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="M62" s="86" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="63" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D63" s="85" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="M63" s="85" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="64" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D64" s="49" t="s">
+        <v>98</v>
+      </c>
+      <c r="E64" s="49" t="s">
         <v>99</v>
       </c>
-      <c r="E64" s="49" t="s">
+      <c r="F64" s="49" t="s">
         <v>100</v>
       </c>
-      <c r="F64" s="49" t="s">
-        <v>101</v>
-      </c>
       <c r="M64" s="49" t="s">
+        <v>98</v>
+      </c>
+      <c r="N64" s="49" t="s">
         <v>99</v>
       </c>
-      <c r="N64" s="49" t="s">
+      <c r="O64" s="49" t="s">
         <v>100</v>
-      </c>
-      <c r="O64" s="49" t="s">
-        <v>101</v>
       </c>
     </row>
     <row r="65" spans="4:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15976,7 +15833,7 @@
     <row r="66" spans="4:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" spans="4:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D67" s="89" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E67" s="90">
         <f>SUM(D65:F65)</f>
@@ -15987,7 +15844,7 @@
         <v>t CH4</v>
       </c>
       <c r="M67" s="89" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="N67" s="90">
         <f>SUM(M65:O65)</f>
@@ -16060,7 +15917,7 @@
     <row r="71" spans="4:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="72" spans="4:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D72" s="45" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E72" s="45" cm="1">
         <f t="array" ref="E72">Common_Equations.Common_ConvertCH4ToCO2e(G69,G70)</f>
@@ -16071,7 +15928,7 @@
         <v>t CO2e</v>
       </c>
       <c r="M72" s="45" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="N72" s="45" cm="1">
         <f t="array" ref="N72">Common_Equations.Common_ConvertCH4ToCO2e(P69,P70)</f>
@@ -16222,7 +16079,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="2" spans="1:21" s="9" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -16445,13 +16302,13 @@
     <row r="25" spans="1:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="17"/>
       <c r="D25" s="6" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="G25" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="J25" s="6" t="s">
         <v>123</v>
-      </c>
-      <c r="J25" s="6" t="s">
-        <v>125</v>
       </c>
       <c r="M25" s="1"/>
     </row>
@@ -16466,10 +16323,10 @@
         <v>63</v>
       </c>
       <c r="G27" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="J27" s="37" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="M27" s="1"/>
     </row>
@@ -16487,7 +16344,7 @@
         <v>Crop</v>
       </c>
       <c r="J28" s="37" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="M28" s="1"/>
     </row>
@@ -16505,7 +16362,7 @@
         <v>Pasture</v>
       </c>
       <c r="J29" s="37" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="M29" s="1"/>
     </row>
@@ -16519,7 +16376,7 @@
         <v>Composting (passive windrow) (m=6)</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="M30" s="1"/>
     </row>
@@ -16533,7 +16390,7 @@
         <v>Direct application (m=13)</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="M31" s="1"/>
     </row>
@@ -16547,7 +16404,7 @@
         <v>Anaerobic lagoon (m=1)</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="M32" s="1"/>
     </row>
@@ -16576,10 +16433,10 @@
     </row>
     <row r="38" spans="4:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D38" s="37" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E38" s="37" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="M38" s="1"/>
     </row>
@@ -16657,25 +16514,25 @@
     </row>
     <row r="49" spans="4:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D49" s="37" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E49" s="37" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F49" s="37" t="s">
         <v>11</v>
       </c>
       <c r="G49" s="37" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="H49" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="I49" s="37" t="s">
         <v>95</v>
       </c>
-      <c r="I49" s="37" t="s">
+      <c r="J49" s="37" t="s">
         <v>96</v>
-      </c>
-      <c r="J49" s="37" t="s">
-        <v>97</v>
       </c>
       <c r="M49" s="24"/>
     </row>
@@ -16999,25 +16856,25 @@
     </row>
     <row r="66" spans="4:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D66" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="E66" s="37" t="s">
         <v>93</v>
-      </c>
-      <c r="E66" s="37" t="s">
-        <v>94</v>
       </c>
       <c r="F66" s="37" t="s">
         <v>11</v>
       </c>
       <c r="G66" s="37" t="s">
+        <v>94</v>
+      </c>
+      <c r="H66" s="37" t="s">
         <v>95</v>
       </c>
-      <c r="H66" s="37" t="s">
+      <c r="I66" s="37" t="s">
         <v>96</v>
       </c>
-      <c r="I66" s="37" t="s">
-        <v>97</v>
-      </c>
       <c r="J66" s="37" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="M66" s="24"/>
     </row>
@@ -17443,7 +17300,7 @@
     </row>
     <row r="88" spans="4:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D88" s="37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E88" s="37" t="s">
         <v>80</v>
@@ -17741,13 +17598,13 @@
     </row>
     <row r="100" spans="4:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D100" s="37" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E100" s="37" t="s">
         <v>80</v>
       </c>
       <c r="F100" s="37" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="G100" s="37" t="s">
         <v>78</v>
@@ -17887,13 +17744,13 @@
     </row>
     <row r="112" spans="4:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D112" s="95" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E112" s="95" t="s">
         <v>80</v>
       </c>
       <c r="F112" s="95" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="G112" s="95" t="s">
         <v>78</v>
@@ -20273,7 +20130,7 @@
     </row>
     <row r="142" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D142" s="37" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E142" s="37" t="s">
         <v>75</v>
@@ -20633,16 +20490,16 @@
     </row>
     <row r="186" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D186" s="37" t="s">
+        <v>117</v>
+      </c>
+      <c r="E186" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="F186" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="E186" s="37" t="s">
+      <c r="G186" s="37" t="s">
         <v>120</v>
-      </c>
-      <c r="F186" s="37" t="s">
-        <v>121</v>
-      </c>
-      <c r="G186" s="37" t="s">
-        <v>122</v>
       </c>
       <c r="H186" s="37" t="s">
         <v>25</v>
@@ -20963,7 +20820,7 @@
         <v>8</v>
       </c>
       <c r="E206" s="37" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="207" spans="4:8" x14ac:dyDescent="0.25">
@@ -20994,10 +20851,10 @@
     </row>
     <row r="212" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D212" s="37" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E212" s="37" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="213" spans="4:5" x14ac:dyDescent="0.25">
@@ -21143,49 +21000,49 @@
         <v>42</v>
       </c>
       <c r="E231" s="37" t="s">
+        <v>147</v>
+      </c>
+      <c r="F231" s="36" t="s">
+        <v>148</v>
+      </c>
+      <c r="G231" s="37" t="s">
         <v>149</v>
       </c>
-      <c r="F231" s="36" t="s">
+      <c r="H231" s="37" t="s">
         <v>150</v>
       </c>
-      <c r="G231" s="37" t="s">
+      <c r="I231" s="37" t="s">
         <v>151</v>
       </c>
-      <c r="H231" s="37" t="s">
+      <c r="J231" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="I231" s="37" t="s">
+      <c r="K231" s="37" t="s">
         <v>153</v>
       </c>
-      <c r="J231" s="37" t="s">
+      <c r="L231" s="37" t="s">
         <v>154</v>
       </c>
-      <c r="K231" s="37" t="s">
+      <c r="M231" s="37" t="s">
         <v>155</v>
       </c>
-      <c r="L231" s="37" t="s">
+      <c r="N231" s="37" t="s">
         <v>156</v>
       </c>
-      <c r="M231" s="37" t="s">
+      <c r="O231" s="37" t="s">
         <v>157</v>
       </c>
-      <c r="N231" s="37" t="s">
+      <c r="P231" s="37" t="s">
         <v>158</v>
       </c>
-      <c r="O231" s="37" t="s">
+      <c r="Q231" s="37" t="s">
+        <v>144</v>
+      </c>
+      <c r="R231" s="37" t="s">
         <v>159</v>
       </c>
-      <c r="P231" s="37" t="s">
+      <c r="S231" s="37" t="s">
         <v>160</v>
-      </c>
-      <c r="Q231" s="37" t="s">
-        <v>146</v>
-      </c>
-      <c r="R231" s="37" t="s">
-        <v>161</v>
-      </c>
-      <c r="S231" s="37" t="s">
-        <v>162</v>
       </c>
     </row>
     <row r="232" spans="4:19" x14ac:dyDescent="0.25">
@@ -23159,7 +23016,7 @@
 </file>
 
 <file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsAFwAbgAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ATABvAG8AawB1AHAALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQAsAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEwAbwBvAGsAdQBwACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVAAsACAAXABuACAAIAAgACAAIAAgACAAIABDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcABcAG4AIAAgACAAIAAgACAAIAAgACkALABcAG4AIAAgACAAIAAgACAAIAAgAEkARgAoAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAEYAcgBhAGMAVwBFAFQAIAArACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAD4AMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQwByAG8AcABUAHkAcABlACwAIABDAHIAbwBwAFQAeQBwAGUAQQByAHIAYQB5ACwAIABSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgADEALwAoADEAKwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAoAEMAcgBvAHAAVAB5AHAAZQAsACAAQwByAG8AcABUAHkAcABlAEEAcgByAGEAeQAsACAAUgBlAHMAaQBkAHUAZQBDAHIAbwBwAFIAYQB0AGkAbwBBAHIAcgBhAHkAKQApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBSAGUAcwBpAGQAdQBlAEMAcgBvAHAAUgBhAHQAaQBvAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAASABhAHIAdgBlAHMAdABJAG4AZABlAHgALABcAG4AIAAgACAAIAAoADEALQBIAGEAcgB2AGUAcwB0AEkAbgBkAGUAeAApAC8ASABhAHIAdgBlAHMAdABJAG4AZABlAHgAXABuACkAOwBcAG4AXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBDAGEAbABjAHUAbABhAHQAZQBGAHIAYQBjAHQAaQBvAG4AUgBlAHMAaQBkAHUAZQBSAGUAbQBvAHYAZQBkAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABvAHQAYQBsAFIAZQBzAGkAZAB1AGUALAAgAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQALABcAG4AIAAgACAAIAAoAEEAbQBvAHUAbgB0AFIAZQBtAG8AdgBlAGQAKgAxADAAXgAzACkALwAoAFQAbwB0AGEAbABSAGUAcwBpAGQAdQBlACoAMQAwAF4AMwApAFwAbgApACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAIgAsACIAdABlAHgAdAAiADoAIgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGwAbwBzAHQAIABpAG4AIAB0AGgAZQAgAHAAcgBpAG0AYQByAHkAIABNAE0AUwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGUAZQBkAGwAbwB0ACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGQAdQByAGkAbgBnACAAcwB0AG8AcgBhAGcAZQAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAFMATABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgA1ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB0AG8AIABlAGEAYwBoACAAdABlAHIAdABpAGEAcgB5ACAAcwB5AHMAdABlAG0AIABhAHMAcwB1AG0AZQBkACAAdABoAGEAdAAgADIAIABwAGUAcgAgAGMAZQBuAHQAIABpAHMAIAByAHUAbgAgAC0AIABvAGYAZgAgAGYAcgBvAG0AIAB0AGgAZQAgAGYAZQBlAGQAIABwAGEAZAAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIAB0AG8AIABlAGEAYwBoACAAdABlAHIAdABpAGEAcgB5ACAAcwB5AHMAdABlAG0AIABhAHMAcwB1AG0AZQBkACAAdABoAGEAdAAgADIAIABwAGUAcgAgAGMAZQBuAHQAIABpAHMAIAByAHUAbgAgAC0AIABvAGYAZgAgAGYAcgBvAG0AIAB0AGgAZQAgAGYAZQBlAGQAIABwAGEAZAAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATQBTAG0AMQBUADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAwADIAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AFwAbgBBAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBzAGgAIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAbQBhAG4AdQByAGUALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMQA2ACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABcAG4ATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwALgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBtADMAIABDAEgANAAgAC8AIABrAGcAIABWAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADIALgAzACAAQwBPAE4AUwBUAEEATgBUAFMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4AMQA5ACkAOwBcAG4AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFMAdABhAGcAZQAxAE0ATQBTAE8AcAB0AGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAxACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADIATQBNAFMATwBwAHQAaQBvAG4AcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwAgAE0ATQBTAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBTAHQAYQBnAGUAMwBNAE0AUwBPAHAAdABpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBMAGkAdgBlAHMAdABvAGMAawBDAGwAYQBzAHMAZQBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQB4AHAAbwByAHQAIABtAGkAZAAgAGYAZQBkAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAeABwAG8AcgB0ACAAbABvAG4AZwAgAGYAZQBkAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADEALgAxADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIAAoAGQAYQB5AHMAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAKABkAGEAeQBzACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADEAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgACgAZABhAHkAcwApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAXAAiACwAIABcACIATABlAG4AZwB0AGgAIABvAGYAIABTAHQAYQB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIAMQAtADgAMAAgAGQAYQB5AHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIAOAAxAC0AMgAwADAAIABkAGEAeQBzAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0AZgBlAGQAXAAiACwAIABcACIAMgAwADEAKwAgAGQAYQB5AHMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADIAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAAQQBuAGkAbQBhAGwAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEEAbgBpAG0AYQBsACAAYwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgAyADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEEAbgBpAG0AYQBsACAAYwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAHYAZQBkACAAZgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAcwAgAHQAbwAgAGEAIABzAGUAcABhAHIAYQB0AGUAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBhAG0AZQBkACAAJwBjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAJwAgAGMAbwBsAHUAbQBuACAALQAgAG8AcgBpAGcAaQBuAGEAbAAgAGgAYQBzACAAaABlAGEAZABlAHIAIAAnAFUAbgBpAHQAJwAgAHcAaABpAGMAaAAgAGMAbwB2AGUAcgBzACAAdAB3AG8AIABjAG8AbAB1AG0AbgBzACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMAAsACAANwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAXAAiACwAIABcACIAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAFwAIgAsACAAXAAiAFUAbgBpAHQAXAAiACwAIABcACIAMgAwADAANQAtADIAMAAwADkAXAAiACwAIABcACIAMgAwADEAMAAtADIAMAAxADQAXAAiACwAIABcACIAMgAwADEANQAtADIAMAAxADkAXAAiACwAIABcACIAMgAwADIAMAAtADIAMAAyADMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBEAGEAeQBzACAAbwBuACAAZgBlAGUAZABcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAANwAwACwAIAA3ADAALAAgADcAMAAsACAANwA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBGAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACwAIABcACIAawBnACAARABNAC8AZABhAHkAXAAiACwAIAAxADAALgAwACwAIAAxADAALgAwACwAIAAxADAALgA0ACwAIAAxADAALgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBOACAAcgBlAHQAZQBuAHQAaQBvAG4AXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0ACAAbwBmACAAaQBuAHQAYQBrAGUAXAAiACwAIAAyADEALgAxACwAIAAyADAALgA0ACwAIAAyADAALgA0ACwAIAAyADAALgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIARABhAHkAcwAgAG8AbgAgAGYAZQBlAGQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgADEAMQA1ACwAIAAxADEANQAsACAAMQAyADAALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGQAYQB5AFwAIgAsACAAMQAxAC4AMgAsACAAMQAwAC4AOAAsACAAMQAwAC4AOAAsACAAMQAwAC4AOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAE4AIAByAGUAdABlAG4AdABpAG8AbgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAIABvAGYAIABpAG4AdABhAGsAZQBcACIALAAgADEAMgAuADUALAAgADEAMgAuADcALAAgADEAMgAuADcALAAgADEAMgAuADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAGYAZQBkAFwAIgAsACAAXAAiAEQAYQB5AHMAIABvAG4AIABmAGUAZQBkAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIAAyADUAMAAsACAAMgA1ADAALAAgADIANQAwACwAIAAyADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0AZgBlAGQAXAAiACwAIABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGQAYQB5AFwAIgAsACAAOQAuADAALAAgADgALgA1ACwAIAA4AC4AMgAsACAAOAAuADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAGYAZQBkAFwAIgAsACAAXAAiAE4AIAByAGUAdABlAG4AdABpAG8AbgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAIABvAGYAIABpAG4AdABhAGsAZQBcACIALAAgADYALgA2ACwAIAA3AC4AMAAsACAANwAuADAALAAgADcALgAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4AMwA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAGkAZQB0ACAAcAByAG8AcABlAHIAdABpAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAGkAZQB0ACAAcAByAG8AcABlAHIAdABpAGUAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4AMwA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAGkAZQB0ACAAcAByAG8AcABlAHIAdABpAGUAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBDAG8AbgB2AGUAcgB0AGUAZAAgAHQAbwAgAGYAcgBhAGMAdABpAG8AbgAgAGMAbwBsAHUAbQBuACAAYQBuAGQAIABjAG8AbgB2AGUAcgB0AGUAZAAgAE4ARABGACAAYQBuAGQAIABFAHQAaABlAHIAIABlAHgAdAByAGEAYwB0ACAAdgBhAGwAdQBlAHMAIAB0AG8AIABmAHIAYQBjAHQAaQBvAG4AcwAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AdgBlAGQAIABmAGUAZQBkAGwAbwB0ACAAdAB5AHAAZQBzACAAdABvACAAYQAgAHMAZQBwAGEAcgBhAHQAZQAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAA4ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAZQBkAGwAbwB0ACAAdAB5AHAAZQBcACIALAAgAFwAIgBOAHUAdAByAGkAZQBuAHQAIABhAG4AYQBsAHkAcwBpAHMAXAAiACwAIABcACIAVQBuAGkAdABcACIALAAgAFwAIgAyADAAMAA1AC0AMgAwADAAOQBcACIALAAgAFwAIgAyADAAMQAwAC0AMgAwADEANABcACIALAAgAFwAIgAyADAAMQA1AC0AMgAwADEAOQBcACIALAAgAFwAIgAyADAAMgAwAC0AMgAwADIAMwBcACIALAAgAFwAIgBDAG8AbgB2AGUAcgB0AGUAZAAgAHQAbwAgAGYAcgBhAGMAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjAFwAIgAsACAAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjAFwAIgAsACAAXAAiAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAMAAuADEANAAsACAAMAAuADEANAAsACAAMAAuADEANAAsACAAMAAuADEANAAsACAAMAAuADEANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIATgBEAEYAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAMgAzAC4AMAAsACAAMgAyAC4AMAAsACAAMgAyAC4AMAAsACAAMgAyAC4AMAAsACAAMAAuADIAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIARQB0AGgAZQByACAARQB4AHQAcgBhAGMAdABcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAA0AC4ANQAsACAANAAuADUALAAgADQALgA4ACwAIAA0AC4AOAAsACAAMAAuADAANAA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAMAAuADEAMwAsACAAMAAuADEAMgA1ACwAIAAwAC4AMQAyACwAIAAwAC4AMQAyACwAIAAwAC4AMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIATgBEAEYAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAMgA0AC4AMAAsACAAMgAyAC4AMAAsACAAMgAyAC4AMAAsACAAMgAyAC4AMAAsACAAMAAuADIAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAEUAdABoAGUAcgAgAEUAeAB0AHIAYQBjAHQAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAANQAuADAALAAgADUALgAwACwAIAA1AC4AMAAsACAANQAuADAALAAgADAALgAwADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAEYAZQBkAFwAIgAsACAAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAEYAZQBkAFwAIgAsACAAXAAiAEMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAMAAuADEAMwAsACAAMAAuADEAMgA1ACwAIAAwAC4AMQAyACwAIAAwAC4AMQAyACwAIAAwAC4AMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBGAGUAZABcACIALAAgAFwAIgBOAEQARgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAAyADQALgAwACwAIAAyADQALgAwACwAIAAyADQALgAwACwAIAAyADQALgAwACwAIAAwAC4AMgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBGAGUAZABcACIALAAgAFwAIgBFAHQAaABlAHIAIABFAHgAdAByAGEAYwB0AFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADUALgAwACwAIAA1AC4AMAAsACAANQAuADUALAAgADUALgA1ACwAIAAwAC4AMAA1ADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADEALgA0ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAE0AQwBGAHMAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AVAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAbABvAHQAIAAtACAATQBDAEYAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADQAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQBUACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAE4AUwBXACAAdgBhAGwAdQBlAHMAIABmAG8AcgAgAEEAQwBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABOAFQAIABjAG8AbAB1AG0AbgAgAHQAaABhAHQAIABkAHUAcABsAGkAYwBhAHQAZQBzACAAUQBMAEQAIAB2AGEAbAB1AGUAcwAgAGEAcwAgAHAAZQByACAAYQBkAHYAaQBjAGUAIABmAHIAbwBtACAAcwBvAHUAcgBjAGUAIABkAGEAdABhACAAcAByAG8AdgBpAGQAZQByAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFQAQQBTACAAYwBvAGwAdQBtAG4AIAB0AGgAYQB0ACAAZAB1AHAAbABpAGMAYQB0AGUAcwAgAFYASQBDACAAdgBhAGwAdQBlAHMAIABhAHMAIABwAGUAcgAgAGEAZAB2AGkAYwBlACAAZgByAG8AbQAgAHMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHAAcgBvAHYAaQBkAGUAcgAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAAnAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAATQBNAFMAIABuAGEAbQBlAHMAIAB0AGgAYQB0ACAAbQBhAHQAYwBoACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMQAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAE4AUwBXAFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAFEATABEAFwAIgAsACAAXAAiAE4AVABcACIALAAgAFwAIgBTAEEAXAAiACwAIABcACIAVgBJAEMAXAAiACwAIABcACIAVwBBAFwAIgAsACAAXAAiAFQAQQBTAFwAIgAsACAAXAAiAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAGkAbQBhAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGwAbwB0ACAAKABGAGUAZQBkAHAAYQBkACkAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAzACwAIAAwAC4AMAAzACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAIAAoAFMAdABvAGMAawBwAGkAbABlACkAXAAiACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABQAGEAcwBzAGkAdgBlACAAVwBpAG4AZAByAG8AdwApAFwAIgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQByAHQAaQBhAHIAeQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIAAoAEUAZgBmAGwAdQBlAG4AdAAgAHAAbwBuAGQAKQBcACIALAAgADAALgA3ADUALAAgADAALgA3ADUALAAgADAALgA3ADcALAAgADAALgA3ADcALAAgADAALgA3ADUALAAgADAALgA3ADUALAAgADAALgA3ADcALAAgADAALgA3ADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADEALgA1ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgACgARQBGAG0AVAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAbABvAHQAIAAtACAATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAEUARgBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4ANQA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIAAoAEUARgBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAAnAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAATQBNAFMAIABuAGEAbQBlAHMAIAB0AGgAYQB0ACAAbQBhAHQAYwBoACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIABUAFwAIgAsACAAXAAiAE0ATQBTACAAbQBcACIALAAgAFwAIgBFAEYAbQBUACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAXAAiACwAIABcACIATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAaQBtAGEAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAbABvAHQAIAAoAEYAZQBlAGQAcABhAGQAKQBcACIALAAgADAALgAwADAANQA0ACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlACAAKABTAHQAbwBjAGsAcABpAGwAZQApAFwAIgAsACAAMAAuADAAMAA1ACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAUABhAHMAcwBpAHYAZQAgAFcAaQBuAGQAcgBvAHcAKQBcACIALAAgADAALgAwADEALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQByAHQAaQBhAHIAeQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIAAoAEUAZgBmAGwAdQBlAG4AdAAgAFAAbwBuAGQAKQBcACIALAAgADAALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADYAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTACAAKABGAHIAYQBjAEcAQQBTAE0AbQBUACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGUAZQBkAGwAbwB0ACAALQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABiAHkAIABNAE0AUwAgACgARgByAGEAYwBHAEEAUwBNAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADYAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTACAAKABGAHIAYQBjAEcAQQBTAE0AbQBUACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAAnAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAATQBNAFMAIABuAGEAbQBlAHMAIAB0AGgAYQB0ACAAbQBhAHQAYwBoACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEYAcgBhAGMARwBBAFMATQBtAFQAIAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACwAIABcACIATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAaQBtAGEAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAbABvAHQAIAAoAEYAZQBlAGQAcABhAGQAKQBcACIALAAgADAALgA2ACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlACAAKABTAHQAbwBjAGsAcABpAGwAZQApAFwAIgAsACAAMAAuADIANQAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAFAAYQBzAHMAaQB2AGUAIABXAGkAbgBkAHIAbwB3ACkAXAAiACwAIAAwAC4ANAAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgADAALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAHIAdABpAGEAcgB5AFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgARQBmAGYAbAB1AGUAbgB0ACAAcABvAG4AZAApAFwAIgAsACAAMAAuADMANQAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADEAOgAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4AMQAuADEALgAxACAATQBlAHQAaABvAGQAIAAxACAALQAgAE0AYQBuAHUAcgBlACAATQBlAHQAaABhAG4AZQAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAXABuAEUAXwBDAEgANABcAG4AdAAgAEMASAA0AFwAbgB7AEUAfQBfAHsAQwBIADQAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgARABfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAF8AewBqAG0AVAB9AFwAXAB0AGkAbQBlAHMAIABOAF8AewBqAH0AKQBcAFwAdABpAG0AZQBzADEAMABeAHsALQAzAH0AXABuAEQAXwBqACAAPQAgAGwAZQBuAGcAdABoACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAgADoAIABkAGEAeQBzAFwAbgBNAF8AagBtAFQAIAA9ACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABwAGUAcgAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACwAIABNAE0AUwAsACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADoAIABrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcAG4ATgBfAGoAIAA9ACAAbgB1AG0AYgBlAHIAcwAgAG8AZgAgAGIAZQBlAGYAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIAA6ACAAaABlAGEAZABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAARABfAGoALAAgAE0AXwBqAG0AVAAsACAATgBfAGoALABcAG4AIAAgACAAIAAoAEQAXwBqACAAKgAgAE0AXwBqAG0AVAAgACoAIABOAF8AagApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHQAIABDAEgANABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAHsARQB9AF8AewBDAEgANAB9AD0AXABcAHMAdQBtAF8AewBqAH0AXABcAHMAdQBtAF8AewBtAH0AXABcAHMAdQBtAF8AewBUAH0AKABEAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE0AXwB7AGoAbQBUAH0AXABcAHQAaQBtAGUAcwAgAE4AXwB7AGoAfQApAFwAXAB0AGkAbQBlAHMAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAXwBqAFwAIgAsAFwAIgBsAGUAbgBnAHQAaAAgAG8AZgAgAHMAdABhAHkAIABvAGYAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AXwBqAG0AVABcACIALABcACIAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABwAGUAcgAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACwAIABNAE0AUwAsACAAYQBuAGQAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQBcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgAxAC4AMQAuADEAIAAoADIAKQAoADMAKQAoADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBfAGoAXAAiACwAXAAiAG4AdQBtAGIAZQByAHMAIABvAGYAIABiAGUAZQBmACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwAFwAIgAsACAAXAAiAGgAZQBhAGQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXABuAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGUAdABoAGEAbgBlACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAXABuAE0AXwBqAG0ANQBUADEAXABuAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAbgBNAF8AewBqAG0APQA1ACwAVAA9ADEAfQA9AFYAUwBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBtAD0ANQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAgAE0AQwBGAF8AewBpAG0APQA1AH0AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcAG4AVgBTAF8AagAgAD0AIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIAA6ACAAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBCAE8AIAA9ACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAgADoAIABtADMAIABDAEgANAAvAGsAZwAgAFYAUwBcAG4ATQBNAFMAXwBtADUAVAAxACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAE0AQwBGAF8AaQBtADUAIAA9ACAAbQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAYQBuAGQAIABkAHIAeQBsAG8AdAAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4AcgBoAG8AIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAA6ACAAawBnAC8AbQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVgBTAF8AagAsACAAQgBPACwAIABNAE0AUwBfAG0ANQBUADEALAAgAE0AQwBGAF8AaQBtADUALAAgAHIAaABvACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAATQBDAEYAXwBpAG0ANQAsACAASQBGACgASQBTAE4AVQBNAEIARQBSACgATQBDAEYAXwBpAG0ANQApACwAIABNAEMARgBfAGkAbQA1ACwAIAAwACkALABcAG4AIAAgACAAIAAgACAAVgBTAF8AagAgACoAIABCAE8AIAAqACAATQBNAFMAXwBtADUAVAAxACAAKgAgAE0AQwBGAF8AaQBtADUAIAAqACAAcgBoAG8AXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABtAGUAdABoAGEAbgBlACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAG0ANQBUADEAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB7AGoAbQA9ADUALABUAD0AMQB9AD0AVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEIATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AG0APQA1ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQA9ADUAfQBcAFwAdABpAG0AZQBzACAAXABcAHIAaABvAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAUwBfAGoAXAAiACwAXAAiAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGcAcgBvAHUAcABcACIALAAgAFwAIgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4AMQAuADEALgAxACAAKAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIATwBcACIALABcACIAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbABcACIALAAgAFwAIgBtADMAIABDAEgANAAvAGsAZwAgAFYAUwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAF8AbQA1AFQAMQBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AIABkAHIAeQBsAG8AdAAgAE0ATQBTAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQwBGAF8AaQBtADUAXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHMAdABhAHQAZQAgAGEAbgBkACAAZAByAHkAbABvAHQAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgByAGgAbwBcACIALABcACIAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACwAIABcACIAawBnAC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAaQBcACIALAAgAFwAIgBzAHQAYQB0AGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAEEAcgBnAHUAbQBlAG4AdABzAF8ATQBlAHQAaABvAGQAMgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAF8AagBcACIALABcACIAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgAxAC4AMQAuADEAIAAoADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBPAFwAIgAsAFwAIgBlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgAsACAAXAAiAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBtADUAVAAxAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBDAEYAXwBpAG0ANQBcACIALABcACIAbQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAcwB0AGEAdABlACAAYQBuAGQAIABkAHIAeQBsAG8AdAAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAaABvAFwAIgAsAFwAIgBkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIALAAgAFwAIgBrAGcALwBtADMAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBpAFwAIgAsACAAXAAiAHMAdABhAHQAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcAG4ATQBfAGoAbQBUADIAXABuAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAbgBNAF8AewBqAG0AVAA9ADIAfQA9ACgAMQAtAFYAUwBMACkAXABcAHQAaQBtAGUAcwAgAFYAUwBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBtAFQAPQAyAH0AXABcAHQAaQBtAGUAcwAgAE0AQwBGAF8AewBpAG0AfQBcAFwAdABpAG0AZQBzACAAXABcAHIAaABvAFwAbgBWAFMATAAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGwAbwBzAHQAIABkAHUAcgBpAG4AZwAgAHMAdABvAHIAYQBnAGUAIABpAG4AIAB0AGgAZQAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAFYAUwBfAGoAIAA9ACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAOgAgAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcAG4AQgBPACAAPQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAIAA6ACAAbQAzACAAQwBIADQALwBrAGcAIABWAFMAXABuAE0ATQBTAF8AbQBUADIAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIABpAG4AIABlAGEAYwBoACAAcwBlAGMAbwBuAGQAYQByAHkAIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAE0AQwBGAF8AaQBtACAAPQAgAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAGEAbgBkACAATQBNAFMAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgByAGgAbwAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgADoAIABrAGcALwBtADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABWAFMATAAsACAAVgBTAF8AagAsACAAQgBPACwAIABNAE0AUwBfAG0AVAAyACwAIABNAEMARgBfAGkAbQAsACAAcgBoAG8ALABcAG4AIAAgACAAIAAoADEAIAAtACAAVgBTAEwAKQAgACoAIABWAFMAXwBqACAAKgAgAEIATwAgACoAIABNAE0AUwBfAG0AVAAyACAAKgAgAE0AQwBGAF8AaQBtACAAKgAgAHIAaABvAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAbQBUADIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADMAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwB7AGoAbQBUAD0AMgB9AD0AKAAxAC0AVgBTAEwAKQBcAFwAdABpAG0AZQBzACAAVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEIATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AG0AVAA9ADIAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQB9AFwAXAB0AGkAbQBlAHMAIABcAFwAcgBoAG8AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADcALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAEwAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGQAdQByAGkAbgBnACAAcwB0AG8AcgBhAGcAZQAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAUwBfAGoAXAAiACwAXAAiAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGcAcgBvAHUAcABcACIALAAgAFwAIgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4AMQAuADEALgAxACAAKAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIATwBcACIALABcACIAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbABcACIALAAgAFwAIgBtADMAIABDAEgANAAvAGsAZwAgAFYAUwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAF8AbQBUADIAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAZQBhAGMAaAAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBDAEYAXwBpAG0AXAAiACwAXAAiAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHMAdABhAHQAZQAgAGEAbgBkACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcgBoAG8AXAAiACwAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAGsAZwAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIAcwB0AGEAdABlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA3ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAUwBMAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAGwAbwBzAHQAIABkAHUAcgBpAG4AZwAgAHMAdABvAHIAYQBnAGUAIABpAG4AIAB0AGgAZQAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFMAXwBqAFwAIgAsAFwAIgB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAXAAiACwAIABcACIAawBnAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADEALgAxAC4AMQAgACgANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBCAE8AXAAiACwAXAAiAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwAXAAiACwAIABcACIAbQAzACAAQwBIADQALwBrAGcAIABWAFMAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAG0AVAAyAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAGUAYQBjAGgAIABzAGUAYwBvAG4AZABhAHIAeQAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQwBGAF8AaQBtAFwAIgAsAFwAIgBtAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABhAG4AZAAgAE0ATQBTAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAHIAaABvAFwAIgAsAFwAIgBkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIALAAgAFwAIgBrAGcALwBtADMAXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBpAFwAIgAsACAAXAAiAE0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIALAAgAFwAIgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBcAG4AUAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADMAIABNAE0AUwBcAG4ATQBfAGoAbQAxAFQAMwBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwB7AGoAbQA9ADEALABUAD0AMwB9AD0AVgBTAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEIATwBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AG0APQAxACwAVAA9ADMAfQBcAFwAdABpAG0AZQBzACAATQBDAEYAXwB7AGkAbQA9ADEAfQBcAFwAdABpAG0AZQBzACAAXABcAHIAaABvAFwAbgBWAFMAXwBqACAAPQAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgADoAIABrAGcALwBoAGUAYQBkAC8AZABhAHkAXABuAEIATwAgAD0AIABlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAOgAgAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAbgBNAE0AUwBfAG0AMQBUADMAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIAB0AG8AIAB0AGUAcgB0AGkAYQByAHkAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACAAcwB5AHMAdABlAG0AIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgBNAEMARgBfAGkAbQAxACAAPQAgAG0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAGEAbgBkACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4AcgBoAG8AIAA9ACAAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAIAA6ACAAawBnAC8AbQAzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVgBTAF8AagAsACAAQgBPACwAIABNAE0AUwBfAG0AMQBUADMALAAgAE0AQwBGAF8AaQBtADEALAAgAHIAaABvACwAXABuACAAIAAgACAAVgBTAF8AagAgACoAIABCAE8AIAAqACAATQBNAFMAXwBtADEAVAAzACAAKgAgAE0AQwBGAF8AaQBtADEAIAAqACAAcgBoAG8AXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAbQBlAHQAaABhAG4AZQAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMwAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AagBtADEAVAAzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AewBqAG0APQAxACwAVAA9ADMAfQA9AFYAUwBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABCAE8AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBtAD0AMQAsAFQAPQAzAH0AXABcAHQAaQBtAGUAcwAgAE0AQwBGAF8AewBpAG0APQAxAH0AXABcAHQAaQBtAGUAcwAgAFwAXAByAGgAbwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAFMAXwBqAFwAIgAsAFwAIgB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIABqAFwAIgAsACAAXAAiAGsAZwAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADQALgAxAC4AMQAuADEAIAAoADUAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQgBPAFwAIgAsAFwAIgBlAG0AaQBzAHMAaQBvAG4AcwAgAHAAbwB0AGUAbgB0AGkAYQBsAFwAIgAsACAAXAAiAG0AMwAgAEMASAA0AC8AawBnACAAVgBTAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBtADEAVAAzAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAHQAbwAgAHQAZQByAHQAaQBhAHIAeQAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEMARgBfAGkAbQAxAFwAIgAsAFwAIgBtAGUAdABoAGEAbgBlACAAYwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABzAHQAYQB0AGUAIABhAG4AZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgByAGgAbwBcACIALABcACIAZABlAG4AcwBpAHQAeQAgAG8AZgAgAG0AZQB0AGgAYQBuAGUAXAAiACwAIABcACIAawBnAC8AbQAzAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAaQBcACIALAAgAFwAIgBzAHQAYQB0AGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAF8ATQBlAHQAaABvAGQAMgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBTAF8AagBcACIALABcACIAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABpAG4AIABlAGEAYwBoACAAZwByAG8AdQBwACAAagBcACIALAAgAFwAIgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4AMQAuADEALgAxACAAKAA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIATwBcACIALABcACIAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbABcACIALAAgAFwAIgBtADMAIABDAEgANAAvAGsAZwAgAFYAUwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAF8AbQAxAFQAMwBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAAbQBhAG4AdQByAGUAIAB0AG8AIAB0AGUAcgB0AGkAYQByAHkAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBDAEYAXwBpAG0AMQBcACIALABcACIAbQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAYQBuAGQAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAcgBoAG8AXAAiACwAXAAiAGQAZQBuAHMAaQB0AHkAIABvAGYAIABtAGUAdABoAGEAbgBlAFwAIgAsACAAXAAiAGsAZwAvAG0AMwBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGkAXAAiACwAIABcACIATQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBWAG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAIABwAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgBWAFMAXwBqAFwAbgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXABuAFYAUwBfAHsAagB9AD0ASQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAKAAxAC0ARABNAEQAXwB7AGoAfQApAFwAXAB0AGkAbQBlAHMAKAAxAC0AQQApAFwAbgBJAF8AagAgAD0AIABkAHIAeQAgAG0AYQB0AHQAZQByACAAaQBuAHQAYQBrAGUAIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIAA6ACAAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBEAE0ARABfAGoAIAA9ACAAZAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAIABmAG8AcgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgBBACAAPQAgAGEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEkAXwBqACwAIABEAE0ARABfAGoALAAgAEEALABcAG4AIAAgACAAIABJAF8AagAgACoAIAAoADEAIAAtACAARABNAEQAXwBqACkAIAAqACAAKAAxACAALQAgAEEAKQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZAAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA1ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAFMAXwB7AGoAfQA9AEkAXwB7AGoAfQBcAFwAdABpAG0AZQBzACgAMQAtAEQATQBEAF8AewBqAH0AKQBcAFwAdABpAG0AZQBzACgAMQAtAEEAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAF8AagBcACIALABcACIAZAByAHkAIABtAGEAdAB0AGUAcgAgAGkAbgB0AGEAawBlACAAZgBvAHIAIABlAGEAYwBoACAAZwByAG8AdQBwACAAagBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAE0ARABfAGoAXAAiACwAXAAiAGQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5ACAAZgBvAHIAIABlAGEAYwBoACAAZwByAG8AdQBwACAAagBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAFwAIgAsAFwAIgBhAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4AMQA6ACAAQgBlAGUAZgAgAEYAZQBlAGQAbABvAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgAxAC4AMQAuADkAIABNAGEAbgB1AHIAZQAgAEEAcABwAGwAaQBlAGQAIAB0AG8AIABTAG8AaQBsAHMAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBcAG4ATQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGEAcABwAGwAaQBlAGQAIAB0AG8AIABzAG8AaQBsAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADEAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ATQBOAFMAbwBpAGwAXwBzAGMAbwBwAGUAMQBcAG4AawBnACAATgBcAG4ATQBOAFMAbwBpAGwAXwB7AHMAYwBvAHAAZQAxAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAPQAyACwAMwB9AFwAXAB0AGkAbQBlAHMAKAAxAC0ARQBGAF8AewBtAFQAPQAyACwAMwB9AC0ARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAPQAyACwAMwB9ACkAKQBcAFwAdABpAG0AZQBzACAAUABGAFwAbgBNAE4AXwBqAG0AVAAyADMAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIABpAG4AIABzAGUAYwBvAG4AZABhAHIAeQAgAGEAbgBkACAAdABlAHIAdABpAGEAcgB5ACAAdAByAGUAYQB0AG0AZQBuAHQAIABNAE0AUwAgAHMAdABhAGcAZQBzACAAYQBzACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAbwByACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAOgAgAGsAZwAgAE4AXABuAEUARgBfAG0AVAAyADMAIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcAG4ARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAMwAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABhAG4AaQBtAGEAbAAgAHcAYQBzAHQAZQAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABpAG4AIABlAGEAYwBoACAATQBNAFMAIABmAG8AcgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAgADoAIAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXABuAFAARgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGEAcABwAGwAaQBlAGQAIAB0AG8AIABzAG8AaQBsACAAdwBpAHQAaABpAG4AIAB0AGgAZQAgAGYAZQBlAGQAbABvAHQAIABiAG8AdQBuAGQAYQByAHkAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBfAGoAbQBUADIAMwAsACAARQBGAF8AbQBUADIAMwAsACAARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAMwAsACAAUABGACwAXABuACAAIAAgACAAKABNAE4AXwBqAG0AVAAyADMAIAAqACAAKAAxACAALQAgAEUARgBfAG0AVAAyADMAIAAtACAARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAMwApACkAIAAqACAAUABGAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAxACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AUwBvAGkAbABfAHMAYwBvAHAAZQAxAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADkALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AUwBvAGkAbABfAHsAcwBjAG8AcABlADEAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAA9ADIALAAzAH0AXABcAHQAaQBtAGUAcwAoADEALQBFAEYAXwB7AG0AVAA9ADIALAAzAH0ALQBGAHIAYQBjAEcAQQBTAE0AXwB7AG0AVAA9ADIALAAzAH0AKQApAFwAXAB0AGkAbQBlAHMAIABQAEYAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATgBfAGoAbQBUADIAMwBcACIALABcACIAbQBhAHMAcwAgAG8AZgAgAE4AIABpAG4AIABzAGUAYwBvAG4AZABhAHIAeQAgAGEAbgBkACAAdABlAHIAdABpAGEAcgB5ACAAdAByAGUAYQB0AG0AZQBuAHQAIABNAE0AUwAgAHMAdABhAGcAZQBzACAAYQBzACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAbwByACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0AFwAIgAsAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADEALgAxAC4AMwAgACgANgApACgAOAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBtAFQAMgAzAFwAIgAsAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwBcACIALABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMARwBBAFMATQBfAG0AVAAyADMAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAGEAbgBpAG0AYQBsACAAdwBhAHMAdABlACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgAGYAbwByACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwAFwAIgAsAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAIAB3AGkAdABoAGkAbgAgAHQAaABlACAAZgBlAGUAZABsAG8AdAAgAGIAbwB1AG4AZABhAHIAeQBcACIALABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBcAG4ATQBhAHMAcwAgAG8AZgAgAG4AaQB0AHIAbwBnAGUAbgAgAGEAcABwAGwAaQBlAGQAIAB0AG8AIABzAG8AaQBsAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ATQBOAFMAbwBpAGwAXwBzAGMAbwBwAGUAMwBcAG4AawBnACAATgBcAG4ATQBOAFMAbwBpAGwAXwB7AHMAYwBvAHAAZQAzAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAPQAyACwAMwB9AFwAXAB0AGkAbQBlAHMAKAAxAC0ARQBGAF8AewBtAFQAPQAyACwAMwB9AC0ARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAPQAyACwAMwB9ACkAKQBcAFwAdABpAG0AZQBzACgAMQAtAFAARgApAFwAbgBNAE4AXwBqAG0AVAAyADMAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIABpAG4AIABzAGUAYwBvAG4AZABhAHIAeQAgAGEAbgBkACAAdABlAHIAdABpAGEAcgB5ACAAdAByAGUAYQB0AG0AZQBuAHQAIABNAE0AUwAgAHMAdABhAGcAZQBzACAAYQBzACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAbwByACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAOgAgAGsAZwAgAE4AXABuAEUARgBfAG0AVAAyADMAIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABlAGEAYwBoACAATQBNAFMAIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcAG4ARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAMwAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABhAG4AaQBtAGEAbAAgAHcAYQBzAHQAZQAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABpAG4AIABlAGEAYwBoACAATQBNAFMAIABmAG8AcgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAgADoAIAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXABuAFAARgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGEAcABwAGwAaQBlAGQAIAB0AG8AIABzAG8AaQBsACAAdwBpAHQAaABpAG4AIAB0AGgAZQAgAGYAZQBlAGQAbABvAHQAIABiAG8AdQBuAGQAYQByAHkAIAA6ACAAZgByAGEAYwB0AGkAbwBuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBfAGoAbQBUADIAMwAsACAARQBGAF8AbQBUADIAMwAsACAARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAMwAsACAAUABGACwAXABuACAAIAAgACAAKABNAE4AXwBqAG0AVAAyADMAIAAqACAAKAAxACAALQAgAEUARgBfAG0AVAAyADMAIAAtACAARgByAGEAYwBHAEEAUwBNAF8AbQBUADIAMwApACkAIAAqACAAKAAxACAALQAgAFAARgApAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AZwBlAG4AIABhAHAAcABsAGkAZQBkACAAdABvACAAcwBvAGkAbABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzACAAZQBtAGkAcwBzAGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AUwBvAGkAbABfAHMAYwBvAHAAZQAzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADkALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AUwBvAGkAbABfAHsAcwBjAG8AcABlADMAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAA9ADIALAAzAH0AXABcAHQAaQBtAGUAcwAoADEALQBFAEYAXwB7AG0AVAA9ADIALAAzAH0ALQBGAHIAYQBjAEcAQQBTAE0AXwB7AG0AVAA9ADIALAAzAH0AKQApAFwAXAB0AGkAbQBlAHMAKAAxAC0AUABGACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATgBfAGoAbQBUADIAMwBcACIALABcACIAbQBhAHMAcwAgAG8AZgAgAE4AIABpAG4AIABzAGUAYwBvAG4AZABhAHIAeQAgAGEAbgBkACAAdABlAHIAdABpAGEAcgB5ACAAdAByAGUAYQB0AG0AZQBuAHQAIABNAE0AUwAgAHMAdABhAGcAZQBzACAAYQBzACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAbwByACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0AFwAIgAsAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADEALgAxAC4AMwAgACgANgApACgAOAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAXwBtAFQAMgAzAFwAIgAsAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGUAYQBjAGgAIABNAE0AUwBcACIALABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMARwBBAFMATQBfAG0AVAAyADMAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAGEAbgBpAG0AYQBsACAAdwBhAHMAdABlACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgAGYAbwByACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwAFwAIgAsAFwAIgAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXAAiACwAIABcACIAQwBvAG4AcwB0AGEAbgB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEYAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAYQBwAHAAbABpAGUAZAAgAHQAbwAgAHMAbwBpAGwAIAB3AGkAdABoAGkAbgAgAHQAaABlACAAZgBlAGUAZABsAG8AdAAgAGIAbwB1AG4AZABhAHIAeQBcACIALABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgAxADoAIABCAGUAZQBmACAARgBlAGUAZABsAG8AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4ANAAuADEALgAxAC4ANQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABNAGEAbgB1AHIAZQAgAEEAdABtAG8AcwBwAGgAZQByAGkAYwAgAEQAZQBwAG8AcwBpAHQAaQBvAG4AIABCAGUAZQBmACAARgBlAGUAZABsAG8AdABcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMAXABuAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAYQB0AG0AbwBzAHAAaABlAHIAaQBjACAAZABlAHAAbwBzAGkAdABpAG8AbgAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcAG4ARQBfAE4AMgBPAGEAZABcAG4AdAAgAE4AMgBPAFwAbgBFAF8AewBOADIATwAsAGEAZAB9AD0AKABNAE0AUwBfAHsAQQBUAE0ATwBTAH0AXABcAHQAaQBtAGUAcwAgAEUARgBfAHsATgAyAE8AfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQApAFwAXAB0AGkAbQBlAHMAMQAwAF4AewAtADMAfQBcAG4ATQBNAFMAXwBBAFQATQBPAFMAIAA9ACAAbQBhAHMAcwAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAATQBNAFMAIAA6ACAAawBnACAATgBcAG4ARQBGAF8ATgAyAE8AIAA9ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABhAHQAbQBvAHMAcABoAGUAcgBpAGMAIABkAGUAcABvAHMAaQB0AGkAbwBuACAAOgAgAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXABuAEMAXwBOADIATwAgAD0AIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzACAAOgAgAHIAYQB0AGkAbwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATQBTAF8AQQBUAE0ATwBTACwAIABFAEYAXwBOADIATwAsACAAQwBfAE4AMgBPACwAXABuACAAIAAgACAAKABNAE0AUwBfAEEAVABNAE8AUwAgACoAIABFAEYAXwBOADIATwAgACoAIABDAF8ATgAyAE8AKQAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABhAHQAbQBvAHMAcABoAGUAcgBpAGMAIABkAGUAcABvAHMAaQB0AGkAbwBuACAAZQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAAbQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8ATgAyAE8AYQBkAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAE4AMgBPAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADUALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsATgAyAE8ALABhAGQAfQA9ACgATQBNAFMAXwB7AEEAVABNAE8AUwB9AFwAXAB0AGkAbQBlAHMAIABFAEYAXwB7AE4AMgBPAH0AXABcAHQAaQBtAGUAcwAgAEMAXwB7AE4AMgBPAH0AKQBcAFwAdABpAG0AZQBzADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBNAFMAXwBBAFQATQBPAFMAXAAiACwAXAAiAG0AYQBzAHMAIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAZgByAG8AbQAgAE0ATQBTAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4AMQAuADEALgA1ACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAE4AMgBPAFwAIgAsAFwAIgBuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGEAdABtAG8AcwBwAGgAZQByAGkAYwAgAGQAZQBwAG8AcwBpAHQAaQBvAG4AXAAiACwAIABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAXwBOADIATwBcACIALABcACIAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIALAAgAFwAIgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAGoAXAAiACwAIABcACIAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAaQBcACIALAAgAFwAIgBpAHIAcgBpAGcAYQB0AGkAbwBuACAAbQBlAHQAaABvAGQAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgByAFwAIgAsACAAXAAiAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiACwAIABcACIAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABcAG4AVgBvAGwAYQB0AGkAbABpAHMAZQBkACAAbgBpAHQAcgBvAGcAZQBuACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdABcAG4ATQBNAFMAXwBBAFQATQBPAFMAXABuAGsAZwAgAE4AXABuAE0ATQBTAF8AewBBAFQATQBPAFMAfQA9AFwAXABzAHUAbQBfAHsAagB9AFwAXABzAHUAbQBfAHsAbQB9AFwAXABzAHUAbQBfAHsAVAB9ACgATQBOAF8AewBqAG0AVAB9AFwAXAB0AGkAbQBlAHMAIABGAHIAYQBjAEcAQQBTAE0AXwB7AG0AVAB9ACkAXABuAE0ATgBfAGoAbQBUACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAGUAYQBjAGgAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAE0ATQBTACAAKABlAHgAYwBsAHUAZABpAG4AZwAgAE0ATgBfAGkAagBtADEAMwBUADIAKQAgADoAIABrAGcAIABOAFwAbgBGAHIAYQBjAEcAQQBTAE0AXwBtAFQAIAA9ACAAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGkAbgAgAGUAYQBjAGgAIABNAE0AUwAgADoAIAAoAGsAZwAgAE4ASAAzAC0ATgAgACsAIABOAE8AeAAtAE4AKQAvAGsAZwAgAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBfAGoAbQBUACwAIABGAHIAYQBjAEcAQQBTAE0AXwBtAFQALABcAG4AIAAgACAAIABNAE4AXwBqAG0AVAAgACoAIABGAHIAYQBjAEcAQQBTAE0AXwBtAFQAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAG4AaQB0AHIAbwBnAGUAbgAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBNAFMAXwBBAFQATQBPAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgA1ACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBfAHsAQQBUAE0ATwBTAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAfQBcAFwAdABpAG0AZQBzACAARgByAGEAYwBHAEEAUwBNAF8AewBtAFQAfQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBOAF8AagBtAFQAXAAiACwAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAGUAYQBjAGgAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAE0ATQBTACAAKABlAHgAYwBsAHUAZABpAG4AZwAgAE0ATgBfAGkAagBtADEAMwBUADIAKQBcACIALAAgAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADEALgAxAC4AMwAgACgAMgApACgANgApACgAOAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AXwBtAFQAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABpAG4AIABlAGEAYwBoACAATQBNAFMAXAAiACwAIABcACIAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA0AC4AMQA6ACAAQgBlAGUAZgAgAEYAZQBlAGQAbABvAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADQALgAxAC4AMQAuADMAIABNAGUAdABoAG8AZAAgADEAIAAtACAATQBhAG4AdQByAGUAIABEAGkAcgBlAGMAdAAgAE4AMgBPACAAQgBlAGUAZgAgAEYAZQBlAGQAbABvAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAGQAaQByAGUAYwB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAG0AYQBuAHUAcgBlACAAbQBhAG4AYQBnAGUAbQBlAG4AdAAgAHMAeQBzAHQAZQBtAHMAXABuAEUAXwBOADIATwBkAGkAcgBcAG4AdAAgAE4AMgBPAFwAbgBFAF8AewBOADIATwAsAGQAaQByAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBqAG0AfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQApAFwAXAB0AGkAbQBlAHMAMQAwAF4AewAtADMAfQBcAG4ATQBOAF8AagBtAFQAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAcABlAHIAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAsACAATQBNAFMAIABhAG4AZAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAOgAgAGsAZwAgAE4AXABuAEUARgBfAGoAbQAgAD0AIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAE0ATQBTACAAOgAgAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AXABuAEMAXwBOADIATwAgAD0AIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzACAAOgAgAHIAYQB0AGkAbwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBfAGoAbQBUACwAIABFAEYAXwBqAG0ALAAgAEMAXwBOADIATwAsAFwAbgAgACAAIAAgAFMAVQBNAFAAUgBPAEQAVQBDAFQAKABNAE4AXwBqAG0AVAAsACAARQBGAF8AagBtACwAIABDAF8ATgAyAE8AKQAgACoAIAAxADAAIABeACAALQAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABkAGkAcgBlAGMAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABtAGEAbgB1AHIAZQAgAG0AYQBuAGEAZwBlAG0AZQBuAHQAIABzAHkAcwB0AGUAbQBzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8ATgAyAE8AZABpAHIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAATgAyAE8AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewBOADIATwAsAGQAaQByAH0APQBcAFwAcwB1AG0AXwB7AGoAfQBcAFwAcwB1AG0AXwB7AG0AfQBcAFwAcwB1AG0AXwB7AFQAfQAoAE0ATgBfAHsAagBtAFQAfQBcAFwAdABpAG0AZQBzACAARQBGAF8AewBqAG0AfQBcAFwAdABpAG0AZQBzACAAQwBfAHsATgAyAE8AfQApAFwAXAB0AGkAbQBlAHMAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0AVABcACIALABcACIAbgBpAHQAcgBvAGcAZQBuACAAcABlAHIAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAsACAATQBNAFMAIABhAG4AZAAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4AMQAuADEALgAzACAAKAAyACkAKAA2ACkAKAA4ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAGoAbQBcACIALABcACIAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABNAE0AUwBcACIALABcACIAawBnACAATgAyAE8ALQBOAC8AawBnACAATgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAXwBOADIATwBcACIALABcACIAZgBhAGMAdABvAHIAIAB0AG8AIABjAG8AbgB2AGUAcgB0ACAAZQBsAGUAbQBlAG4AdABhAGwAIABtAGEAcwBzACAAbwBmACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIALABcACIAcgBhAHQAaQBvAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABcAG4ATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxACAATQBNAFMAXABuAE0ATgBfAGoAbQA1AFQAMQBcAG4AawBnACAATgBcAG4ATQBOAF8AewBqAG0APQA1ACwAVAA9ADEAfQA9AEEARQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABNAE0AUwBfAHsAagBtAD0ANQAsAFQAPQAxAH0AXABuAEEARQBfAGoAIAA9ACAAdABvAHQAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwACAAOgAgAGsAZwAgAE4AXABuAE0ATQBTAF8AagBtADUAVAAxACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAcAByAGkAbQBhAHIAeQAgAHMAeQBzAHQAZQBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQBFAF8AagAsACAATQBNAFMAXwBqAG0ANQBUADEALABcAG4AIAAgACAAIABBAEUAXwBqACAAKgAgAE0ATQBTAF8AagBtADUAVAAxAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMQAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AagBtADUAVAAxAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEQAcgB5AGwAbwB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMgApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AXwB7AGoAbQA9ADUALABUAD0AMQB9AD0AQQBFAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBqAG0APQA1ACwAVAA9ADEAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBFAF8AagBcACIALABcACIAdABvAHQAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4AMQAuADEALgAzACAAKAAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAF8AagBtADUAVAAxAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAHAAcgBpAG0AYQByAHkAIABzAHkAcwB0AGUAbQAgAGQAcgB5AGwAbwB0ACAATQBNAFMAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFwAbgBBAG4AbgB1AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGkAbwBuACAAZgByAG8AbQAgAGUAYQBjAGgAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAXABuAEEARQBfAGoAXABuAGsAZwAgAE4AXABuAEEARQBfAHsAagB9AD0ATgBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABOAEUAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAARABfAHsAagB9AFwAbgBOAF8AagAgAD0AIABuAHUAbQBiAGUAcgAgAG8AZgAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGcAcgBvAHUAcAAgADoAIABoAGUAYQBkAFwAbgBOAEUAXwBqACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGkAbwBuACAAOgAgAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAXABuAEQAXwBqACAAPQAgAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAGYAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAgADoAIABkAGEAeQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADMAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATgBfAGoALAAgAE4ARQBfAGoALAAgAEQAXwBqACwAXABuACAAIAAgACAATgBfAGoAIAAqACAATgBFAF8AagAgACoAIABEAF8AagBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADMAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAbgBuAHUAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAaQBvAG4AIABmAHIAbwBtACAAZQBhAGMAaAAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcABcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBFAF8AagBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADMAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAzACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADMAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADMAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEUAXwB7AGoAfQA9AE4AXwB7AGoAfQBcAFwAdABpAG0AZQBzACAATgBFAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAEQAXwB7AGoAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagBcACIALABcACIAbgB1AG0AYgBlAHIAIABvAGYAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABnAHIAbwB1AHAAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARQBfAGoAXAAiACwAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGkAbwBuAFwAIgAsACAAXAAiAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4AMQAuADEALgAzACAAKAA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAXwBqAFwAIgAsAFwAIgBkAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAbwBmACAAYwBhAHQAdABsAGUAIABnAHIAbwB1AHAAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAFwAbgBOAGkAdAByAG8AZwBlAG4AIABlAHgAYwByAGUAdABpAG8AbgAgAHAAZQByACAAaABlAGEAZAAgAHAAZQByACAAZABhAHkAXABuAE4ARQBfAGoAXABuAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAXABuAE4ARQBfAHsAagB9AD0ATgBJAF8AewBqAH0AXABcAHQAaQBtAGUAcwAoADEALQBOAFIAXwB7AGoAfQApAFwAbgBOAEkAXwBqACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgB0AGEAawBlACAAOgAgAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAXABuAE4AUgBfAGoAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAcgBlAHQAZQBuAHQAaQBvAG4AIABlAHgAcAByAGUAcwBzAGUAZAAgAGEAcwAgAGEAIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABpAG4AdABhAGsAZQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE4ASQBfAGoALAAgAE4AUgBfAGoALABcAG4AIAAgACAAIABOAEkAXwBqACAAKgAgACgAMQAgAC0AIABOAFIAXwBqACkAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGkAbwBuACAAcABlAHIAIABoAGUAYQBkACAAcABlAHIAIABkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAEUAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA0ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBFAF8AewBqAH0APQBOAEkAXwB7AGoAfQBcAFwAdABpAG0AZQBzACgAMQAtAE4AUgBfAHsAagB9ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEkAXwBqAFwAIgAsAFwAIgBuAGkAdAByAG8AZwBlAG4AIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABOAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADEALgAxAC4AMwAgACgANQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAFIAXwBqAFwAIgAsAFwAIgBuAGkAdAByAG8AZwBlAG4AIAByAGUAdABlAG4AdABpAG8AbgAgAGUAeABwAHIAZQBzAHMAZQBkACAAYQBzACAAYQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AdABhAGsAZQBcAG4ATgBpAHQAcgBvAGcAZQBuACAAaQBuAHQAYQBrAGUAIABvAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAXABuAE4ASQBfAGoAXABuAGsAZwAgAE4ALwBoAGUAYQBkAC8AZABhAHkAXABuAE4ASQBfAHsAagB9AD0ASQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABDAFAAXwB7AGoAfQBcAFwAZABpAHYAIAA2AC4AMgA1AFwAbgBJAF8AagAgAD0AIABkAHIAeQAgAG0AYQB0AHQAZQByACAAaQBuAHQAYQBrAGUAIAA6ACAAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAbgBDAFAAXwBqACAAPQAgAGMAcgB1AGQAZQAgAHAAcgBvAHQAZQBpAG4AIABjAG8AbgB0AGUAbgB0ACAAbwBmACAAZgBlAGUAZAAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuADYALgAyADUAIAA9ACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGMAbwBuAHYAZQByAHQAaQBuAGcAIABjAHIAdQBkAGUAIABwAHIAbwB0AGUAaQBuACAAaQBuAHQAbwAgAG4AaQB0AHIAbwBnAGUAbgAgADoAIAByAGEAdABpAG8AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AdABhAGsAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABJAF8AagAsACAAQwBQAF8AagAsAFwAbgAgACAAIAAgAEkAXwBqACAAKgAgAEMAUABfAGoAIAAvACAANgAuADIANQBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgB0AGEAawBlACAAbwBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAEkAXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AdABhAGsAZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAA0AC4AMQAuADEALgAzACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AdABhAGsAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AdABhAGsAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4ASQBfAHsAagB9AD0ASQBfAHsAagB9AFwAXAB0AGkAbQBlAHMAIABDAFAAXwB7AGoAfQBcAFwAZABpAHYAIAA2AC4AMgA1AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAXwBqAFwAIgAsAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAaQBuAHQAYQBrAGUAXAAiACwAIABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBQAF8AagBcACIALABcACIAYwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABmAGUAZQBkAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiADYALgAyADUAXAAiACwAXAAiAGYAYQBjAHQAbwByACAAZgBvAHIAIABjAG8AbgB2AGUAcgB0AGkAbgBnACAAYwByAHUAZABlACAAcAByAG8AdABlAGkAbgAgAGkAbgB0AG8AIABuAGkAdAByAG8AZwBlAG4AXAAiACwAIABcACIAcgBhAHQAaQBvAFwAIgAsACAAXAAiAEMAbwBuAHMAdABhAG4AdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBcAG4ATgBpAHQAcgBvAGcAZQBuACAAaQBuACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyACAATQBNAFMAXABuAE0ATgBfAGoAbQBUADIAXABuAGsAZwAgAE4AXABuAE0ATgBfAHsAagBtACwAVAA9ADIAfQA9AE4AVABfAHsAagBtACwAVAA9ADIAfQBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AGoAbQAsAFQAPQAyAH0AXABuAE4AVABfAGoAbQBUADIAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAdAByAGEAbgBzAGYAZQByAHIAZQBkACAAdABvACAAcwBlAGMAbwBuAGQAYQByAHkAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAE0ATQBTACAAOgAgAGsAZwAgAE4AXABuAE0ATQBTAF8AagBtAFQAMgAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAGkAbgAgAGUAYQBjAGgAIABzAGUAYwBvAG4AZABhAHIAeQAgAHMAeQBzAHQAZQBtACAAOgAgAGYAcgBhAGMAdABpAG8AbgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABOAFQAXwBqAG0AVAAyACwAIABNAE0AUwBfAGoAbQBUADIALABcAG4AIAAgACAAIABOAFQAXwBqAG0AVAAyACAAKgAgAE0ATQBTAF8AagBtAFQAMgBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGkAdAByAG8AZwBlAG4AIABpAG4AIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADIAIABNAE0AUwBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATgBfAGoAbQBUADIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAxAC4AMwAsACAARQBxAHUAYQB0AGkAbwBuACAAKAA2ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0ATgBfAHsAagBtACwAVAA9ADIAfQA9AE4AVABfAHsAagBtACwAVAA9ADIAfQBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AGoAbQAsAFQAPQAyAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AVABfAGoAbQBUADIAXAAiACwAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAdAByAGUAYQB0AG0AZQBuAHQAIABNAE0AUwBcACIALAAgAFwAIgBrAGcAIABOAFwAIgAsACAAXAAiAEMAYQBsAGMAdQBsAGEAdABlAGQAIABmAHIAbwBtACAANAAuADEALgAxAC4AMwAgACgANwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE0AUwBfAGoAbQBUADIAXAAiACwAXAAiAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAG0AYQBuAHUAcgBlACAAaQBuACAAZQBhAGMAaAAgAHMAZQBjAG8AbgBkAGEAcgB5ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXABuAE4AaQB0AHIAbwBnAGUAbgAgAHQAcgBhAG4AcwBmAGUAcgByAGUAZAAgAHQAbwAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMgAgAE0ATQBTAFwAbgBOAFQAXwBqAG0AVAAyAFwAbgBrAGcAIABOAFwAbgBOAFQAXwB7AGoAbQAsAFQAPQAyAH0APQAoAE0ATgBfAHsAagBtAD0ANQAsAFQAPQAxAH0AXABcAHQAaQBtAGUAcwAoADEALQBGAHIAYQBjAEcAQQBTAE0AXwB7AG0APQA1AH0ALQBFAEYAXwB7AG0APQA1AH0AKQApAC0ATQBOAF8AewBqAG0ALABUAD0AMwB9AFwAbgBNAE4AXwBqAG0ANQBUADEAIAA9ACAAbgBpAHQAcgBvAGcAZQBuACAAaQBuACAATQBNAFMAIAB0AHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgADEAIAA6ACAAawBnACAATgBcAG4ARgByAGEAYwBHAEEAUwBNAF8AbQA1ACAAPQAgAGYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB2AG8AbABhAHQAaQBsAGkAcwBlAGQAIABmAHIAbwBtACAAZAByAHkAbABvAHQAIABNAE0AUwAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAEUARgBfAG0ANQAgAD0AIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAGQAcgB5AGwAbwB0ACAATQBNAFMAIAA6ACAAawBnACAATgAyAE8ALQBOAC8AawBnACAATgAgAGQAZQBwAG8AcwBpAHQAZQBkAFwAbgBNAE4AXwBqAG0AVAAzACAAPQAgAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAE0ATQBTACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAzACAAOgAgAGsAZwAgAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0ATgBfAGoAbQA1AFQAMQAsACAARgByAGEAYwBHAEEAUwBNAF8AbQA1ACwAIABFAEYAXwBtADUALAAgAE0ATgBfAGoAbQBUADMALABcAG4AIAAgACAAIAAoAE0ATgBfAGoAbQA1AFQAMQAgACoAIAAoADEAIAAtACAARgByAGEAYwBHAEEAUwBNAF8AbQA1ACAALQAgAEUARgBfAG0ANQApACkAIAAtACAATQBOAF8AagBtAFQAMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAGcAZQBuACAAdAByAGEAbgBzAGYAZQByAHIAZQBkACAAdABvACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAyACAATQBNAFMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBUAF8AagBtAFQAMgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgANwApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AVABfAHsAagBtACwAVAA9ADIAfQA9ACgATQBOAF8AewBqAG0APQA1ACwAVAA9ADEAfQBcAFwAdABpAG0AZQBzACgAMQAtAEYAcgBhAGMARwBBAFMATQBfAHsAbQA9ADUAfQAtAEUARgBfAHsAbQA9ADUAfQApACkALQBNAE4AXwB7AGoAbQAsAFQAPQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAE4AXwBqAG0ANQBUADEAXAAiACwAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAE0ATQBTACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAxAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4AMQAuADEALgAzACAAKAAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAcgBhAGMARwBBAFMATQBfAG0ANQBcACIALABcACIAZgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGYAcgBvAG0AIABkAHIAeQBsAG8AdAAgAE0ATQBTAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARgBfAG0ANQBcACIALABcACIAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIABkAHIAeQBsAG8AdAAgAE0ATQBTAFwAIgAsACAAXAAiAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AIABkAGUAcABvAHMAaQB0AGUAZABcACIALAAgAFwAIgBDAG8AbgBzAHQAYQBuAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATgBfAGoAbQBUADMAXAAiACwAXAAiAG4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAE0ATQBTACAAdAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIAAzAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4AMQAuADEALgAzACAAKAA4ACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXABuAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMwAgAE0ATQBTAFwAbgBNAE4AXwBqAG0AMQBUADMAXABuAGsAZwAgAE4AXABuAE0ATgBfAHsAagBtAD0AMQAsAFQAPQAzAH0APQBBAEUAXwB7AGoAfQBcAFwAdABpAG0AZQBzACAATQBNAFMAXwB7AGoAbQA9ADEALABUAD0AMwB9AFwAbgBBAEUAXwBqACAAPQAgAHQAbwB0AGEAbAAgAG4AaQB0AHIAbwBnAGUAbgAgAGUAeABjAHIAZQB0AGUAZAAgAGIAeQAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGcAcgBvAHUAcAAgADoAIABrAGcAIABOAFwAbgBNAE0AUwBfAGoAbQAxAFQAMwAgAD0AIABmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAHQAbwAgAHQAZQByAHQAaQBhAHIAeQAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIABzAHkAcwB0AGUAbQAgADoAIABmAHIAYQBjAHQAaQBvAG4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQBFAF8AagAsACAATQBNAFMAXwBqAG0AMQBUADMALABcAG4AIAAgACAAIABBAEUAXwBqACAAKgAgAE0ATQBTAF8AagBtADEAVAAzAFwAbgAgACAAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwBnAGUAbgAgAGkAbgAgAHQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAMwAgAE0ATQBTAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBOAF8AagBtADEAVAAzAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMQAuADMALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAOAApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE4AXwB7AGoAbQA9ADEALABUAD0AMwB9AD0AQQBFAF8AewBqAH0AXABcAHQAaQBtAGUAcwAgAE0ATQBTAF8AewBqAG0APQAxACwAVAA9ADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBFAF8AagBcACIALABcACIAdABvAHQAYQBsACAAbgBpAHQAcgBvAGcAZQBuACAAZQB4AGMAcgBlAHQAZQBkACAAYgB5ACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAZwByAG8AdQBwAFwAIgAsACAAXAAiAGsAZwAgAE4AXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAA0AC4AMQAuADEALgAzACAAKAAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0ATQBTAF8AagBtADEAVAAzAFwAIgAsAFwAIgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABtAGEAbgB1AHIAZQAgAHQAbwAgAHQAZQByAHQAaQBhAHIAeQAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAxADoAIABFAG4AdABlAHIAaQBjACAATQBlAHQAaABhAG4AZQAgAC0AIABGAGUAZQBkAGwAbwB0ACAAQgBlAGUAZgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMwAuADEALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABFAG4AdABlAHIAaQBjACAAQgBlAGUAZgAgAEYAZQBlAGQAbABvAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGkAbgAgAGYAZQBlAGQAbABvAHQAIABiAGUAZQBmACAAYwBhAHQAdABsAGUAXABuAEUAXwBlAG4AdABlAHIAaQBjAFwAbgB0ACAAQwBIADQAXABuAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoAEQAXwBqAFwAXAB0AGkAbQBlAHMAIABNAF8AagBcAFwAdABpAG0AZQBzACAATgBfAGoAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ARABfAGoAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGwAbwB0ACAAKABkAGEAeQBzACkAXABuAE0AXwBqACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBOAF8AagAgAD0AIABuAHUAbQBiAGUAcgBzACAAbwBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAbABvAHQAIAAoAGgAZQBhAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEQAXwBqACwAIABNAF8AagAsACAATgBfAGoALABcAG4AIAAgACAAIAAoAEQAXwBqACAAKgAgAE0AXwBqACAAKgAgAE4AXwBqACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZgBlAGUAZABsAG8AdAAgAGIAZQBlAGYAIABjAGEAdAB0AGwAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGUAbgB0AGUAcgBpAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewBlAG4AdABlAHIAaQBjAH0APQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAGoAKABEAF8AagBcAFwAdABpAG0AZQBzACAATQBfAGoAXABcAHQAaQBtAGUAcwAgAE4AXwBqACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGwAbwB0AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAF8AagBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAxAC4AMQAuADEALAAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgBzACAAbwBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAbABvAHQAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4ARABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlAFwAbgBNAF8AagBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwBqAD0AKAA1AC4AMQAxAFwAXAB0AGkAbQBlAHMAIABJAF8AagAtADQALgAwADAAXABcAHQAaQBtAGUAcwAgAEUARQBfAGoAKwAyAC4AMgA2AFwAXAB0AGkAbQBlAHMAIABOAEQARgBfAGoAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ASQBfAGoAIAA9ACAAZAByAHkAIABtAGEAdAB0AGUAcgAgAGkAbgB0AGEAawBlACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARQBFAF8AagAgAD0AIABlAHQAaABlAHIAIABlAHgAdAByAGEAYwB0ACAAYQBzACAAYQAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABvAGYAIABJAF8AagAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAE4ARABGAF8AagAgAD0AIABuAGUAdQB0AHIAYQBsACAAZABlAHQAZQByAGcAZQBuAHQAIABmAGkAYgByAGUAIABhAHMAIABhACAAcABlAHIAYwBlAG4AdABhAGcAZQAgAG8AZgAgAEkAXwBqACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEkAXwBqACwAIABFAEUAXwBqACwAIABOAEQARgBfAGoALABcAG4AIAAgACAAIAAoADUALgAxADEAIAAqACAASQBfAGoAIAAtACAANAAuADAAMAAgACoAIABFAEUAXwBqACAAKwAgADIALgAyADYAIAAqACAATgBEAEYAXwBqACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAGwAbQBlAGkAZABhACAAZQB0ACAAYQBsAC4AIAAoADIAMAAyADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAD0AKAA1AC4AMQAxAFwAXAB0AGkAbQBlAHMAIABJAF8AagAtADQALgAwADAAXABcAHQAaQBtAGUAcwAgAEUARQBfAGoAKwAyAC4AMgA2AFwAXAB0AGkAbQBlAHMAIABOAEQARgBfAGoAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAF8AagBcACIALAAgAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAaQBuAHQAYQBrAGUAXAAiACwAIABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBFAF8AagBcACIALAAgAFwAIgBlAHQAaABlAHIAIABlAHgAdAByAGEAYwB0ACAAYQBzACAAYQAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABvAGYAIABJAF8AagBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEQARgBfAGoAXAAiACwAIABcACIAbgBlAHUAdAByAGEAbAAgAGQAZQB0AGUAcgBnAGUAbgB0ACAAZgBpAGIAcgBlACAAYQBzACAAYQAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABvAGYAIABJAF8AagBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAEgAYQByAHYAZQBzAHQASQBuAGQAZQB4ACIALAAiAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEMAYQBsAGMAdQBsAGEAdABlAFIAZQBzAGkAZAB1AGUAQwByAG8AcABSAGEAdABpAG8AIgAsACIAQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8AQwBhAGwAYwB1AGwAYQB0AGUARgByAGEAYwB0AGkAbwBuAFIAZQBzAGkAZAB1AGUAUgBlAG0AbwB2AGUAZAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADEATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADIATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADMATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATABpAHYAZQBzAHQAbwBjAGsAQwBsAGEAcwBzAGUAcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBEAGEAdABhACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMgBfAFMAdABhAGcAZQAxAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBEAHIAeQBsAG8AdABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADIAXwBTAHQAYQBnAGUAMQBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4ARAByAHkAbABvAHQAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAyAF8AUwB0AGEAZwBlADEATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEQAcgB5AGwAbwB0AF8AQQByAGcAdQBtAGUAbgB0AHMAXwBNAGUAdABoAG8AZAAyACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwAzAF8AUwB0AGEAZwBlADIATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8AMwBfAFMAdABhAGcAZQAyAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADMAXwBTAHQAYQBnAGUAMgBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBfAE0AZQB0AGgAbwBkADIAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADQAXwBTAHQAYQBnAGUAMwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA0AF8AUwB0AGEAZwBlADMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANABfAFMAdABhAGcAZQAzAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAF8ATQBlAHQAaABvAGQAMgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAxAF8AXwA1AF8AVgBvAGwAYQB0AGkAbABlAFMAbwBsAGkAZABQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMQBfAF8ANQBfAFYAbwBsAGEAdABpAGwAZQBTAG8AbABpAGQAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADEAXwBfADUAXwBWAG8AbABhAHQAaQBsAGUAUwBvAGwAaQBkAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADEAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAxAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAxAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMQBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADEAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBNAGEAbgB1AHIAZQBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADkAXwBfADIAXwBNAGEAcwBzAE8AZgBOAGkAdAByAG8AZwBlAG4AQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATQBhAG4AdQByAGUAQQBwAHAAbABpAGUAZABUAG8AUwBvAGkAbABzAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA5AF8AXwAyAF8ATQBhAHMAcwBPAGYATgBpAHQAcgBvAGcAZQBuAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBTAGMAbwBwAGUAMwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE0AYQBuAHUAcgBlAEEAcABwAGwAaQBlAGQAVABvAFMAbwBpAGwAcwBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AOQBfAF8AMgBfAE0AYQBzAHMATwBmAE4AaQB0AHIAbwBnAGUAbgBBAHAAcABsAGkAZQBkAFQAbwBTAG8AaQBsAHMAUwBjAG8AcABlADMAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwAQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4ARQBtAGkAcwBzAGkAbwBuAHMAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAEUAbQBpAHMAcwBpAG8AbgBzAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBFAG0AaQBzAHMAaQBvAG4AcwBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAEEAdABtAG8AcwBwAGgAZQByAGkAYwBEAGUAcABvAHMAaQB0AGkAbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwA1AF8AXwAyAF8AVgBvAGwAYQB0AGkAbABpAHMAZQBkAE4AaQB0AHIAbwBnAGUAbgBGAHIAbwBtAE0AYQBuAHUAcgBlAE0AYQBuAGEAZwBlAG0AZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBBAHQAbQBvAHMAcABoAGUAcgBpAGMARABlAHAAbwBzAGkAdABpAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8ANQBfAF8AMgBfAFYAbwBsAGEAdABpAGwAaQBzAGUAZABOAGkAdAByAG8AZwBlAG4ARgByAG8AbQBNAGEAbgB1AHIAZQBNAGEAbgBhAGcAZQBtAGUAbgB0AF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8AQQB0AG0AbwBzAHAAaABlAHIAaQBjAEQAZQBwAG8AcwBpAHQAaQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADUAXwBfADIAXwBWAG8AbABhAHQAaQBsAGkAcwBlAGQATgBpAHQAcgBvAGcAZQBuAEYAcgBvAG0ATQBhAG4AdQByAGUATQBhAG4AYQBnAGUAbQBlAG4AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABEAGkAcgBlAGMAdABOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAG0AaQBzAHMAaQBvAG4AcwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwARABpAHIAZQBjAHQATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBtAGkAcwBzAGkAbwBuAHMAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAEQAaQByAGUAYwB0AE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUAbQBpAHMAcwBpAG8AbgBzAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEQAcgB5AGwAbwB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADIAXwBTAHQAYQBnAGUAMQBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEQAcgB5AGwAbwB0AF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMgBfAFMAdABhAGcAZQAxAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMARAByAHkAbABvAHQAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAyAF8AUwB0AGEAZwBlADEATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBEAHIAeQBsAG8AdABfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AMwBfAEEAbgBuAHUAYQBsAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADMAXwBBAG4AbgB1AGEAbABOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwAzAF8AQQBuAG4AdQBhAGwATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADQAXwBOAGkAdAByAG8AZwBlAG4ARQB4AGMAcgBlAHQAaQBvAG4AUABlAHIASABlAGEAZABfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA0AF8ATgBpAHQAcgBvAGcAZQBuAEUAeABjAHIAZQB0AGkAbwBuAFAAZQByAEgAZQBhAGQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANABfAE4AaQB0AHIAbwBnAGUAbgBFAHgAYwByAGUAdABpAG8AbgBQAGUAcgBIAGUAYQBkAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBUAGkAdABsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA1AF8ATgBpAHQAcgBvAGcAZQBuAEkAbgB0AGEAawBlAF8AUwBvAHUAcgBjAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANQBfAE4AaQB0AHIAbwBnAGUAbgBJAG4AdABhAGsAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADUAXwBOAGkAdAByAG8AZwBlAG4ASQBuAHQAYQBrAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANgBfAFMAdABhAGcAZQAyAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAXwBVAG4AaQB0ACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA2AF8AUwB0AGEAZwBlADIATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADYAXwBTAHQAYQBnAGUAMgBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8AVABpAHQAbABlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFUAbgBpAHQAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADcAXwBOAGkAdAByAG8AZwBlAG4AVAByAGEAbgBzAGYAZQByAHIAZQBkAFQAbwBTAHQAYQBnAGUAMgBfAFMAbwB1AHIAYwBlACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA3AF8ATgBpAHQAcgBvAGcAZQBuAFQAcgBhAG4AcwBmAGUAcgByAGUAZABUAG8AUwB0AGEAZwBlADIAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8ANwBfAE4AaQB0AHIAbwBnAGUAbgBUAHIAYQBuAHMAZgBlAHIAcgBlAGQAVABvAFMAdABhAGcAZQAyAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIATQBNAFMAXwBGAGUAZQBkAGwAbwB0AF8ATgAyAE8ARABpAHIAZQBjAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADQAXwAxAF8AMQBfADMAXwBfADgAXwBTAHQAYQBnAGUAMwBOAGkAdAByAG8AZwBlAG4ASQBuAE0ATQBTAEEAbgBhAGUAcgBvAGIAaQBjAEwAYQBnAG8AbwBuAF8AVQBuAGkAdAAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBNAE0AUwBfAEYAZQBlAGQAbABvAHQAXwBOADIATwBEAGkAcgBlAGMAdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8ANABfADEAXwAxAF8AMwBfAF8AOABfAFMAdABhAGcAZQAzAE4AaQB0AHIAbwBnAGUAbgBJAG4ATQBNAFMAQQBuAGEAZQByAG8AYgBpAGMATABhAGcAbwBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAE0ATQBTAF8ARgBlAGUAZABsAG8AdABfAE4AMgBPAEQAaQByAGUAYwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwA0AF8AMQBfADEAXwAzAF8AXwA4AF8AUwB0AGEAZwBlADMATgBpAHQAcgBvAGcAZQBuAEkAbgBNAE0AUwBBAG4AYQBlAHIAbwBiAGkAYwBMAGEAZwBvAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgACcARgByAHkAJwAgAHQAbwAgACcARAByAHkAJwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQA1ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAWgBvAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAG8AcgAgAEQAcgB5ACAAWgBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIAB3AGUAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGgAaQBnAGgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAdwBhAHIAbQAgAC8AIABjAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAvACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAIABhAG4AZAAgAGgAaQBnAGgAIAB0AGUAbQBwACAAYwBsAGEAcwBzAGUAcwAgAHQAbwAgAGEAYwBjAG8AbQBtAG8AZABhAHQAZQAgAGMAbABpAG0AYQB0AGUAIABzAGMAZQBuAGEAcgBpAG8AcwAgAGUAeABjAGwAdQBkAGUAZAAgAGIAeQAgAFYARQBFAFIARwAgAGMAcgBpAHQAZQByAGkAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGkAeABlAGQAIAB0AHkAcABvACAAaQBuACAATQBBAFQAIAB2AGEAbAB1AGUAIABmAG8AcgAgAHcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGMAaABhAG4AZwBlAGQAIAAxADAAIAB0AG8AIAAxADEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAbQBpAG4AIABhAG4AZAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAGYAbwByACAATQBBAFQALAAgAE0AQQBQACwAIABmAHIAbwBzAHQAIABkAGEAeQBzACAAcABlAHIAIAB5AGUAYQByACwAIABlAGwAZQB2AGEAdABpAG8AbgAsACAATQBBAFAAOgBQAEUAVAAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQBzACAAZgByAG8AbQAgAHIAZQBhAGwAIABjAGwAaQBtAGEAdABlACAAZABhAHQAYQAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBHAEEARgAgAGEAYwBjAGUAcAB0AHMAIAByAGEAaQBuAGYAYQBsAGwAIABhAHMAIABhACAAcAByAG8AeAB5ACAAZgBvAHIAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADEANgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAXAAiACwAIABcACIATQBBAFAAXAAiACwAIABcACIARgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgBcACIALAAgAFwAIgBFAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAAdABlAG0AcABcACIALAAgAFwAIgBNAGEAeAAgAHQAZQBtAHAAXAAiACwAIABcACIATQBpAG4AIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBhAHgAIAByAGEAaQBuAGYAYQBsAGwAXAAiACwAIABcACIATQBpAG4AIABmAHIAbwBzAHQAIABkAGEAeQBzAFwAIgAsACAAXAAiAE0AYQB4ACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGkAbgAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AYQB4ACAAZQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBpAG4AIABNAEEAUAA6AFAARQBUAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAG4AdABhAG4AZQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAPgAgADEAOAAgAEMAXAAiACwAIABcACIAPgAgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAyADAAMAAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQAuADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBpAHMAdABcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgA+ACAAMQAwADAAMAAgAG0AbQAgAC0AIABkIiAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADEAMAAwADAALgAwADAAMQAsACAAMgAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAbwBwAGkAYwBhAGwAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMQA4ACAAQwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAD4AIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAxAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5AFwAIgAsACAAXAAiAD4AIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAAxAFwAIgAsACAAMQAwAC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAgAC0AOQA5ADkAOQA5ADkALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAD4AIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgA+ACAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgA+ACAAMAAgAEMAIAAtACAAZCIgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBBAHAAcABlAG4AZABpAGMAZQBzAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdABlADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AQQBUACAAPQAgAG0AZQBhAG4AIABhAG4AbgB1AGEAbAAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFAAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABFAFQAIAA9ACAAcABvAHQAZQBuAHQAaQBhAGwAIABlAHYAYQBwAG8AdAByAGEAbgBzAHAAaQByAGEAdABpAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABNAEEAVAAgAG0AaQBuACAAYQBuAGQAIABNAEEAVAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAWgBvAG4AZQBcACIALAAgAFwAIgBNAGUAZABpAGEAbgAgAEEAbgBuAHUAYQBsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACAAKABNAEEAVAApAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFQAXAAiACwAIABcACIATQBhAHgAIABNAEEAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgAFwAIgBlIiAAMgA2ACAAQwBcACIALAAgADIANgAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIABcACIAMQA1ACAALQAgADIANQAgAEMAXAAiACwAIAAxADUALAAgADIANQAuADkAOQA5ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIABcACIAZCIgADEANAAgAEMAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADQALgA5ADkAOQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQQBkAGQAZQBkACAAZQB4AHQAcgBhACAAUgBhAGkAbgBmAGEAbABsACAAbQBpAG4AIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGMAYQBsAGMAdQBsAGEAdABlACAAegBvAG4AZQAgAGYAcgBvAG0AIAByAGUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAZABhAHQAYQAuAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQBcAG4AIAAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBhAGkAbgBmAGEAbABsACAAWgBvAG4AZQBcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgBcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABtAGEAeABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAD4AIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAPgCjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAGQAbwBlAHMAIABuAG8AdAAgAG8AYwBjAHUAcgBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAZCKjAygANdg43DXYR9wwACkAKwA12GDcNdhc3DXYVtw12FncIAA12GTcNdhO3DXYYdw12FLcNdhf3CAADiE12FzcNdhZ3DXYUdw12FbcNdhb3DXYVNwgADXYUNw12E7cNdhd3DXYTtw12FDcNdhW3DXYYdw12GbcXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdABoAGEAdAAgAGkAcwAgAGEAdgBhAGkAbABhAGIAbABlACAAZgBvAHIAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHMAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBZAGUAcwAgAC0AIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AIAAtACAAbgBvAHQAIABpAG4AIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlAFwAIgAsACAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABkAGEAdABhACAAcwBjAG8AcgBlAHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAWABYAFgAWABYAFgAWABYAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAYQB0AGEAIABzAG8AdQByAGMAZQBcACIALAAgAFwAIgBEAGEAdABhACAAcwBjAG8AcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAG4AdABlAHIAbgBhAHQAaQBvAG4AYQBsACAAcwBjAG8AcABlACAAMwAgAGQAYQB0AGEAYgBhAHMAZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AHMAdAByAGEAbABpAGEAbgAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAgAG8AcgAgAHIAZQBnAGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUAbQBpAHMAcwBpAG8AbgBzACAAaQBuAHQAZQBuAHMAaQB0AHkAIABjAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgAGEAcABwAHIAbwB2AGUAZAAgAG0AZQB0AGgAbwBkAFwAIgAsACAANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAGUAcgBpAGYAaQBlAGQAIABjAHIAZQBkAGUAbgB0AGkAYQBsACAAbQBhAHQAYwBoAGkAbgBnACAASQBTAE8AMQA0ADAANgA3AFwAIgAsACAANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAEQAaQBtAGUAbgBzAGkAbwBuAGwAZQBzAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgAFYAbwBsAHUAbQBlACAAMQA6ACAATABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgAgACgAMwAuAEQALgBiAC4AMgApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAHIAYQBjAEwARQBBAEMASABcACIALAAwAC4AMgA0AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXABuADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAbgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAGYAbwByACAAbgBpAHQAcgBvAGcAZQBuACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ADUALgA1AC4AMgAuADMAIABDAG8AbgBzAHQAYQBuAHQAIABQAGEAcgBhAG0AZQB0AGUAcgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgAgADMALgBEAC4AQgBfADEAMABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAEYAbABlAGEAYwBoAFwAIgAsADAALgAwADEAMQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAoAFwAIgBcACIAKQApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAFwAbgBUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAbgBOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAZQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAcwAgAGYAbwByACAAaQBuAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAKABrAGcAIABOADIATwAtAE4ALwBrAGcAIABOACkAIAAoAEUARgBOADIATwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABrAGcAIABOADIATwAtAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAANQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAagBcACIALABcACIARQBGAE4AMgBPAFwAIgAsACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAG8AbgBsAHkAXAAiACwAIABcACIASQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADUAOQAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAwAC4AMAAwADcALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAFAAYQBzAHQAdQByAGUAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIASABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAIAAoAGwAbwB3ACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAAyADkALAAgAFwAIgBDAHIAbwBwAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACkAXAAiACwAMAAuADAAMAA4ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdQBnAGEAcgBcACIALAAwAC4AMAAxADkAOQAsACAAXAAiAFMAdQBnAGEAcgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAHQAdABvAG4AXAAiACwAMAAuADAAMAA1ADMALAAgAFwAIgBDAG8AdAB0AG8AbgBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASABvAHIAdABpAGMAdQBsAHQAdQByAGEAbAAgAGMAcgBvAHAAcwBcACIALAAwAC4AMAAwADYANAAsACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAGMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAKQBcACIALAAwAC4AMAAwADMALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAEMAbwBuAHQAaQBuAHUAbwB1AHMAIABmAGwAbwBvAGQAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAaQBjAGUAIAAoAHMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAKQBcACIALAAwAC4AMAAwADUALAAgAFwAIgBSAGkAYwBlAFwAIgAsACAAXAAiAFMAaQBuAGcAbABlACAAYQBuAGQAIABtAHUAbAB0AGkAcABsAGUAIABkAHIAYQBpAG4AYQBnAGUALAAgAG8AcgAgAGEAbAB0AGUAcgBuAGEAdABlACAAdwBlAHQAdABpAG4AZwAgAGEAbgBkACAAZAByAHkAaQBuAGcAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAwAC4AMAAwADIANgAsACAAXAAiAEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsADAALgAwADAAMQA4ACwAIABcACIARgBvAHIAZQBzAHQAcgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUgBlAG0AbwB2AGUAZAAgAGQAdQBwAGwAaQBjAGEAdABlACAAJwBBAHEAdQBhAGMAdQBsAHQAdQByAGUAJwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAJwBwAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5ACcALAAgACcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAnACAAYQBuAGQAIAAnAGkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZAAnACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAbgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAJwAgAHIAbwB3ACAAdwBpAHQAaAAgAHMAYQBtAGUAIABFAEYAIABmAG8AcgAgAGwAbwB3ACAAYQBuAGQAIABoAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAFwAbgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABDAGgAYQBwAHQAZQByACAAMQAsACAAcwBlAGMAdABpAG8AbgAgADEALgA4AC4AMgAgAEwAZQBhAGMAaABpAG4AZwAsACAAYwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBzAFwAbgBJAFAAQwBDADoAIABOADIATwAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAE0AQQBOAEEARwBFAEQAIABTAE8ASQBMAFMALAAgAEEATgBEACAAQwBPADIAIABFAE0ASQBTAFMASQBPAE4AUwAgAEYAUgBPAE0AIABMAEkATQBFACAAQQBOAEQAIABVAFIARQBBACAAQQBQAFAATABJAEMAQQBUAEkATwBOAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwBXAEUAVAAgAGYAbwByACAAaQByAHIAaQBnAGEAdABpAG8AbgAgAHQAeQBwAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBJAFAAQwBDACAAMgAwADEAOQAgAFIAZQBmAGkAbgBlAG0AZQBuAHQAIABWAG8AbAB1AG0AZQAgADQAOgAgAEMAaABhAHAAdABlAHIAIAAxADEAOgAgAE4AMgBPACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATQBhAG4AYQBnAGUAZAAgAFMAbwBpAGwAcwAsACAAYQBuAGQAIABDAE8AMgAgAEUAbQBpAHMAcwBpAG8AbgBzACAAZgByAG8AbQAgAEwAaQBtAGUAIABhAG4AZAAgAFUAcgBlAGEAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQAgAGkAcgBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAcAByAGkAbgBrAGwAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB1AHIAZgBhAGMAZQAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AdABoAGUAcgAgAGkAcgByAGkAZwBhAHQAaQBvAG4AXAAiACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAgACAAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAVABhAGIAbABlACAAYwByAGUAYQB0AGUAZAAgAGIAYQBzAGUAZAAgAG8AbgAgAFYARQBFAFIARwAgAHQAZQB4AHQAIAAnAEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuACcAXAAiACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMgA6ACAARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYAUABSAFAAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAHUAcgBpAG4AZQAgAGEAbgBkACAAZAB1AG4AZwAgAGQAZQBwAG8AcwBpAHQAZQBkACAAbwBuACAAcABhAHMAdAB1AHIAZQAsACAAcgBhAG4AZwBlACAAbwByACAAcABhAGQAZABvAGMAawBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABOADIATwAgAC0AIABOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgAFwAIgBFAEYAUABSAFAAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAAMgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAARgBSAE8ATQAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6ACAAQwBoAGEAbgBnAGUAZAAgACcARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBzACcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIAAnAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAJwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAG8AbgB0AGgAcwAgAHQAbwAgAFMAZQBhAHMAbwBuAHMAIABNAGEAcABwAGkAbgBnAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAG4AdABoAFwAIgAsACAAXAAiAFMAZQBhAHMAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAGEAbgB1AGEAcgB5AFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAYgByAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQByAGMAaABcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBwAHIAaQBsAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGEAeQBcACIALAAgAFwAIgBBAHUAdAB1AG0AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AG4AZQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASgB1AGwAeQBcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQB1AGcAdQBzAHQAXAAiACwAIABcACIAVwBpAG4AdABlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBwAHQAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBPAGMAdABvAGIAZQByAFwAIgAsACAAXAAiAFMAcAByAGkAbgBnAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdgBlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAZQBjAGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBhAG4AdQByAGUAIABNAGEAbgBhAGcAZQBtAGUAbgB0ACAAEyAgAE0AZQB0AGgAYQBuAGUAIABjAG8AbgB2AGUAcgBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABwAGUAcgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AOAAuADEAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIAMgAsACAAMQA2ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUACAAKAC6AEMAKQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBcACIALAAgAFwAIgBMAGkAcQB1AGkAZAAgAFMAbAB1AHIAcgB5ACAAKAB3AGkAdABoAG8AdQB0ACAAbgBhAHQAdQByAGEAbAAgAGMAcgB1AHMAdAApAFwAIgAsACAAXAAiAEQAYQBpAGwAeQAgAHMAcAByAGUAYQBkACAAKABiACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIALAAgAFwAIgBTAG8AbABpAGQAIABTAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAUwB0AG8AcgBhAGcAZQAgADwAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgACcAUABvAHUAbAB0AHIAeQAgAHcAaQB0AGgAIABhAG4AZAAgAHcAaQB0AGgAbwB1AHQAIABsAGkAdAB0AGUAcgAnACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAAcwBlAHAAYQByAGEAdABlACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AIABBAGQAZABlAGQAIAAnAE0AQQBUACAAcgBhAHcAJwAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBsAGwAbwB3ACAAbABvAG8AawB1AHAAIABvAGYAIABuAHUAbQBiAGUAcgBzAC4AXAAiACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALABcAG4AIAAgACAAIABSAE8AVwAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACkAIAArACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAgAC0AIAAxAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACwAXABuACAAIABDAE8ATABVAE0ATgAoAFQAYQBiAGwAZQBIAGUAYQBkAGUAcgBDAGUAbABsACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAQQByAHIAYQB5AEQAYQB0AGEALAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACwAIABbAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAXQAsAFwAbgAgAEkARgBFAFIAUgBPAFIAKABcAG4AIAAgACAAIAAgAEkATgBEAEUAWAAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABVAE4ASQBRAFUARQAoAEEAcgByAGEAeQBEAGEAdABhACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAE8AVwAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAAsACAAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAQwBPAEwAVQBNAE4AKAApAC0AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEEAcgByAGEAeQBUAGEAYgBsAGUAQwBvAGwAdQBtAG4AUwB0AGEAcgB0AE4AdQBtAGIAZQByACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQApACwAIAAxACwAIABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAIABcACIAXAAiAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATgB1AG0AYgBlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAASQBGACgASQBTAE4AVQBNAEIARQBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgAgACAAIAAgACkALAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkALAAgADAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoADEALAAgACgATABvAG8AawB1AHAAQQByAHIAYQB5ADEAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQApACoAKABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAyACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEMAZQBsAGwALAAgAEQAZQBsAGkAbQBpAHQAZQByACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAxAF0ALAAgAFsAQwBoAGEAcgBhAGMAdABlAHIAVABvAFIAZQBtAG8AdgBlADIAXQAsAFwAbgAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAWABNAEwAKABcAG4AIAAgACAAIAAgACAAIAAgAFwAIgA8AHQAPgA8AHMAPgBcACIAIAAmAFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiADwALwBzAD4APABzAD4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAKQAgACYAXABuACAAIAAgACAAIAAgACAAIABcACIAPAAvAHMAPgA8AC8AdAA+AFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQA8AD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFQAZQBtAHAAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPAA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAPgA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBGAHIAbwBzAHQAQQByAHIAYQB5ACkAPAA9AGYAcgBvAHMAdABEAGEAeQBzACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARgByAG8AcwB0AEEAcgByAGEAeQApAD4APQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApADwAPQBlAGwAZQB2ACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBhAHgARQBsAGUAdgBhAHQAaQBvAG4AQQByAHIAYQB5ACkAPgA9AGUAbABlAHYAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGkAbgBQAEUAVABBAHIAcgBhAHkAKQA8AD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAD4APQBtAGEAcABfAHAAZQB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAFQAQQBLAEUAKABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAARgBJAEwAVABFAFIAKABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAbQBhAHMAawAsACAAXAAiAE4AbwAgAG0AYQB0AGMAaABcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABNAGkAbgBBAHIAcgBhAHkALAAgAE0AYQB4AEEAcgByAGEAeQAsACAASQB0AGUAbQBBAHIAcgBhAHkALABcAG4AIAAgACAAIABMAEUAVAAoAFwAbgAgACAAIAAgACAAIAAgACAAbQBhAHMAawAsAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGkAbgBBAHIAcgBhAHkAKQA8AD0ATABvAG8AawB1AHAAVgBhAGwAdQBlACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBhAHgAQQByAHIAYQB5ACkAPgA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAPAAgAFMAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQA+ACAARQApACwAXABuACAAIAAgACAAIAAgACAAIABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBnAGUAdABPAHYAZQByAGwAYQBwAHAAaQBuAGcAUgBlAHAAbwByAHQAaQBuAGcAUABlAHIAaQBvAGQAcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAFMAdABhAHIAdAAsAFAAcgBvAGQAdQBjAHQAaQBvAG4AQwB5AGMAbABlAEUAbgBkACwAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABTACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAAIAAgACAAIABFACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABcAG4AIAAgACAAIAAgACAAIAAgAG0ALABNAE8ATgBUAEgAKABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACkALABcAG4AIAAgACAAIAAgACAAIAAgAGQALABEAEEAWQAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsACAALwAqAGgAZQBsAHAAZQByADoAIABlAG4AZAAgAGQAYQB0AGUAIABmAG8AcgAgAGEAIAByAGUAcABvAHIAdABpAG4AZwAgAHAAZQByAGkAbwBkACAAcwB0AGEAcgB0AGkAbgBnACAAYQB0ACAAYQAgAGcAaQB2AGUAbgAgAGQAYQB0AGUAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAUABlAHIAaQBvAGQARQBuAGQALABMAEEATQBCAEQAQQAoAHMAdAAsAEUARABBAFQARQAoAHMAdAAsADEAMgApAC0AMQApACwAIAAvACoAbwBuAGwAeQAgAG4AZQBlAGQAIAB0AG8AIABsAG8AbwBrACAAYgBhAGMAawAgADMANgA1ACAAZABhAHkAcwAoAG0AYQB4ACAAbwB2AGUAcgBsAGEAcAAgAHcAaQBuAGQAbwB3ACkAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAQQAsAFMALQAzADYANQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBhACwAWQBFAEEAUgAoAEEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQBiACwAWQBFAEEAUgAoAEUAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYQAgAGUAbgBkAHMAIABiAGUAZgBvAHIAZQAgAFMALABpAHQAIABjAGEAbgAnAHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQA8AFMAKQAsACAALwAqAGkAZgAgAHQAaABlACAAYQBuAGMAaABvAHIAIABmAG8AcgAgAHkAYgAgAHMAdABhAHIAdABzACAAYQBmAHQAZQByACAARQAsAGkAdAAgAGMAYQBuACcAdAAgAG8AdgBlAHIAbABhAHAAOwAgAG0AbwB2AGUAIAB0AG8AIABwAHIAZQB2AGkAbwB1AHMAIAB5AGUAYQByACoALwBcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAPgBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAJgAgAFwAIgAgAHQAbwAgAFwAIgAgACYAIABlAG4AZABzAFQAZQB4AHQAIAAmACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAPgAwACwAIAAxACwAIAAwACkAXABuACAAIAAgACAAKQApADsAXABuAFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEMAbwBuAHYAZQByAHQAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAVABvAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALABcAG4AIAAgACAAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUALAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAEEAcgByAGEAeQAsACAAUwB0AGEAdABlAEEAYgBiAHIAZQB2AGkAYQB0AGkAbwBuAEEAcgByAGEAeQAsACAAXAAiAFwAIgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwAnAFwAIgAgACYAIABzAGgAIAAmACAAXAAiACcAIQBcACIAIAAmACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAxACwAIAAyACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMwBfADQAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABBAHIAZwB1AG0AZQBuAHQAcwBBAHIAcgBhAHkALABcAG4AIAAgACAAIABDAEgATwBPAFMARQBDAE8ATABTACgAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAIAAzACwAIAA0ACkAXABuACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAE0ATQBTACwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABcAG4AIAAgACAAIAAgACAAIAAgAE0ARQBEAEkAQQBOACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0ASQBOACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApACwAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAATQBBAFgAKABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACkAXABuACAAIAAgACAAIAAgACAAIAApACwAXABuACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATQBNAFMALAAgAE0ATQBTAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACkAXABuACAAIAAgACAAKQBcAG4AKQBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAE0ATQBTAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAbABvAHQAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABsAG8AcwB0ACAAZAB1AHIAaQBuAGcAIABzAHQAbwByAGEAZwBlACAAaQBuACAAdABoAGUAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBMAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADUAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAbwAgAGUAYQBjAGgAIAB0AGUAcgB0AGkAYQByAHkAIABzAHkAcwB0AGUAbQAgAGEAcwBzAHUAbQBlAGQAIAB0AGgAYQB0ACAAMgAgAHAAZQByACAAYwBlAG4AdAAgAGkAcwAgAHIAdQBuACAALQAgAG8AZgBmACAAZgByAG8AbQAgAHQAaABlACAAZgBlAGUAZAAgAHAAYQBkAC4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAbwAgAGUAYQBjAGgAIAB0AGUAcgB0AGkAYQByAHkAIABzAHkAcwB0AGUAbQAgAGEAcwBzAHUAbQBlAGQAIAB0AGgAYQB0ACAAMgAgAHAAZQByACAAYwBlAG4AdAAgAGkAcwAgAHIAdQBuACAALQAgAG8AZgBmACAAZgByAG8AbQAgAHQAaABlACAAZgBlAGUAZAAgAHAAYQBkAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBNAFMAbQAxAFQAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADAAMgApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXABuAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAC4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAxADYAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAFwAbgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBCADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAG0AMwAgAEMASAA0ACAALwAgAGsAZwAgAFYAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAxADkAKQA7AFwAbgBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADEATQBNAFMATwBwAHQAaQBvAG4AcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADEALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBTAHQAYQBnAGUAMgBNAE0AUwBPAHAAdABpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAATQBNAFMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFMAdABhAGcAZQAzAE0ATQBTAE8AcAB0AGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAxACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEwAaQB2AGUAcwB0AG8AYwBrAEMAbABhAHMAcwBlAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAHgAcABvAHIAdAAgAG0AaQBkACAAZgBlAGQAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQB4AHAAbwByAHQAIABsAG8AbgBnACAAZgBlAGQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADEAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgACgAZABhAHkAcwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIAAoAGQAYQB5AHMAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4AMQA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAKABkAGEAeQBzACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAZQBkAGwAbwB0ACAAdAB5AHAAZQBcACIALAAgAFwAIgBMAGUAbgBnAHQAaAAgAG8AZgAgAFMAdABhAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgAxAC0AOAAwACAAZABhAHkAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgA4ADEALQAyADAAMAAgAGQAYQB5AHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBmAGUAZABcACIALAAgAFwAIgAyADAAMQArACAAZABhAHkAcwBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4AMgA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABBAG4AaQBtAGEAbAAgAGMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAAQQBuAGkAbQBhAGwAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADIAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAAQQBuAGkAbQBhAGwAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AdgBlAGQAIABmAGUAZQBkAGwAbwB0ACAAdAB5AHAAZQBzACAAdABvACAAYQAgAHMAZQBwAGEAcgBhAHQAZQAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAGEAbQBlAGQAIAAnAGMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwAnACAAYwBvAGwAdQBtAG4AIAAtACAAbwByAGkAZwBpAG4AYQBsACAAaABhAHMAIABoAGUAYQBkAGUAcgAgACcAVQBuAGkAdAAnACAAdwBoAGkAYwBoACAAYwBvAHYAZQByAHMAIAB0AHcAbwAgAGMAbwBsAHUAbQBuAHMAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAwACwAIAA3ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAZQBkAGwAbwB0ACAAdAB5AHAAZQBcACIALAAgAFwAIgBDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAXAAiACwAIABcACIAVQBuAGkAdABcACIALAAgAFwAIgAyADAAMAA1AC0AMgAwADAAOQBcACIALAAgAFwAIgAyADAAMQAwAC0AMgAwADEANABcACIALAAgAFwAIgAyADAAMQA1AC0AMgAwADEAOQBcACIALAAgAFwAIgAyADAAMgAwAC0AMgAwADIAMwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjAFwAIgAsACAAXAAiAEQAYQB5AHMAIABvAG4AIABmAGUAZQBkAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIAA3ADAALAAgADcAMAAsACAANwAwACwAIAA3ADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjAFwAIgAsACAAXAAiAEYAZQBlAGQAIABpAG4AdABhAGsAZQBcACIALAAgAFwAIgBrAGcAIABEAE0ALwBkAGEAeQBcACIALAAgADEAMAAuADAALAAgADEAMAAuADAALAAgADEAMAAuADQALAAgADEAMAAuADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjAFwAIgAsACAAXAAiAE4AIAByAGUAdABlAG4AdABpAG8AbgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAIABvAGYAIABpAG4AdABhAGsAZQBcACIALAAgADIAMQAuADEALAAgADIAMAAuADQALAAgADIAMAAuADQALAAgADIAMAAuADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBEAGEAeQBzACAAbwBuACAAZgBlAGUAZABcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAAMQAxADUALAAgADEAMQA1ACwAIAAxADIAMAAsACAAMQA1ADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBGAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACwAIABcACIAawBnACAARABNAC8AZABhAHkAXAAiACwAIAAxADEALgAyACwAIAAxADAALgA4ACwAIAAxADAALgA4ACwAIAAxADAALgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIATgAgAHIAZQB0AGUAbgB0AGkAbwBuAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdAAgAG8AZgAgAGkAbgB0AGEAawBlAFwAIgAsACAAMQAyAC4ANQAsACAAMQAyAC4ANwAsACAAMQAyAC4ANwAsACAAMQAyAC4ANwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0AZgBlAGQAXAAiACwAIABcACIARABhAHkAcwAgAG8AbgAgAGYAZQBlAGQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgADIANQAwACwAIAAyADUAMAAsACAAMgA1ADAALAAgADIANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBmAGUAZABcACIALAAgAFwAIgBGAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACwAIABcACIAawBnACAARABNAC8AZABhAHkAXAAiACwAIAA5AC4AMAAsACAAOAAuADUALAAgADgALgAyACwAIAA4AC4AMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0AZgBlAGQAXAAiACwAIABcACIATgAgAHIAZQB0AGUAbgB0AGkAbwBuAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdAAgAG8AZgAgAGkAbgB0AGEAawBlAFwAIgAsACAANgAuADYALAAgADcALgAwACwAIAA3AC4AMAAsACAANwAuADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADEALgAzADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEQAaQBlAHQAIABwAHIAbwBwAGUAcgB0AGkAZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEQAaQBlAHQAIABwAHIAbwBwAGUAcgB0AGkAZQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgAzADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEQAaQBlAHQAIABwAHIAbwBwAGUAcgB0AGkAZQBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAAnAEMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAZgByAGEAYwB0AGkAbwBuACAAYwBvAGwAdQBtAG4AIABhAG4AZAAgAGMAbwBuAHYAZQByAHQAZQBkACAATgBEAEYAIABhAG4AZAAgAEUAdABoAGUAcgAgAGUAeAB0AHIAYQBjAHQAIAB2AGEAbAB1AGUAcwAgAHQAbwAgAGYAcgBhAGMAdABpAG8AbgBzAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AbwB2AGUAZAAgAGYAZQBlAGQAbABvAHQAIAB0AHkAcABlAHMAIAB0AG8AIABhACAAcwBlAHAAYQByAGEAdABlACAAYwBvAGwAdQBtAG4AIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADMALAAgADgALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBlAGQAbABvAHQAIAB0AHkAcABlAFwAIgAsACAAXAAiAE4AdQB0AHIAaQBlAG4AdAAgAGEAbgBhAGwAeQBzAGkAcwBcACIALAAgAFwAIgBVAG4AaQB0AFwAIgAsACAAXAAiADIAMAAwADUALQAyADAAMAA5AFwAIgAsACAAXAAiADIAMAAxADAALQAyADAAMQA0AFwAIgAsACAAXAAiADIAMAAxADUALQAyADAAMQA5AFwAIgAsACAAXAAiADIAMAAyADAALQAyADAAMgAzAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHQAZQBkACAAdABvACAAZgByAGEAYwB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAG8AbQBlAHMAdABpAGMAXAAiACwAIABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ACwAIAAwAC4AMQA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBOAEQARgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAAyADMALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAwAC4AMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBFAHQAaABlAHIAIABFAHgAdAByAGEAYwB0AFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADQALgA1ACwAIAA0AC4ANQAsACAANAAuADgALAAgADQALgA4ACwAIAAwAC4AMAA0ADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBEAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AMQAzACwAIAAwAC4AMQAyADUALAAgADAALgAxADIALAAgADAALgAxADIALAAgADAALgAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBOAEQARgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAAyADQALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAyADIALgAwACwAIAAwAC4AMgAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIARQB0AGgAZQByACAARQB4AHQAcgBhAGMAdABcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAA1AC4AMAAsACAANQAuADAALAAgADUALgAwACwAIAA1AC4AMAAsACAAMAAuADAANQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0ARgBlAGQAXAAiACwAIABcACIARAByAHkAIABtAGEAdAB0AGUAcgAgAGQAaQBnAGUAcwB0AGkAYgBpAGwAaQB0AHkAXAAiACwAIABcACIAZgByAGEAYwB0AGkAbwBuAFwAIgAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQAsACAAMAAuADgAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0ARgBlAGQAXAAiACwAIABcACIAQwByAHUAZABlACAAcAByAG8AdABlAGkAbgBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AMQAzACwAIAAwAC4AMQAyADUALAAgADAALgAxADIALAAgADAALgAxADIALAAgADAALgAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAEYAZQBkAFwAIgAsACAAXAAiAE4ARABGAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADIANAAuADAALAAgADIANAAuADAALAAgADIANAAuADAALAAgADIANAAuADAALAAgADAALgAyADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAEYAZQBkAFwAIgAsACAAXAAiAEUAdABoAGUAcgAgAEUAeAB0AHIAYQBjAHQAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAANQAuADAALAAgADUALgAwACwAIAA1AC4ANQAsACAANQAuADUALAAgADAALgAwADUANQBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADQAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAATQBDAEYAcwAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQBUACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZABsAG8AdAAgAC0AIABNAEMARgBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4ANAA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHUAcABsAGkAYwBhAHQAZQBkACAATgBTAFcAIAB2AGEAbAB1AGUAcwAgAGYAbwByACAAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAE4AVAAgAGMAbwBsAHUAbQBuACAAdABoAGEAdAAgAGQAdQBwAGwAaQBjAGEAdABlAHMAIABRAEwARAAgAHYAYQBsAHUAZQBzACAAYQBzACAAcABlAHIAIABhAGQAdgBpAGMAZQAgAGYAcgBvAG0AIABzAG8AdQByAGMAZQAgAGQAYQB0AGEAIABwAHIAbwB2AGkAZABlAHIALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAVABBAFMAIABjAG8AbAB1AG0AbgAgAHQAaABhAHQAIABkAHUAcABsAGkAYwBhAHQAZQBzACAAVgBJAEMAIAB2AGEAbAB1AGUAcwAgAGEAcwAgAHAAZQByACAAYQBkAHYAaQBjAGUAIABmAHIAbwBtACAAcwBvAHUAcgBjAGUAIABkAGEAdABhACAAcAByAG8AdgBpAGQAZQByAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgACcATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuACcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABNAE0AUwAgAG4AYQBtAGUAcwAgAHQAaABhAHQAIABtAGEAdABjAGgAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAxADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAVABcACIALAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIATgBTAFcAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAUQBMAEQAXAAiACwAIABcACIATgBUAFwAIgAsACAAXAAiAFMAQQBcACIALAAgAFwAIgBWAEkAQwBcACIALAAgAFwAIgBXAEEAXAAiACwAIABcACIAVABBAFMAXAAiACwAIABcACIATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAaQBtAGEAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAbABvAHQAIAAoAEYAZQBlAGQAcABhAGQAKQBcACIALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADMALAAgADAALgAwADMALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgADAALgAwADEALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQAgACgAUwB0AG8AYwBrAHAAaQBsAGUAKQBcACIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgADAALgAwADIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAFAAYQBzAHMAaQB2AGUAIABXAGkAbgBkAHIAbwB3ACkAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAHIAdABpAGEAcgB5AFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgARQBmAGYAbAB1AGUAbgB0ACAAcABvAG4AZAApAFwAIgAsACAAMAAuADcANQAsACAAMAAuADcANQAsACAAMAAuADcANwAsACAAMAAuADcANwAsACAAMAAuADcANQAsACAAMAAuADcANQAsACAAMAAuADcANwAsACAAMAAuADcANQAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADUAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAEUARgBzACAAKABFAEYAbQBUACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgBlAGUAZABsAG8AdAAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgA1ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgACgARQBGAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgACcATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuACcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABNAE0AUwAgAG4AYQBtAGUAcwAgAHQAaABhAHQAIABtAGEAdABjAGgAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEUARgBtAFQAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQBcACIALAAgAFwAIgBOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBpAG0AYQByAHkAXAAiACwAIABcACIARAByAHkAIABsAG8AdAAgACgARgBlAGUAZABwAGEAZAApAFwAIgAsACAAMAAuADAAMAA1ADQALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAIAAoAFMAdABvAGMAawBwAGkAbABlACkAXAAiACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABQAGEAcwBzAGkAdgBlACAAVwBpAG4AZAByAG8AdwApAFwAIgAsACAAMAAuADAAMQAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgADAALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAHIAdABpAGEAcgB5AFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgARQBmAGYAbAB1AGUAbgB0ACAAUABvAG4AZAApAFwAIgAsACAAMAAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4ANgA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAIAAoAEYAcgBhAGMARwBBAFMATQBtAFQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAbABvAHQAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTACAAKABGAHIAYQBjAEcAQQBTAE0AbQBUACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4ANgA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAIAAoAEYAcgBhAGMARwBBAFMATQBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgACcATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuACcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABNAE0AUwAgAG4AYQBtAGUAcwAgAHQAaABhAHQAIABtAGEAdABjAGgAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADQALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBlAGEAdABtAGUAbgB0ACAAcwB0AGEAZwBlACAAVABcACIALAAgAFwAIgBNAE0AUwAgAG0AXAAiACwAIABcACIARgByAGEAYwBHAEEAUwBNAG0AVAAgACgAawBnACAATgBIADMALQBOACAAKwAgAE4ATwB4AC0ATgApAC8AawBnACAATgBcACIALAAgAFwAIgBOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBpAG0AYQByAHkAXAAiACwAIABcACIARAByAHkAIABsAG8AdAAgACgARgBlAGUAZABwAGEAZAApAFwAIgAsACAAMAAuADYALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAIAAoAFMAdABvAGMAawBwAGkAbABlACkAXAAiACwAIAAwAC4AMgA1ACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAUABhAHMAcwBpAHYAZQAgAFcAaQBuAGQAcgBvAHcAKQBcACIALAAgADAALgA0ACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAMAAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAcgB0AGkAYQByAHkAXAAiACwAIABcACIAVQBuAGMAbwB2AGUAcgBlAGQAIABhAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuACAAKABFAGYAZgBsAHUAZQBuAHQAIABwAG8AbgBkACkAXAAiACwAIAAwAC4AMwA1ACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8ARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAzAC4AMQA6ACAARQBuAHQAZQByAGkAYwAgAE0AZQB0AGgAYQBuAGUAIAAtACAARgBlAGUAZABsAG8AdAAgAEIAZQBlAGYAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAxAC4AMQAuADEAIABNAGUAdABoAG8AZAAgADEAIAAtACAARQBuAHQAZQByAGkAYwAgAEIAZQBlAGYAIABGAGUAZQBkAGwAbwB0AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgAqAC8AXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AVABvAHQAYQBsACAAYQBuAG4AdQBhAGwAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAGYAcgBvAG0AIABlAG4AdABlAHIAaQBjACAAZgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIABpAG4AIABmAGUAZQBkAGwAbwB0ACAAYgBlAGUAZgAgAGMAYQB0AHQAbABlAFwAbgBFAF8AZQBuAHQAZQByAGkAYwBcAG4AdAAgAEMASAA0AFwAbgBFAF8AewBlAG4AdABlAHIAaQBjAH0APQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAGoAKABEAF8AagBcAFwAdABpAG0AZQBzACAATQBfAGoAXABcAHQAaQBtAGUAcwAgAE4AXwBqACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAEQAXwBqACAAPQAgAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAGYAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABsAG8AdAAgACgAZABhAHkAcwApAFwAbgBNAF8AagAgAD0AIABkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgAgACgAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ATgBfAGoAIAA9ACAAbgB1AG0AYgBlAHIAcwAgAG8AZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGwAbwB0ACAAKABoAGUAYQBkACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABEAF8AagAsACAATQBfAGoALAAgAE4AXwBqACwAXABuACAAIAAgACAAKABEAF8AagAgACoAIABNAF8AagAgACoAIABOAF8AagApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGkAbgAgAGYAZQBlAGQAbABvAHQAIABiAGUAZQBmACAAYwBhAHQAdABsAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAXwBlAG4AdABlAHIAaQBjAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMASAA0AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADMALgAxAC4AMQAuADEALAAgAEUAcQB1AGEAdABpAG8AbgAgACgAMQApAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAHsAZQBuAHQAZQByAGkAYwB9AD0AXABcAHMAdQBtAFwAXABuAG8AbABpAG0AaQB0AHMAXwBqACgARABfAGoAXABcAHQAaQBtAGUAcwAgAE0AXwBqAFwAXAB0AGkAbQBlAHMAIABOAF8AagApAFwAXAB0AGkAbQBlAHMAIAAxADAAXgB7AC0AMwB9AFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AQQByAGcAdQBtAGUAbgB0AHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAXwBqAFwAIgAsACAAXAAiAGQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIABvAGYAIABlAGEAYwBoACAAYwBhAHQAdABsAGUAIABsAG8AdABcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBfAGoAXAAiACwAIABcACIAZABhAGkAbAB5ACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AXAAiACwAIABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACwAIABcACIAQwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIAAzAC4AMQAuADEALgAxACwAIAAoADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBfAGoAXAAiACwAIABcACIAbgB1AG0AYgBlAHIAcwAgAG8AZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAGkAbgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGwAbwB0AFwAIgAsACAAXAAiAGgAZQBhAGQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXABuAEQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQBcAG4ATQBfAGoAXABuAGsAZwAgAEMASAA0AC8AaABlAGEAZAAvAGQAYQB5AFwAbgBNAF8AagA9ACgANQAuADEAMQBcAFwAdABpAG0AZQBzACAASQBfAGoALQA0AC4AMAAwAFwAXAB0AGkAbQBlAHMAIABFAEUAXwBqACsAMgAuADIANgBcAFwAdABpAG0AZQBzACAATgBEAEYAXwBqACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXABuAEkAXwBqACAAPQAgAGQAcgB5ACAAbQBhAHQAdABlAHIAIABpAG4AdABhAGsAZQAgACgAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5ACkAXABuAEUARQBfAGoAIAA9ACAAZQB0AGgAZQByACAAZQB4AHQAcgBhAGMAdAAgAGEAcwAgAGEAIABwAGUAcgBjAGUAbgB0AGEAZwBlACAAbwBmACAASQBfAGoAIAAoAHAAZQByACAAYwBlAG4AdAApAFwAbgBOAEQARgBfAGoAIAA9ACAAbgBlAHUAdAByAGEAbAAgAGQAZQB0AGUAcgBnAGUAbgB0ACAAZgBpAGIAcgBlACAAYQBzACAAYQAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABvAGYAIABJAF8AagAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABJAF8AagAsACAARQBFAF8AagAsACAATgBEAEYAXwBqACwAXABuACAAIAAgACAAKAA1AC4AMQAxACAAKgAgAEkAXwBqACAALQAgADQALgAwADAAIAAqACAARQBFAF8AagAgACsAIAAyAC4AMgA2ACAAKgAgAE4ARABGAF8AagApACAAKgAgADEAMAAgAF4AIAAtADMAXABuACAAIAApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBEAGEAaQBsAHkAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAbwBmACAAZQBuAHQAZQByAGkAYwAgAG0AZQB0AGgAYQBuAGUAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAFwAIgApADsAXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAyACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQQBsAG0AZQBpAGQAYQAgAGUAdAAgAGEAbAAuACAAKAAyADAAMgA1ACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAF8AagA9ACgANQAuADEAMQBcAFwAdABpAG0AZQBzACAASQBfAGoALQA0AC4AMAAwAFwAXAB0AGkAbQBlAHMAIABFAEUAXwBqACsAMgAuADIANgBcAFwAdABpAG0AZQBzACAATgBEAEYAXwBqACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBfAGoAXAAiACwAIABcACIAZAByAHkAIABtAGEAdAB0AGUAcgAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEUARQBfAGoAXAAiACwAIABcACIAZQB0AGgAZQByACAAZQB4AHQAcgBhAGMAdAAgAGEAcwAgAGEAIABwAGUAcgBjAGUAbgB0AGEAZwBlACAAbwBmACAASQBfAGoAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBEAEYAXwBqAFwAIgAsACAAXAAiAG4AZQB1AHQAcgBhAGwAIABkAGUAdABlAHIAZwBlAG4AdAAgAGYAaQBiAHIAZQAgAGEAcwAgAGEAIABwAGUAcgBjAGUAbgB0AGEAZwBlACAAbwBmACAASQBfAGoAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AIgB9AF0ALAAiAHAAcgBvAGoAZQBjAHQATgBhAG0AZQBzACIAOgBbACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFYAYQBpAHIAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBSAG8AdwBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAcgBhAHkASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBUAHcAbwBDAG8AbAB1AG0AbgBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE8AbgBlAEMAbwBsAHUAbQBuAEEAbgBkAEgAZQBhAGQAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAcABsAGkAdABTAHQAcgBpAG4AZwBJAG4AdABvAEEAcgByAGEAeQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABDAGwAaQBtAGEAdABlAFoAbwBuAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAASQB0AGUAbQBGAHIAbwBtAE0AaQBuAE0AYQB4ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAFMAdQBtAFEAdQBhAG4AdABpAHQAeQBGAHIAbwBtAEMAcgBpAHQAZQByAGkAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkARgB1AG4AYwB0AGkAbwBuAE4AYQBtAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAATgAyAE8ARQBGAEYAcgBvAG0AUAByAG8AZABJAHIAcgBpAGcAYQB0AGkAbwBuAFIAYQBpAG4AZgBhAGwAbAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAEMAcgBvAHAAcABpAG4AZwBfAEcAZQB0AEYAcgBhAGMAVwBFAFQAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AQwBvAG4AdgBlAHIAdABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBUAG8AQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBvAHUAcgBjAGUASAB5AHAAZQByAGwAaQBuAGsAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAGcAdQBtAGUAbgB0AHMAXwAzAF8ANAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8ARwBlAHQATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFMAdABhAGcAZQAxAE0ATQBTAE8AcAB0AGkAbwBuAHMAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFMAdABhAGcAZQAyAE0ATQBTAE8AcAB0AGkAbwBuAHMAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFMAdABhAGcAZQAzAE0ATQBTAE8AcAB0AGkAbwBuAHMAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEwAaQB2AGUAcwB0AG8AYwBrAEMAbABhAHMAcwBlAHMAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8ARABhAHQAYQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVQBuAGkAdAAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AUwBvAHUAcgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwAiAF0ALAAiAGwAbwBjAGEAbABlACIAOgB7ACIAbABpAHMAdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHIAbwB3AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiADsAIgAsACIAYwBvAGwAdQBtAG4AUwBlAHAAYQByAGEAdABvAHIAIgA6ACIALAAiACwAIgB0AGgAbwB1AHMAYQBuAGQAcwBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFAAbwBzAGkAdABpAG8AbgBzACIAOgBbADMAXQAsACIAZABlAGMAaQBtAGEAbABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAuACIALAAiAGQAYQB0AGUATwByAGQAZQByACIAOgAiAEQATQBZACIALAAiAGMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbAAiADoAIgAkACIALAAiAGkAcwBDAHUAcgByAGUAbgBjAHkAUwB5AG0AYgBvAGwATABlAGEAZAAiADoAdAByAHUAZQAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAGUAcABCAHkAUwBwAGEAYwBlACIAOgBmAGEAbABzAGUALAAiAHIAbwB3AEwAZQB0AHQAZQByACIAOgAiAFIAIgAsACIAYwBvAGwAdQBtAG4ATABlAHQAdABlAHIAIgA6ACIAQwAiACwAIgByAGMATABlAGYAdABCAHIAYQBjAGsAZQB0ACIAOgAiAFsAIgAsACIAcgBjAFIAaQBnAGgAdABCAHIAYQBjAGsAZQB0ACIAOgAiAF0AIgAsACIAcwB0AGEAdABlAG0AZQBuAHQAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBsAG8AYwBhAGwAZQBOAGEAbQBlACIAOgAiAGUAbgAtAHUAcwAiAH0AfQA=</AFEJSONBlob>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
add tables to test input injection
</commit_message>
<xml_diff>
--- a/Excel/3_1_Enteric_Feedlot_WIP_v01.xlsx
+++ b/Excel/3_1_Enteric_Feedlot_WIP_v01.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\htdocs\zneagcrc\GAF-VEERG-Functions\Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E11FC42-28E0-4042-B4E2-E564F6E8BB54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D1B7E754-BA81-46E4-A9B8-FE1439E35DDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="5" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
+    <workbookView xWindow="720" yWindow="195" windowWidth="37140" windowHeight="20475" activeTab="3" xr2:uid="{992023F3-CAB7-4E5B-A348-08D563A0EF40}"/>
   </bookViews>
   <sheets>
     <sheet name="Home" sheetId="71" r:id="rId1"/>
@@ -389,7 +389,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="186">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="287" uniqueCount="188">
   <si>
     <t>Home</t>
   </si>
@@ -695,12 +695,6 @@
   </si>
   <si>
     <t>Number of head in each group</t>
-  </si>
-  <si>
-    <t>Table_E_CH4</t>
-  </si>
-  <si>
-    <t>Methane emissions for each group, MMS and treatment stage</t>
   </si>
   <si>
     <t>Feedlot type</t>
@@ -1071,6 +1065,18 @@
   </si>
   <si>
     <t>EFNi &amp; EFN2Oi</t>
+  </si>
+  <si>
+    <t>M2_Table_E_CH4</t>
+  </si>
+  <si>
+    <t>Methane emissions for each group, MMS and treatment stage (Method 2)</t>
+  </si>
+  <si>
+    <t>M1_Table_E_CH4</t>
+  </si>
+  <si>
+    <t>Methane emissions for each group, MMS and treatment stage (Method 1)</t>
   </si>
 </sst>
 </file>
@@ -6898,7 +6904,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -7296,7 +7302,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="109" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D1" s="110"/>
       <c r="E1" s="110"/>
@@ -7506,7 +7512,7 @@
       </c>
       <c r="C5" s="1"/>
       <c r="D5" s="112" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="E5" s="112"/>
       <c r="F5" s="112"/>
@@ -7573,7 +7579,7 @@
       <c r="A6" s="16"/>
       <c r="C6" s="1"/>
       <c r="D6" s="113" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E6" s="114"/>
       <c r="F6" s="114"/>
@@ -12572,7 +12578,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="102" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" spans="1:12" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -12633,25 +12639,25 @@
       <c r="A6" s="16"/>
       <c r="C6" s="24"/>
       <c r="D6" s="100" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="E6" s="100" t="s">
+        <v>137</v>
+      </c>
+      <c r="F6" s="100" t="s">
+        <v>138</v>
+      </c>
+      <c r="G6" s="100" t="s">
+        <v>128</v>
+      </c>
+      <c r="H6" s="100" t="s">
         <v>139</v>
       </c>
-      <c r="F6" s="100" t="s">
-        <v>140</v>
-      </c>
-      <c r="G6" s="100" t="s">
-        <v>130</v>
-      </c>
-      <c r="H6" s="100" t="s">
+      <c r="I6" s="100" t="s">
         <v>141</v>
       </c>
-      <c r="I6" s="100" t="s">
-        <v>143</v>
-      </c>
       <c r="J6" s="100" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="K6" s="24"/>
       <c r="L6" s="24"/>
@@ -12662,7 +12668,7 @@
       </c>
       <c r="C7" s="24"/>
       <c r="D7" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="E7" s="98">
         <f>'3.1.1.1-2 Enteric Methane'!E67</f>
@@ -12685,7 +12691,7 @@
         <v>991.7664400000001</v>
       </c>
       <c r="J7" s="52" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K7" s="24"/>
       <c r="L7" s="24"/>
@@ -12697,7 +12703,7 @@
       </c>
       <c r="C8" s="24"/>
       <c r="D8" s="31" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="E8" s="25"/>
       <c r="F8" s="31"/>
@@ -12711,7 +12717,7 @@
         <v>991.7664400000001</v>
       </c>
       <c r="J8" s="93" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="K8" s="24"/>
       <c r="L8" s="24"/>
@@ -14606,7 +14612,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="63" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="N1" s="54"/>
       <c r="O1" s="54"/>
@@ -14667,13 +14673,13 @@
       </c>
       <c r="D7" s="58"/>
       <c r="E7" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="F7" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="G7" s="39" t="s">
         <v>98</v>
-      </c>
-      <c r="F7" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="G7" s="39" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="8" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14720,7 +14726,7 @@
         <v>250</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="I9" s="2"/>
       <c r="J9" s="2"/>
@@ -14745,16 +14751,16 @@
     </row>
     <row r="13" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D13" s="58" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E13" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="F13" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="G13" s="39" t="s">
         <v>98</v>
-      </c>
-      <c r="F13" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="G13" s="39" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="14" spans="1:21" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -14762,7 +14768,7 @@
         <v>4</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E14" s="50" cm="1">
         <f t="array" ref="E14">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_AnimalCharacteristics[Feedlot type] = E$13) * (Table_SourceData_Feedlot_AnimalCharacteristics[Characteristic] = $D$14), Table_SourceData_Feedlot_AnimalCharacteristics[2020-2023], "Not Found")</f>
@@ -14789,7 +14795,7 @@
         <v>Constants - Feedlot</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E15" s="50" cm="1">
         <f t="array" ref="E15">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_DietProperties[Feedlot type] = E$13) * (Table_SourceData_Feedlot_DietProperties[Nutrient analysis] = $D$15), Table_SourceData_Feedlot_DietProperties[2020-2023 Converted to fraction], "Not Found")</f>
@@ -14804,7 +14810,7 @@
         <v>5.5</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I15" s="2"/>
       <c r="J15" s="2"/>
@@ -14816,7 +14822,7 @@
         <v>Constants - Livestock</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E16" s="50" cm="1">
         <f t="array" ref="E16">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_DietProperties[Feedlot type] = E$13) * (Table_SourceData_Feedlot_DietProperties[Nutrient analysis] = $D$16), Table_SourceData_Feedlot_DietProperties[2020-2023 Converted to fraction], "Not Found")</f>
@@ -14831,7 +14837,7 @@
         <v>24</v>
       </c>
       <c r="H16" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I16" s="2"/>
       <c r="J16" s="2"/>
@@ -14851,21 +14857,21 @@
         <v>Acknowledgements</v>
       </c>
       <c r="D18" s="58" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="E18" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="F18" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="G18" s="39" t="s">
         <v>98</v>
-      </c>
-      <c r="F18" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="G18" s="39" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="19" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D19" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="E19" s="61" cm="1">
         <f t="array" ref="E19">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_AnimalCharacteristics[Feedlot type] = E$18) * (Table_SourceData_Feedlot_AnimalCharacteristics[Characteristic] = $D$19), Table_SourceData_Feedlot_AnimalCharacteristics[2020-2023], "Not Found")</f>
@@ -14886,7 +14892,7 @@
     </row>
     <row r="20" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D20" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="E20" s="61" cm="1">
         <f t="array" ref="E20">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_DietProperties[Feedlot type] = E$18) * (Table_SourceData_Feedlot_DietProperties[Nutrient analysis] = $D$20), Table_SourceData_Feedlot_DietProperties[2020-2023 Converted to fraction], "Not Found")</f>
@@ -14901,7 +14907,7 @@
         <v>5.5</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I20" s="2"/>
       <c r="J20" s="2"/>
@@ -14910,7 +14916,7 @@
     <row r="21" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="17"/>
       <c r="D21" s="1" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E21" s="61" cm="1">
         <f t="array" ref="E21">_xlfn.XLOOKUP(1, (Table_SourceData_Feedlot_DietProperties[Feedlot type] = E$18) * (Table_SourceData_Feedlot_DietProperties[Nutrient analysis] = $D$21), Table_SourceData_Feedlot_DietProperties[2020-2023 Converted to fraction], "Not Found")</f>
@@ -14925,7 +14931,7 @@
         <v>24</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="I21" s="2"/>
       <c r="J21" s="2"/>
@@ -15161,7 +15167,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="K1"/>
     </row>
@@ -15175,7 +15181,7 @@
       </c>
       <c r="C3" s="4"/>
       <c r="D3" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="E3" s="4"/>
       <c r="F3" s="4"/>
@@ -15185,7 +15191,7 @@
       <c r="J3" s="4"/>
       <c r="L3" s="4"/>
       <c r="M3" s="4" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="N3" s="4"/>
       <c r="O3" s="4"/>
@@ -15347,10 +15353,10 @@
         <v>Constants - Common</v>
       </c>
       <c r="D17" s="86" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="M17" s="86" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15359,30 +15365,30 @@
         <v>Acknowledgements</v>
       </c>
       <c r="D18" s="85" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="M18" s="85" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D19" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="E19" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="F19" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="E19" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="F19" s="39" t="s">
-        <v>100</v>
-      </c>
       <c r="M19" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="N19" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="O19" s="39" t="s">
         <v>98</v>
-      </c>
-      <c r="N19" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="O19" s="39" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15424,38 +15430,38 @@
     </row>
     <row r="22" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D22" s="86" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="M22" s="86" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="23" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D23" s="85" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="M23" s="85" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D24" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="E24" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="F24" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="E24" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="F24" s="39" t="s">
-        <v>100</v>
-      </c>
       <c r="M24" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="N24" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="O24" s="39" t="s">
         <v>98</v>
-      </c>
-      <c r="N24" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="O24" s="39" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15496,38 +15502,38 @@
     <row r="26" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="27" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D27" s="86" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="M27" s="86" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="28" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D28" s="85" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="M28" s="85" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="29" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D29" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="E29" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="F29" s="39" t="s">
         <v>98</v>
       </c>
-      <c r="E29" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="F29" s="39" t="s">
-        <v>100</v>
-      </c>
       <c r="M29" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="N29" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="O29" s="39" t="s">
         <v>98</v>
-      </c>
-      <c r="N29" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="O29" s="39" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15567,38 +15573,38 @@
     <row r="31" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="32" spans="1:16" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D32" s="86" t="s">
+        <v>167</v>
+      </c>
+      <c r="M32" s="86" t="s">
         <v>169</v>
-      </c>
-      <c r="M32" s="86" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="33" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D33" s="85" t="s">
+        <v>168</v>
+      </c>
+      <c r="M33" s="85" t="s">
         <v>170</v>
-      </c>
-      <c r="M33" s="85" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="34" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D34" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="E34" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="F34" s="49" t="s">
         <v>98</v>
       </c>
-      <c r="E34" s="49" t="s">
-        <v>99</v>
-      </c>
-      <c r="F34" s="49" t="s">
-        <v>100</v>
-      </c>
       <c r="M34" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="N34" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="O34" s="49" t="s">
         <v>98</v>
-      </c>
-      <c r="N34" s="49" t="s">
-        <v>99</v>
-      </c>
-      <c r="O34" s="49" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="35" spans="3:18" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15771,13 +15777,13 @@
     </row>
     <row r="54" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D54" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="E54" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="F54" s="39" t="s">
         <v>98</v>
-      </c>
-      <c r="E54" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="F54" s="39" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="55" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15811,13 +15817,13 @@
     </row>
     <row r="59" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D59" s="39" t="s">
+        <v>96</v>
+      </c>
+      <c r="E59" s="39" t="s">
+        <v>97</v>
+      </c>
+      <c r="F59" s="39" t="s">
         <v>98</v>
-      </c>
-      <c r="E59" s="39" t="s">
-        <v>99</v>
-      </c>
-      <c r="F59" s="39" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="60" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15841,38 +15847,38 @@
     <row r="61" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="62" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D62" s="86" t="s">
-        <v>90</v>
+        <v>186</v>
       </c>
       <c r="M62" s="86" t="s">
-        <v>90</v>
+        <v>184</v>
       </c>
     </row>
     <row r="63" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D63" s="85" t="s">
-        <v>91</v>
+        <v>187</v>
       </c>
       <c r="M63" s="85" t="s">
-        <v>91</v>
+        <v>185</v>
       </c>
     </row>
     <row r="64" spans="4:15" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D64" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="E64" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="F64" s="49" t="s">
         <v>98</v>
       </c>
-      <c r="E64" s="49" t="s">
-        <v>99</v>
-      </c>
-      <c r="F64" s="49" t="s">
-        <v>100</v>
-      </c>
       <c r="M64" s="49" t="s">
+        <v>96</v>
+      </c>
+      <c r="N64" s="49" t="s">
+        <v>97</v>
+      </c>
+      <c r="O64" s="49" t="s">
         <v>98</v>
-      </c>
-      <c r="N64" s="49" t="s">
-        <v>99</v>
-      </c>
-      <c r="O64" s="49" t="s">
-        <v>100</v>
       </c>
     </row>
     <row r="65" spans="4:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
@@ -15912,7 +15918,7 @@
     <row r="66" spans="4:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" spans="4:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D67" s="89" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E67" s="90">
         <f>SUM(D65:F65)</f>
@@ -15923,7 +15929,7 @@
         <v>t CH4</v>
       </c>
       <c r="M67" s="89" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="N67" s="90">
         <f>SUM(M65:O65)</f>
@@ -15996,7 +16002,7 @@
     <row r="71" spans="4:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="72" spans="4:17" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D72" s="45" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="E72" s="45" cm="1">
         <f t="array" ref="E72">Common_Equations.Common_ConvertCH4ToCO2e(G69,G70)</f>
@@ -16007,7 +16013,7 @@
         <v>t CO2e</v>
       </c>
       <c r="M72" s="45" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="N72" s="45" cm="1">
         <f t="array" ref="N72">Common_Equations.Common_ConvertCH4ToCO2e(P69,P70)</f>
@@ -16158,7 +16164,7 @@
         <v>#VALUE!</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="2" spans="1:21" s="9" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -16384,10 +16390,10 @@
         <v>83</v>
       </c>
       <c r="G25" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="J25" s="6" t="s">
         <v>121</v>
-      </c>
-      <c r="J25" s="6" t="s">
-        <v>123</v>
       </c>
       <c r="M25" s="1"/>
     </row>
@@ -16402,10 +16408,10 @@
         <v>63</v>
       </c>
       <c r="G27" s="37" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="J27" s="37" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="M27" s="1"/>
     </row>
@@ -16423,7 +16429,7 @@
         <v>Crop</v>
       </c>
       <c r="J28" s="37" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="M28" s="1"/>
     </row>
@@ -16441,7 +16447,7 @@
         <v>Pasture</v>
       </c>
       <c r="J29" s="37" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="M29" s="1"/>
     </row>
@@ -16455,7 +16461,7 @@
         <v>Composting (passive windrow) (m=6)</v>
       </c>
       <c r="J30" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="M30" s="1"/>
     </row>
@@ -16469,7 +16475,7 @@
         <v>Direct application (m=13)</v>
       </c>
       <c r="J31" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="M31" s="1"/>
     </row>
@@ -16483,7 +16489,7 @@
         <v>Anaerobic lagoon (m=1)</v>
       </c>
       <c r="J32" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="M32" s="1"/>
     </row>
@@ -16512,10 +16518,10 @@
     </row>
     <row r="38" spans="4:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D38" s="37" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E38" s="37" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="M38" s="1"/>
     </row>
@@ -16593,25 +16599,25 @@
     </row>
     <row r="49" spans="4:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D49" s="37" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E49" s="37" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F49" s="37" t="s">
         <v>11</v>
       </c>
       <c r="G49" s="37" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H49" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="I49" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="J49" s="37" t="s">
         <v>94</v>
-      </c>
-      <c r="I49" s="37" t="s">
-        <v>95</v>
-      </c>
-      <c r="J49" s="37" t="s">
-        <v>96</v>
       </c>
       <c r="M49" s="24"/>
     </row>
@@ -16935,25 +16941,25 @@
     </row>
     <row r="66" spans="4:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D66" s="37" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="E66" s="37" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="F66" s="37" t="s">
         <v>11</v>
       </c>
       <c r="G66" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="H66" s="37" t="s">
+        <v>93</v>
+      </c>
+      <c r="I66" s="37" t="s">
         <v>94</v>
       </c>
-      <c r="H66" s="37" t="s">
-        <v>95</v>
-      </c>
-      <c r="I66" s="37" t="s">
-        <v>96</v>
-      </c>
       <c r="J66" s="37" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="M66" s="24"/>
     </row>
@@ -17683,7 +17689,7 @@
         <v>80</v>
       </c>
       <c r="F100" s="37" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="G100" s="37" t="s">
         <v>78</v>
@@ -17829,7 +17835,7 @@
         <v>80</v>
       </c>
       <c r="F112" s="95" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="G112" s="95" t="s">
         <v>78</v>
@@ -20209,7 +20215,7 @@
     </row>
     <row r="142" spans="4:77" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D142" s="37" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E142" s="37" t="s">
         <v>75</v>
@@ -20569,16 +20575,16 @@
     </row>
     <row r="186" spans="4:68" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="D186" s="37" t="s">
+        <v>115</v>
+      </c>
+      <c r="E186" s="37" t="s">
+        <v>116</v>
+      </c>
+      <c r="F186" s="37" t="s">
         <v>117</v>
       </c>
-      <c r="E186" s="37" t="s">
+      <c r="G186" s="37" t="s">
         <v>118</v>
-      </c>
-      <c r="F186" s="37" t="s">
-        <v>119</v>
-      </c>
-      <c r="G186" s="37" t="s">
-        <v>120</v>
       </c>
       <c r="H186" s="37" t="s">
         <v>25</v>
@@ -20899,7 +20905,7 @@
         <v>8</v>
       </c>
       <c r="E206" s="37" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="207" spans="4:8" x14ac:dyDescent="0.25">
@@ -20930,10 +20936,10 @@
     </row>
     <row r="212" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D212" s="37" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E212" s="37" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
     </row>
     <row r="213" spans="4:5" x14ac:dyDescent="0.25">
@@ -21079,49 +21085,49 @@
         <v>42</v>
       </c>
       <c r="E231" s="37" t="s">
+        <v>145</v>
+      </c>
+      <c r="F231" s="36" t="s">
+        <v>146</v>
+      </c>
+      <c r="G231" s="37" t="s">
         <v>147</v>
       </c>
-      <c r="F231" s="36" t="s">
+      <c r="H231" s="37" t="s">
         <v>148</v>
       </c>
-      <c r="G231" s="37" t="s">
+      <c r="I231" s="37" t="s">
         <v>149</v>
       </c>
-      <c r="H231" s="37" t="s">
+      <c r="J231" s="37" t="s">
         <v>150</v>
       </c>
-      <c r="I231" s="37" t="s">
+      <c r="K231" s="37" t="s">
         <v>151</v>
       </c>
-      <c r="J231" s="37" t="s">
+      <c r="L231" s="37" t="s">
         <v>152</v>
       </c>
-      <c r="K231" s="37" t="s">
+      <c r="M231" s="37" t="s">
         <v>153</v>
       </c>
-      <c r="L231" s="37" t="s">
+      <c r="N231" s="37" t="s">
         <v>154</v>
       </c>
-      <c r="M231" s="37" t="s">
+      <c r="O231" s="37" t="s">
         <v>155</v>
       </c>
-      <c r="N231" s="37" t="s">
+      <c r="P231" s="37" t="s">
         <v>156</v>
       </c>
-      <c r="O231" s="37" t="s">
+      <c r="Q231" s="37" t="s">
+        <v>142</v>
+      </c>
+      <c r="R231" s="37" t="s">
         <v>157</v>
       </c>
-      <c r="P231" s="37" t="s">
+      <c r="S231" s="37" t="s">
         <v>158</v>
-      </c>
-      <c r="Q231" s="37" t="s">
-        <v>144</v>
-      </c>
-      <c r="R231" s="37" t="s">
-        <v>159</v>
-      </c>
-      <c r="S231" s="37" t="s">
-        <v>160</v>
       </c>
     </row>
     <row r="232" spans="4:19" x14ac:dyDescent="0.25">
@@ -22404,10 +22410,10 @@
     </row>
     <row r="257" spans="4:5" x14ac:dyDescent="0.25">
       <c r="D257" s="37" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="E257" s="37" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="258" spans="4:5" x14ac:dyDescent="0.25">
@@ -22944,6 +22950,19 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAE0ATQBTACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAaQB0AGwAZQBDAGUAbABsACwAIABTAG8AdQByAGMAZQBDAGUAbABsACwAXABuACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAEwARQBGAFQAKABTAG8AdQByAGMAZQBDAGUAbABsACwAIABGAEkATgBEACgAXAAiACwAXAAiACwAIABTAG8AdQByAGMAZQBDAGUAbABsACkAIAAtADEAKQAsACAAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFwAIgAsACAAXAAiAFwAIgApACAAXAB1ADAAMAAyADYAIABcACIAIABcACIAIABcAHUAMAAwADIANgAgAFQAaQB0AGwAZQBDAGUAbABsAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAE0ATQBTAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAbABvAHQAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABsAG8AcwB0ACAAZAB1AHIAaQBuAGcAIABzAHQAbwByAGEAZwBlACAAaQBuACAAdABoAGUAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBMAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADUAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAbwAgAGUAYQBjAGgAIAB0AGUAcgB0AGkAYQByAHkAIABzAHkAcwB0AGUAbQAgAGEAcwBzAHUAbQBlAGQAIAB0AGgAYQB0ACAAMgAgAHAAZQByACAAYwBlAG4AdAAgAGkAcwAgAHIAdQBuACAALQAgAG8AZgBmACAAZgByAG8AbQAgAHQAaABlACAAZgBlAGUAZAAgAHAAYQBkAC4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAbwAgAGUAYQBjAGgAIAB0AGUAcgB0AGkAYQByAHkAIABzAHkAcwB0AGUAbQAgAGEAcwBzAHUAbQBlAGQAIAB0AGgAYQB0ACAAMgAgAHAAZQByACAAYwBlAG4AdAAgAGkAcwAgAHIAdQBuACAALQAgAG8AZgBmACAAZgByAG8AbQAgAHQAaABlACAAZgBlAGUAZAAgAHAAYQBkAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBNAFMAbQAxAFQAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADAAMgApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXABuAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAC4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAxADYAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAFwAbgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBCADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAG0AMwAgAEMASAA0ACAALwAgAGsAZwAgAFYAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAxADkAKQA7AFwAbgBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADEATQBNAFMATwBwAHQAaQBvAG4AcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADEALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBTAHQAYQBnAGUAMgBNAE0AUwBPAHAAdABpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAATQBNAFMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFMAdABhAGcAZQAzAE0ATQBTAE8AcAB0AGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAxACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEwAaQB2AGUAcwB0AG8AYwBrAEMAbABhAHMAcwBlAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAHgAcABvAHIAdAAgAG0AaQBkACAAZgBlAGQAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQB4AHAAbwByAHQAIABsAG8AbgBnACAAZgBlAGQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADEAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgACgAZABhAHkAcwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIAAoAGQAYQB5AHMAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4AMQA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAKABkAGEAeQBzACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAZQBkAGwAbwB0ACAAdAB5AHAAZQBcACIALAAgAFwAIgBMAGUAbgBnAHQAaAAgAG8AZgAgAFMAdABhAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgAxAC0AOAAwACAAZABhAHkAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgA4ADEALQAyADAAMAAgAGQAYQB5AHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBmAGUAZABcACIALAAgAFwAIgAyADAAMQArACAAZABhAHkAcwBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4AMgA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABBAG4AaQBtAGEAbAAgAGMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAAQQBuAGkAbQBhAGwAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADIAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAAQQBuAGkAbQBhAGwAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AdgBlAGQAIABmAGUAZQBkAGwAbwB0ACAAdAB5AHAAZQBzACAAdABvACAAYQAgAHMAZQBwAGEAcgBhAHQAZQAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAGEAbQBlAGQAIABcAHUAMAAwADIANwBjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAC0AIABvAHIAaQBnAGkAbgBhAGwAIABoAGEAcwAgAGgAZQBhAGQAZQByACAAXAB1ADAAMAAyADcAVQBuAGkAdABcAHUAMAAwADIANwAgAHcAaABpAGMAaAAgAGMAbwB2AGUAcgBzACAAdAB3AG8AIABjAG8AbAB1AG0AbgBzACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMAAsACAANwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAXAAiACwAIABcACIAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAFwAIgAsACAAXAAiAFUAbgBpAHQAXAAiACwAIABcACIAMgAwADAANQAtADIAMAAwADkAXAAiACwAIABcACIAMgAwADEAMAAtADIAMAAxADQAXAAiACwAIABcACIAMgAwADEANQAtADIAMAAxADkAXAAiACwAIABcACIAMgAwADIAMAAtADIAMAAyADMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBEAGEAeQBzACAAbwBuACAAZgBlAGUAZABcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAANwAwACwAIAA3ADAALAAgADcAMAAsACAANwA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBGAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACwAIABcACIAawBnACAARABNAC8AZABhAHkAXAAiACwAIAAxADAALgAwACwAIAAxADAALgAwACwAIAAxADAALgA0ACwAIAAxADAALgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBOACAAcgBlAHQAZQBuAHQAaQBvAG4AXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0ACAAbwBmACAAaQBuAHQAYQBrAGUAXAAiACwAIAAyADEALgAxACwAIAAyADAALgA0ACwAIAAyADAALgA0ACwAIAAyADAALgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIARABhAHkAcwAgAG8AbgAgAGYAZQBlAGQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgADEAMQA1ACwAIAAxADEANQAsACAAMQAyADAALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGQAYQB5AFwAIgAsACAAMQAxAC4AMgAsACAAMQAwAC4AOAAsACAAMQAwAC4AOAAsACAAMQAwAC4AOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAE4AIAByAGUAdABlAG4AdABpAG8AbgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAIABvAGYAIABpAG4AdABhAGsAZQBcACIALAAgADEAMgAuADUALAAgADEAMgAuADcALAAgADEAMgAuADcALAAgADEAMgAuADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAGYAZQBkAFwAIgAsACAAXAAiAEQAYQB5AHMAIABvAG4AIABmAGUAZQBkAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIAAyADUAMAAsACAAMgA1ADAALAAgADIANQAwACwAIAAyADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0AZgBlAGQAXAAiACwAIABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGQAYQB5AFwAIgAsACAAOQAuADAALAAgADgALgA1ACwAIAA4AC4AMgAsACAAOAAuADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAGYAZQBkAFwAIgAsACAAXAAiAE4AIAByAGUAdABlAG4AdABpAG8AbgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAIABvAGYAIABpAG4AdABhAGsAZQBcACIALAAgADYALgA2ACwAIAA3AC4AMAAsACAANwAuADAALAAgADcALgAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4AMwA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAGkAZQB0ACAAcAByAG8AcABlAHIAdABpAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAGkAZQB0ACAAcAByAG8AcABlAHIAdABpAGUAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4AMwA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAGkAZQB0ACAAcAByAG8AcABlAHIAdABpAGUAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAQwBvAG4AdgBlAHIAdABlAGQAIAB0AG8AIABmAHIAYQBjAHQAaQBvAG4AIABjAG8AbAB1AG0AbgAgAGEAbgBkACAAYwBvAG4AdgBlAHIAdABlAGQAIABOAEQARgAgAGEAbgBkACAARQB0AGgAZQByACAAZQB4AHQAcgBhAGMAdAAgAHYAYQBsAHUAZQBzACAAdABvACAAZgByAGEAYwB0AGkAbwBuAHMALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAHYAZQBkACAAZgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAcwAgAHQAbwAgAGEAIABzAGUAcABhAHIAYQB0AGUAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAOAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAXAAiACwAIABcACIATgB1AHQAcgBpAGUAbgB0ACAAYQBuAGEAbAB5AHMAaQBzAFwAIgAsACAAXAAiAFUAbgBpAHQAXAAiACwAIABcACIAMgAwADAANQAtADIAMAAwADkAXAAiACwAIABcACIAMgAwADEAMAAtADIAMAAxADQAXAAiACwAIABcACIAMgAwADEANQAtADIAMAAxADkAXAAiACwAIABcACIAMgAwADIAMAAtADIAMAAyADMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAdABlAGQAIAB0AG8AIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBEAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBDAHIAdQBkAGUAIABwAHIAbwB0AGUAaQBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgADAALgAxADQALAAgADAALgAxADQALAAgADAALgAxADQALAAgADAALgAxADQALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjAFwAIgAsACAAXAAiAE4ARABGAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADIAMwAuADAALAAgADIAMgAuADAALAAgADIAMgAuADAALAAgADIAMgAuADAALAAgADAALgAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjAFwAIgAsACAAXAAiAEUAdABoAGUAcgAgAEUAeAB0AHIAYQBjAHQAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAANAAuADUALAAgADQALgA1ACwAIAA0AC4AOAAsACAANAAuADgALAAgADAALgAwADQAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBDAHIAdQBkAGUAIABwAHIAbwB0AGUAaQBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgADAALgAxADMALAAgADAALgAxADIANQAsACAAMAAuADEAMgAsACAAMAAuADEAMgAsACAAMAAuADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAE4ARABGAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADIANAAuADAALAAgADIAMgAuADAALAAgADIAMgAuADAALAAgADIAMgAuADAALAAgADAALgAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBFAHQAaABlAHIAIABFAHgAdAByAGEAYwB0AFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADUALgAwACwAIAA1AC4AMAAsACAANQAuADAALAAgADUALgAwACwAIAAwAC4AMAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBGAGUAZABcACIALAAgAFwAIgBEAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBGAGUAZABcACIALAAgAFwAIgBDAHIAdQBkAGUAIABwAHIAbwB0AGUAaQBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgADAALgAxADMALAAgADAALgAxADIANQAsACAAMAAuADEAMgAsACAAMAAuADEAMgAsACAAMAAuADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0ARgBlAGQAXAAiACwAIABcACIATgBEAEYAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAMgA0AC4AMAAsACAAMgA0AC4AMAAsACAAMgA0AC4AMAAsACAAMgA0AC4AMAAsACAAMAAuADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0ARgBlAGQAXAAiACwAIABcACIARQB0AGgAZQByACAARQB4AHQAcgBhAGMAdABcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAA1AC4AMAAsACAANQAuADAALAAgADUALgA1ACwAIAA1AC4ANQAsACAAMAAuADAANQA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4ANAA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtAFQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGUAZQBkAGwAbwB0ACAALQAgAE0AQwBGAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgA0ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAE0AQwBGAHMAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABOAFMAVwAgAHYAYQBsAHUAZQBzACAAZgBvAHIAIABBAEMAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAATgBUACAAYwBvAGwAdQBtAG4AIAB0AGgAYQB0ACAAZAB1AHAAbABpAGMAYQB0AGUAcwAgAFEATABEACAAdgBhAGwAdQBlAHMAIABhAHMAIABwAGUAcgAgAGEAZAB2AGkAYwBlACAAZgByAG8AbQAgAHMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHAAcgBvAHYAaQBkAGUAcgAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABUAEEAUwAgAGMAbwBsAHUAbQBuACAAdABoAGEAdAAgAGQAdQBwAGwAaQBjAGEAdABlAHMAIABWAEkAQwAgAHYAYQBsAHUAZQBzACAAYQBzACAAcABlAHIAIABhAGQAdgBpAGMAZQAgAGYAcgBvAG0AIABzAG8AdQByAGMAZQAgAGQAYQB0AGEAIABwAHIAbwB2AGkAZABlAHIALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAATQBNAFMAIABuAGEAbQBlAHMAIAB0AGgAYQB0ACAAbQBhAHQAYwBoACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMQAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAE4AUwBXAFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAFEATABEAFwAIgAsACAAXAAiAE4AVABcACIALAAgAFwAIgBTAEEAXAAiACwAIABcACIAVgBJAEMAXAAiACwAIABcACIAVwBBAFwAIgAsACAAXAAiAFQAQQBTAFwAIgAsACAAXAAiAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAGkAbQBhAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGwAbwB0ACAAKABGAGUAZQBkAHAAYQBkACkAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAzACwAIAAwAC4AMAAzACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAIAAoAFMAdABvAGMAawBwAGkAbABlACkAXAAiACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABQAGEAcwBzAGkAdgBlACAAVwBpAG4AZAByAG8AdwApAFwAIgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQByAHQAaQBhAHIAeQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIAAoAEUAZgBmAGwAdQBlAG4AdAAgAHAAbwBuAGQAKQBcACIALAAgADAALgA3ADUALAAgADAALgA3ADUALAAgADAALgA3ADcALAAgADAALgA3ADcALAAgADAALgA3ADUALAAgADAALgA3ADUALAAgADAALgA3ADcALAAgADAALgA3ADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADEALgA1ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgACgARQBGAG0AVAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAbABvAHQAIAAtACAATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAEUARgBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4ANQA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIAAoAEUARgBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABcAHUAMAAwADIANwBOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABNAE0AUwAgAG4AYQBtAGUAcwAgAHQAaABhAHQAIABtAGEAdABjAGgAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEUARgBtAFQAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQBcACIALAAgAFwAIgBOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBpAG0AYQByAHkAXAAiACwAIABcACIARAByAHkAIABsAG8AdAAgACgARgBlAGUAZABwAGEAZAApAFwAIgAsACAAMAAuADAAMAA1ADQALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAIAAoAFMAdABvAGMAawBwAGkAbABlACkAXAAiACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABQAGEAcwBzAGkAdgBlACAAVwBpAG4AZAByAG8AdwApAFwAIgAsACAAMAAuADAAMQAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgADAALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAHIAdABpAGEAcgB5AFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgARQBmAGYAbAB1AGUAbgB0ACAAUABvAG4AZAApAFwAIgAsACAAMAAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4ANgA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAIAAoAEYAcgBhAGMARwBBAFMATQBtAFQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAbABvAHQAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTACAAKABGAHIAYQBjAEcAQQBTAE0AbQBUACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4ANgA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAIAAoAEYAcgBhAGMARwBBAFMATQBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAE0ATQBTACAAbgBhAG0AZQBzACAAdABoAGEAdAAgAG0AYQB0AGMAaAAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIABUAFwAIgAsACAAXAAiAE0ATQBTACAAbQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQBUACAAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAIgAsACAAXAAiAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAGkAbQBhAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGwAbwB0ACAAKABGAGUAZQBkAHAAYQBkACkAXAAiACwAIAAwAC4ANgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQAgACgAUwB0AG8AYwBrAHAAaQBsAGUAKQBcACIALAAgADAALgAyADUALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABQAGEAcwBzAGkAdgBlACAAVwBpAG4AZAByAG8AdwApAFwAIgAsACAAMAAuADQALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQByAHQAaQBhAHIAeQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIAAoAEUAZgBmAGwAdQBlAG4AdAAgAHAAbwBuAGQAKQBcACIALAAgADAALgAzADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAxADoAIABFAG4AdABlAHIAaQBjACAATQBlAHQAaABhAG4AZQAgAC0AIABGAGUAZQBkAGwAbwB0ACAAQgBlAGUAZgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMwAuADEALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABFAG4AdABlAHIAaQBjACAAQgBlAGUAZgAgAEYAZQBlAGQAbABvAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGkAbgAgAGYAZQBlAGQAbABvAHQAIABiAGUAZQBmACAAYwBhAHQAdABsAGUAXABuAEUAXwBlAG4AdABlAHIAaQBjAFwAbgB0ACAAQwBIADQAXABuAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoAEQAXwBqAFwAXAB0AGkAbQBlAHMAIABNAF8AagBcAFwAdABpAG0AZQBzACAATgBfAGoAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ARABfAGoAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGwAbwB0ACAAKABkAGEAeQBzACkAXABuAE0AXwBqACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBOAF8AagAgAD0AIABuAHUAbQBiAGUAcgBzACAAbwBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAbABvAHQAIAAoAGgAZQBhAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEQAXwBqACwAIABNAF8AagAsACAATgBfAGoALABcAG4AIAAgACAAIAAoAEQAXwBqACAAKgAgAE0AXwBqACAAKgAgAE4AXwBqACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZgBlAGUAZABsAG8AdAAgAGIAZQBlAGYAIABjAGEAdAB0AGwAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGUAbgB0AGUAcgBpAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewBlAG4AdABlAHIAaQBjAH0APQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAGoAKABEAF8AagBcAFwAdABpAG0AZQBzACAATQBfAGoAXABcAHQAaQBtAGUAcwAgAE4AXwBqACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGwAbwB0AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAF8AagBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAxAC4AMQAuADEALAAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgBzACAAbwBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAbABvAHQAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4ARABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlAFwAbgBNAF8AagBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwBqAD0AKAA1AC4AMQAxAFwAXAB0AGkAbQBlAHMAIABJAF8AagAtADQALgAwADAAXABcAHQAaQBtAGUAcwAgAEUARQBfAGoAKwAyAC4AMgA2AFwAXAB0AGkAbQBlAHMAIABOAEQARgBfAGoAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ASQBfAGoAIAA9ACAAZAByAHkAIABtAGEAdAB0AGUAcgAgAGkAbgB0AGEAawBlACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARQBFAF8AagAgAD0AIABlAHQAaABlAHIAIABlAHgAdAByAGEAYwB0ACAAYQBzACAAYQAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABvAGYAIABJAF8AagAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAE4ARABGAF8AagAgAD0AIABuAGUAdQB0AHIAYQBsACAAZABlAHQAZQByAGcAZQBuAHQAIABmAGkAYgByAGUAIABhAHMAIABhACAAcABlAHIAYwBlAG4AdABhAGcAZQAgAG8AZgAgAEkAXwBqACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEkAXwBqACwAIABFAEUAXwBqACwAIABOAEQARgBfAGoALABcAG4AIAAgACAAIAAoADUALgAxADEAIAAqACAASQBfAGoAIAAtACAANAAuADAAMAAgACoAIABFAEUAXwBqACAAKwAgADIALgAyADYAIAAqACAATgBEAEYAXwBqACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAGwAbQBlAGkAZABhACAAZQB0ACAAYQBsAC4AIAAoADIAMAAyADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAD0AKAA1AC4AMQAxAFwAXAB0AGkAbQBlAHMAIABJAF8AagAtADQALgAwADAAXABcAHQAaQBtAGUAcwAgAEUARQBfAGoAKwAyAC4AMgA2AFwAXAB0AGkAbQBlAHMAIABOAEQARgBfAGoAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAF8AagBcACIALAAgAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAaQBuAHQAYQBrAGUAXAAiACwAIABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBFAF8AagBcACIALAAgAFwAIgBlAHQAaABlAHIAIABlAHgAdAByAGEAYwB0ACAAYQBzACAAYQAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABvAGYAIABJAF8AagBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEQARgBfAGoAXAAiACwAIABcACIAbgBlAHUAdAByAGEAbAAgAGQAZQB0AGUAcgBnAGUAbgB0ACAAZgBpAGIAcgBlACAAYQBzACAAYQAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABvAGYAIABJAF8AagBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADEATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADIATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADMATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATABpAHYAZQBzAHQAbwBjAGsAQwBsAGEAcwBzAGUAcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100ACB660BB23738846A00119B5826AC974" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3e3613359d4ae7f6bda6c57be713f101">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7291119c-fce9-4911-96ae-b800be5dccd8" xmlns:ns3="09eef6d6-daa8-4301-8f9f-b1ec38079286" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="87491bfad7f11426ad96486e70428b3e" ns2:_="" ns3:_="">
     <xsd:import namespace="7291119c-fce9-4911-96ae-b800be5dccd8"/>
@@ -23138,19 +23157,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item4.xml><?xml version="1.0" encoding="utf-8"?>
-<AFEJSONBlob xmlns="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0">ewAiAHMAYwBoAGUAbQBhACIAOgAiAGgAdAB0AHAAOgAvAC8AcwBjAGgAZQBtAGEAcwAuAGEAZAB2AGEAbgBjAGUAZABmAG8AcgBtAHUAbABhAGUAbgB2AGkAcgBvAG4AbQBlAG4AdAAuAG8AZgBmAGkAYwBlAGEAcABwAHMALgBsAGkAdgBlAC4AYwBvAG0ALwBhAGYAZQBwAHIAbwBqAGUAYwB0AHMALwAwAC4AMgAiACwAIgBmAGkAbABlAHMAIgA6AFsAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBXAG8AcgBrAGIAbwBvAGsAIgAsACIAdABlAHgAdAAiADoAIgAvAC8AIAAtAC0ALQAgAFcAbwByAGsAYgBvAG8AawAgAG0AbwBkAHUAbABlACAALQAtAC0AXABuAC8ALwAgAEEAIABmAGkAbABlACAAbwBmACAAbgBhAG0AZQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAG8AZgAgAHQAaABlACAAZgBvAHIAbQA6AFwAbgAvAC8AIAAgACAAIABuAGEAbQBlACAAPQAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AOwBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHQAaABhAHQAIABpAHMAIABjAG8AbQBtAG8AbgAgAGEAYwByAG8AcwBzACAAYQBsAGwAIABlAG4AdABlAHIAcAByAGkAcwBlACAAdAB5AHAAZQBzAFwAbgBFAHgAYwBlAGwAIABtAG8AZAB1AGwAZQAgAG4AYQBtAGUAOgAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AUwBvAHUAcgBjAGUAOgAgAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIAAyADAAMgAzACAAVgBvAGwAdQBtAGUAIAAxAFwAbgBOAEkAUgBfADIAMAAyADMAXwBWAG8AbAAxAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AKgAvAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBcAG4AcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQAgACgAMAAuADYANwA4ADQAIABrAGcALwBtADMAKQBcAG4AVABhAGsAZQBuACAAZgByAG8AbQAgAHQAaABlACAATgBhAHQAaQBvAG4AYQBsACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAGEAbgBkACAARQBuAGUAcgBnAHkAIABSAGUAcABvAHIAdABpAG4AZwAgAFwAbgAoAE0AZQBhAHMAdQByAGUAbQBlAG4AdAApACAARABlAHQAZQByAG0AaQBuAGEAdABpAG8AbgAgADIAMAAwADgAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAcAAgAD0AIABkAGUAbgBzAGkAdAB5ACAAbwBmACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAvAG0AMwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABlAG4AcwBpAHQAeQBPAGYATQBlAHQAaABhAG4AZQBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAARQBxAHUAYQB0AGkAbwBuAHMAIAAzAC4AQgAuADEAYQBfADIALAAgADMALgBCAC4AMQBjAF8AMgAsACAAMwAuAEIALgAzAF8AMQAsACAAMwAuAEIALgA0AGcAXwAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAwAC4ANgA3ADgANAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXABuAEMAZwAgAD0AIAA0ADQALwAyADgAIABmAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABOADIATwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAE4AMgBPACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAZgBhAGMAdABvAHIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAA0ADQALwAyADgAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXABuAEYAYQBjAHQAbwByACAAdABvACAAYwBvAG4AdgBlAHIAdAAgAGUAbABlAG0AZQBuAHQAYQBsACAAbQBhAHMAcwAgAG8AZgAgAGcAYQBzACAAdABvACAAbQBvAGwAZQBjAHUAbABhAHIAIABtAGEAcwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQARwBhAHMARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGEAYwB0AG8AcgAgAHQAbwAgAGMAbwBuAHYAZQByAHQAIABlAGwAZQBtAGUAbgB0AGEAbAAgAG0AYQBzAHMAIABvAGYAIABnAGEAcwAgAHQAbwAgAG0AbwBsAGUAYwB1AGwAYQByACAAbQBhAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEMAZwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByAFwAIgAsACAAXAAiAEMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgADEAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAMgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPADIAXAAiACwAIABcACIANAA0AC8AMQAyAFwAIgAsACAANAA0ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBIADQAXAAiACwAIABcACIAMQA2AC8AMQAyAFwAIgAsACAAMQA2ACwAIAAxADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgAyAE8AXAAiACwAIABcACIANAA0AC8AMgA4AFwAIgAsACAANAA0ACwAIAAyADgAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHgAXAAiACwAIABcACIANAA2AC8AMQA0AFwAIgAsACAANAA2ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBPAFwAIgAsACAAXAAiADIAOAAvADEAMgBcACIALAAgADIAOAAsACAAMQAyADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyACAATABpAG0AZQBcACIALAAgAFwAIgA0ADQALwAxADIAXAAiACwAIAA0ADQALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAE0AVgBPAEMAXAAiACwAIABcACIAMQA0AC8AMQAyAFwAIgAsACAAMQA0ACwAIAAxADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAE4AMgBPAFwAbgBHAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAZwByAGUAZQBuAGgAbwB1AHMAZQAgAGcAYQBzAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBHAFcAUABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARwBsAG8AYgBhAGwAIAB3AGEAcgBtAGkAbgBnACAAcABvAHQAZQBuAHQAaQBhAGwAIABmAG8AcgAgAGcAcgBlAGUAbgBoAG8AdQBzAGUAIABnAGEAcwBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBHAFcAUABOADIATwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBmAGEAYwB0AG8AcgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAOAAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBhAHMAXAAiACwAIABcACIAQwBPADIALQBlACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMATwAyAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAEgANABcACIALAAgADIAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOADIATwBcACIALAAgADIANgA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMARgA0AFwAIgAsACAANgA2ADMAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDADIARgA2AFwAIgAsACAAMQAyADIAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMARgA2AFwAIgAsACAAMgAyADgAMAAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4ARgAzAFwAIgAsACAAMQA3ADIAMAAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQQB1AHMAdAByAGEAbABpAGEAbgBTAHQAYQB0AGUAcwBUAGUAcgByAGkAdABvAHIAaQBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAHQAYQB0AGUAcwAgAGEAbgBkACAAdABlAHIAcgBpAHQAbwByAGkAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADMALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAdABhAHQAZQAvAFQAZQByAHIAaQB0AG8AcgB5AFwAIgAsACAAXAAiAEMAbwBtAG0AbwBuACAATgBhAG0AZQBcACIALAAgAFwAIgBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBlAHcAIABTAG8AdQB0AGgAIABXAGEAbABlAHMAXAAiACwAIABcACIATgBTAFcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABDAGEAcABpAHQAYQBsACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIAQQBDAFQAXAAiACwAIABcACIAQQBDAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAaQBjAHQAbwByAGkAYQBcACIALAAgAFwAIgBWAGkAYwB0AG8AcgBpAGEAXAAiACwAIABcACIAVgBJAEMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFEAdQBlAGUAbgBzAGwAYQBuAGQAXAAiACwAIABcACIAUQB1AGUAZQBuAHMAbABhAG4AZABcACIALAAgAFwAIgBRAEwARABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBvAHUAdABoACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAXAAiACwAIABcACIAVwBlAHMAdABlAHIAbgAgAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgAsACAAXAAiAFcAQQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABhAHMAbQBhAG4AaQBhAFwAIgAsACAAXAAiAFQAYQBzAG0AYQBuAGkAYQBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBvAHIAdABoAGUAcgBuACAAVABlAHIAcgBpAHQAbwByAHkAXAAiACwAIABcACIATgBUAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAEIAUwAgAFMAdABhAHQAaQBzAHQAYwBhAGwAIABBAHIAZQBhAHMAIABMAGUAdgBlAGwAIAA0ACAALQAgAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAQgB1AHIAZQBhAHUAIABvAGYAIABTAHQAYQB0AGkAcwB0AGkAYwBzACAAKABBAEIAUwApACAALQAgAFMAdABhAHQAaQBzAHQAaQBjAGEAbAAgAEEAcgBlAGEAcwAgAEwAZQB2AGUAbAAgADIAIAAtACAAMgAwADIAMQAgAC0AIABTAGgAYQBwAGUAZgBpAGwAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMQAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBBACAANAAgAE4AYQBtAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEIAdQBuAGIAdQByAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQBuAGQAdQByAGEAaABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAEkAbgBuAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAE4AbwByAHQAaAAgAEUAYQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAZQByAHQAaAAgAC0AIABOAG8AcgB0AGgAIABXAGUAcwB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAGUAcgB0AGgAIAAtACAAUwBvAHUAdABoACAARQBhAHMAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUABlAHIAdABoACAALQAgAFMAbwB1AHQAaAAgAFcAZQBzAHQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABXAGgAZQBhAHQAIABCAGUAbAB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAcwB0AGUAcgBuACAAQQB1AHMAdAByAGEAbABpAGEAIAAtACAATwB1AHQAYgBhAGMAawAgACgATgBvAHIAdABoACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAZQBzAHQAZQByAG4AIABBAHUAcwB0AHIAYQBsAGkAYQAgAC0AIABPAHUAdABiAGEAYwBrACAAKABTAG8AdQB0AGgAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADIAOgAgAFQAcgBhAG4AcwBsAGEAdABpAG4AZwAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAIAB0AG8AIAB3AGUAdAAgAGEAbgBkACAAZAByAHkAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ARgAgAFMATwBVAFIAQwBFACAARABBAFQAQQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIAB3AGEAcgBtACAALwAgAGMAbwBvAGwAIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC8AIABkAHIAeQAgAC0AIABsAG8AdwAgAGYAcgBvAHMAdAAgAGEAbgBkACAAaABpAGcAaAAgAHQAZQBtAHAAIABjAGwAYQBzAHMAZQBzACAAdABvACAAYQBjAGMAbwBtAG0AbwBkAGEAdABlACAAYwBsAGkAbQBhAHQAZQAgAHMAYwBlAG4AYQByAGkAbwBzACAAZQB4AGMAbAB1AGQAZQBkACAAYgB5ACAAVgBFAEUAUgBHACAAYwByAGkAdABlAHIAaQBhAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAaQB4AGUAZAAgAHQAeQBwAG8AIAAtACAAQwBoAGEAbgBnAGUAZAAgAFwAdQAwADAAMgA3AEYAcgB5AFwAdQAwADAAMgA3ACAAdABvACAAXAB1ADAAMAAyADcARAByAHkAXAB1ADAAMAAyADcALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEANQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAFoAbwBuAGUAXAAiACwAIABcACIAVwBlAHQAIABvAHIAIABEAHIAeQAgAFoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAGQAcgB5AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAFcAZQB0ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0AFwAIgAsACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AIAB0AGUAbQBwAGUAcgBhAHQAZQAgAG0AbwBpAHMAdAAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABoAGkAZwBoACAAdABlAG0AcABcACIALAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAIAAtACAAbABvAHcAIABmAHIAbwBzAHQAXAAiACwAIABcACIARAByAHkAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAHcAYQByAG0AIAAvACAAYwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAbQBvAGkAcwB0ACAALwAgAGQAcgB5ACAALQAgAGwAbwB3ACAAZgByAG8AcwB0ACAAYQBuAGQAIABoAGkAZwBoACAAdABlAG0AcAAgAGMAbABhAHMAcwBlAHMAIAB0AG8AIABhAGMAYwBvAG0AbQBvAGQAYQB0AGUAIABjAGwAaQBtAGEAdABlACAAcwBjAGUAbgBhAHIAaQBvAHMAIABlAHgAYwBsAHUAZABlAGQAIABiAHkAIABWAEUARQBSAEcAIABjAHIAaQB0AGUAcgBpAGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBpAHgAZQBkACAAdAB5AHAAbwAgAGkAbgAgAE0AQQBUACAAdgBhAGwAdQBlACAAZgBvAHIAIAB3AGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQAgAC0AIABjAGgAYQBuAGcAZQBkACAAMQAwACAAdABvACAAMQAxAC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAG0AaQBuACAAYQBuAGQAIABtAGEAeAAgAGMAbwBsAHUAbQBuAHMAIABmAG8AcgAgAE0AQQBUACwAIABNAEEAUAAsACAAZgByAG8AcwB0ACAAZABhAHkAcwAgAHAAZQByACAAeQBlAGEAcgAsACAAZQBsAGUAdgBhAHQAaQBvAG4ALAAgAE0AQQBQADoAUABFAFQAIAB0AG8AIABjAGEAbABjAHUAbABhAHQAZQAgAHoAbwBuAGUAcwAgAGYAcgBvAG0AIAByAGUAYQBsACAAYwBsAGkAbQBhAHQAZQAgAGQAYQB0AGEALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBBAEYAIABhAGMAYwBlAHAAdABzACAAcgBhAGkAbgBmAGEAbABsACAAYQBzACAAYQAgAHAAcgBvAHgAeQAgAGYAbwByACAAcAByAGUAYwBpAHAAaQB0AGEAdABpAG8AbgAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA5ACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AQQBUAFwAIgAsACAAXAAiAE0AQQBQAFwAIgAsACAAXAAiAEYAcgBvAHMAdAAgAGQAYQB5AHMAIABwAGUAcgAgAHkAZQBhAHIAXAAiACwAIABcACIARQBsAGUAdgBhAHQAaQBvAG4AXAAiACwAIABcACIATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAHQAZQBtAHAAXAAiACwAIABcACIATQBhAHgAIAB0AGUAbQBwAFwAIgAsACAAXAAiAE0AaQBuACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AYQB4ACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAE0AaQBuACAAZgByAG8AcwB0ACAAZABhAHkAcwBcACIALAAgAFwAIgBNAGEAeAAgAGYAcgBvAHMAdAAgAGQAYQB5AHMAXAAiACwAIABcACIATQBpAG4AIABlAGwAZQB2AGEAdABpAG8AbgBcACIALAAgAFwAIgBNAGEAeAAgAGUAbABlAHYAYQB0AGkAbwBuAFwAIgAsACAAXAAiAE0AaQBuACAATQBBAFAAOgBQAEUAVABcACIALAAgAFwAIgBNAGkAbgAgAE0AQQBQADoAUABFAFQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAcgBvAHAAaQBjAGEAbAAgAG0AbwBuAHQAYQBuAGUAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA3ACwAIAAxADAAMAAwACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAdwBlAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMgAwADAAMAAgAG0AbQBcACIALAAgAFwAIgBkIiAANwBcACIALAAgAFwAIgBkIiAAMQAwADAAMAAgAG0AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIAAxADgALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgADIAMAAwADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAbQBvAGkAcwB0AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQA4ACAAQwBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAwADAAIABtAG0AIAAtACAAZCIgADIAMAAwADAAIABtAG0AXAAiACwAIABcACIAZCIgADcAXAAiACwAIABcACIAZCIgADEAMAAwADAAIABtAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAMQA4AC4AMAAwADEALAAgADkAOQA5ADkAOQA5ACwAIAAxADAAMAAwAC4AMAAwADEALAAgADIAMAAwADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADcALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5AC4AOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAG8AcABpAGMAYQBsACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADgAIABDAFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBtAFwAIgAsACAAXAAiAGQiIAA3AFwAIgAsACAAXAAiAGQiIAAxADAAMAAwACAAbQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgADEAOAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAMQAwADAAMAAsACAALQA5ADkAOQA5ADkAOQAsACAANwAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkALgA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAxADAAIABDAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAFwAdQAwADAAMwBlACAAMQBcACIALAAgADEAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAMQAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtACAAdABlAG0AcABlAHIAYQB0AGUAIABkAHIAeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAMAAgAEMAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAZCIgADEAXAAiACwAIAAxADAALgAwADAAMQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgACAALQA5ADkAOQA5ADkAOQAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsACAAdABlAG0AcABlAHIAYQB0AGUAIABtAG8AaQBzAHQAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBcAHUAMAAwADMAZQAgADEAXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAAxADAALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgADEALgAwADAAMQAsACAAOQA5ADkAOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbAAgAHQAZQBtAHAAZQByAGEAdABlACAAZAByAHkAXAAiACwAIABcACIAXAB1ADAAMAAzAGUAIAAwACAAQwAgAC0AIABkIiAAMQAwACAAQwBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBkIiAAMQBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEAMAAsACAALQA5ADkAOQA5ADkAOQAsACAAOQA5ADkAOQA5ADkALAAgAC0AOQA5ADkAOQA5ADkALAAgADkAOQA5ADkAOQA5ACwAIAAtADkAOQA5ADkAOQA5ACwAIAA5ADkAOQA5ADkAOQAsACAAIAAtADkAOQA5ADkAOQA5ACwAIAAxAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAEEAcABwAGUAbgBkAGkAYwBlAHMAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB0AGUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBBAFQAIAA9ACAAbQBlAGEAbgAgAGEAbgBuAHUAYQBsACAAdABlAG0AcABlAHIAYQB0AHUAcgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAEEAUAAgAD0AIABtAGUAYQBuACAAYQBuAG4AdQBhAGwAIABwAHIAZQBjAGkAcABpAHQAYQB0AGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAEUAVAAgAD0AIABwAG8AdABlAG4AdABpAGEAbAAgAGUAdgBhAHAAbwB0AHIAYQBuAHMAcABpAHIAYQB0AGkAbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAHQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIAAxAC4AMwA6ACAAQwBsAGkAbQBhAHQAZQAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQAgAGMAbABhAHMAcwBpAGYAaQBjAGEAdABpAG8AbgBzACAAYQBuAGQAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAEYAIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEEAZABkAGUAZAAgAGUAeAB0AHIAYQAgAE0AQQBUACAAbQBpAG4AIABhAG4AZAAgAE0AQQBUACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAB0AGUAbQBwAGUAcgBhAHQAdQByAGUAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAIABaAG8AbgBlAFwAIgAsACAAXAAiAE0AZQBkAGkAYQBuACAAQQBuAG4AdQBhAGwAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUAIAAoAE0AQQBUACkAXAAiACwAIABcACIATQBpAG4AIABNAEEAVABcACIALAAgAFwAIgBNAGEAeAAgAE0AQQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGEAcgBtAFwAIgAsACAAXAAiAGUiIAAyADYAIABDAFwAIgAsACAAMgA2ACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgAFwAIgAxADUAIAAtACAAMgA1ACAAQwBcACIALAAgADEANQAsACAAMgA1AC4AOQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgAFwAIgBkIiAAMQA0ACAAQwBcACIALAAgAC0AOQA5ADkAOQA5ADkALAAgADEANAAuADkAOQA5AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAMQAuADMAOgAgAEMAbABpAG0AYQB0AGUAIABhAG4AZAAgAFIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAIABjAGwAYQBzAHMAaQBmAGkAYwBhAHQAaQBvAG4AcwAgAGEAbgBkACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABBAGQAZABlAGQAIABlAHgAdAByAGEAIABSAGEAaQBuAGYAYQBsAGwAIABtAGkAbgAgAGEAbgBkACAAUgBhAGkAbgBmAGEAbABsACAAbQBhAHgAIABjAG8AbAB1AG0AbgBzACAAdABvACAAYwBhAGwAYwB1AGwAYQB0AGUAIAB6AG8AbgBlACAAZgByAG8AbQAgAHIAZQBhAGwAIAByAGEAaQBuAGYAYQBsAGwAIABkAGEAdABhAC4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIABaAG8AbgBlAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AaQBuAFwAIgAsACAAXAAiAFIAYQBpAG4AZgBhAGwAbAAgAG0AYQB4AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgAsACAAXAAiAEEAbgBuAHUAYQBsACAAcgBhAGkAbgBmAGEAbABsACAAXAB1ADAAMAAzAGUAIAA2ADAAMABtAG0AXAAiACwAIAA2ADAAMAAuADAAMAAxACwAIAA5ADkAOQA5ADkAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AdwAgAHIAYQBpAG4AZgBhAGwAbABcACIALAAgAFwAIgBBAG4AbgB1AGEAbAAgAHIAYQBpAG4AZgBhAGwAbAAgAGQiIAA2ADAAMABtAG0AXAAiACwAIAAtADkAOQA5ADkAOQA5ACwAIAA2ADAAMABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgADEALgAzADoAIABDAGwAaQBtAGEAdABlACAAYQBuAGQAIABSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlACAAYwBsAGEAcwBzAGkAZgBpAGMAYQB0AGkAbwBuAHMAIABhAG4AZAAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAEQAYQB0AGEAXABuACAAIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADQALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAZQBhAGMAaABpAG4AZwAgAFoAbwBuAGUAXAAiACwAIABcACIATABlAGEAYwBoAGkAbgBnACAAYwByAGkAdABlAHIAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABvAGMAYwB1AHIAcwBcACIALAAgAFwAIgCjAygANdhf3DXYTtw12FbcNdhb3CkAXAB1ADAAMAAzAGUAowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAGUAYQBjAGgAaQBuAGcAIABkAG8AZQBzACAAbgBvAHQAIABvAGMAYwB1AHIAXAAiACwAIABcACIAowMoADXYX9w12E7cNdhW3DXYW9wpAGQiowMoADXYONw12EfcMAApACsANdhg3DXYXNw12FbcNdhZ3CAANdhk3DXYTtw12GHcNdhS3DXYX9wgAA4hNdhc3DXYWdw12FHcNdhW3DXYW9w12FTcIAA12FDcNdhO3DXYXdw12E7cNdhQ3DXYVtw12GHcNdhm3FwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHQAaABhAHQAIABpAHMAIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgARABpAG0AZQBuAHMAaQBvAG4AbABlAHMAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBzACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALABcACIARgByAGEAYwBXAEUAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAWQBlAHMAIAAtACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAALQAgAG4AbwB0ACAAaQBuACAAbABlAGEAYwBoAGkAbgBnACAAegBvAG4AZQBcACIALAAgADAAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBuACAAZABhAHQAYQAgAHMAYwBvAHIAZQBzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFgAWABYAFgAWABYAFgAWABcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhAFwAbgAgACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAdABhACAAcwBvAHUAcgBjAGUAXAAiACwAIABcACIARABhAHQAYQAgAHMAYwBvAHIAZQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIASQBuAHQAZQByAG4AYQB0AGkAbwBuAGEAbAAgAHMAYwBvAHAAZQAgADMAIABkAGEAdABhAGIAYQBzAGUAXAAiACwAIAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHQAYQB0AGUAIABvAHIAIAByAGUAZwBpAG8AbgBhAGwAIABzAGMAbwBwAGUAIAAzACAAZABhAHQAYQBiAGEAcwBlAFwAIgAsACAAMwA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAG0AaQBzAHMAaQBvAG4AcwAgAGkAbgB0AGUAbgBzAGkAdAB5ACAAYwBhAGwAYwB1AGwAYQB0AGUAZAAgAGYAcgBvAG0AIABhAHAAcAByAG8AdgBlAGQAIABtAGUAdABoAG8AZABcACIALAAgADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBlAHIAaQBmAGkAZQBkACAAYwByAGUAZABlAG4AdABpAGEAbAAgAG0AYQB0AGMAaABpAG4AZwAgAEkAUwBPADEANAAwADYANwBcACIALAAgADUAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABcAG4ANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIAB0AGgAYQB0ACAAaQBzACAAYQB2AGEAaQBsAGEAYgBsAGUAIABmAG8AcgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAKABEAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoANQAuADUALgAyAC4AMwAgAEMAbwBuAHMAdABhAG4AdAAgAFAAYQByAGEAbQBlAHQAZQByAHMAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AYQB0AGkAbwBuAGEAbAAgAEkAbgB2AGUAbgB0AG8AcgB5ACAAUgBlAHAAbwByAHQAIABWAG8AbAB1AG0AZQAgADEAOgAgAEwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAIAAoADMALgBEAC4AYgAuADIAKQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgByAGEAYwBMAEUAQQBDAEgAXAAiACwAMAAuADIANABcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAFwAbgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcAG4ARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG4AaQB0AHIAbwBnAGUAbgAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgAoAGsAZwAgAE4AMgBPAC0ATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgA1AC4ANQAuADIALgAzACAAQwBvAG4AcwB0AGEAbgB0ACAAUABhAHIAYQBtAGUAdABlAHIAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAVgBvAGwAdQBtAGUAIAAxADoAIABFAHEAdQBhAHQAaQBvAG4AIAAzAC4ARAAuAEIAXwAxADAAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBGAGwAZQBhAGMAaABcACIALAAwAC4AMAAxADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAKABcACIAXAAiACkAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBcAG4AVABhAGIAbABlACAAQQAuADIALgAyAC4AMQBcAG4ATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByAHMAIABmAG8AcgAgAGkAbgBvAHIAZwBhAG4AaQBjACAAZgBlAHIAdABpAGwAaQBzAGUAcgAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgAgACgAawBnACAATgAyAE8ALQBOAC8AawBnACAATgApACAAKABFAEYATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AIABmAGEAYwB0AG8AcgBzACAAZgBvAHIAIABpAG4AbwByAGcAYQBuAGkAYwAgAGYAZQByAHQAaQBsAGkAcwBlAHIAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiACgAawBnACAATgAyAE8ALQBOACAALwAgAGsAZwAgAE4AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAxAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxADUALAAgADUALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAaQBvAG4AIABzAHkAcwB0AGUAbQAgAGoAXAAiACwAXAAiAEUARgBOADIATwBcACIALAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AIABvAG4AbAB5AFwAIgAsACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIABtAGUAdABoAG8AZABcACIALAAgAFwAIgBSAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAA1ADkALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAGMAcgBvAHAAXAAiACwAMAAuADAAMAA3ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvAG4ALQBpAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAMAAuADAAMAAxADgALAAgAFwAIgBQAGEAcwB0AHUAcgBlAFwAIgAsACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATABvAHcAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAIgAsADAALgAwADAAMQA4ACwAIABcACIAUABhAHMAdAB1AHIAZQBcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwACAAKABsAG8AdwAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAMgA5ACwAIABcACIAQwByAG8AcABcACIALAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAXAAiAEwAbwB3ACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcAAgACgAaABpAGcAaAAgAHIAYQBpAG4AZgBhAGwAbAApAFwAIgAsADAALgAwADAAOAAsACAAXAAiAEMAcgBvAHAAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBIAGkAZwBoACAAcgBhAGkAbgBmAGEAbABsAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAMAAuADAAMQA5ADkALAAgAFwAIgBTAHUAZwBhAHIAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsADAALgAwADAANQAzACwAIABcACIAQwBvAHQAdABvAG4AXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBhAGwAIABjAHIAbwBwAHMAXAAiACwAMAAuADAAMAA2ADQALAAgAFwAIgBIAG8AcgB0AGkAYwB1AGwAdAB1AHIAYQBsACAAYwByAG8AcABzAFwAIgAsACAAXAAiAEEAbgB5AFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABjAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnACkAXAAiACwAMAAuADAAMAAzACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBDAG8AbgB0AGkAbgB1AG8AdQBzACAAZgBsAG8AbwBkAGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBSAGkAYwBlACAAKABzAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnACkAXAAiACwAMAAuADAAMAA1ACwAIABcACIAUgBpAGMAZQBcACIALAAgAFwAIgBTAGkAbgBnAGwAZQAgAGEAbgBkACAAbQB1AGwAdABpAHAAbABlACAAZAByAGEAaQBuAGEAZwBlACwAIABvAHIAIABhAGwAdABlAHIAbgBhAHQAZQAgAHcAZQB0AHQAaQBuAGcAIABhAG4AZAAgAGQAcgB5AGkAbgBnAFwAIgAsACAAXAAiAEEAbgB5AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAMAAuADAAMAAyADYALAAgAFwAIgBBAHEAdQBhAGMAdQBsAHQAdQByAGUAXAAiACwAIABcACIAQQBuAHkAXAAiACwAIABcACIAQQBuAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAwAC4AMAAwADEAOAAsACAAXAAiAEYAbwByAGUAcwB0AHIAeQBcACIALAAgAFwAIgBBAG4AeQBcACIALAAgAFwAIgBBAG4AeQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADUALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBGACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABkAHUAcABsAGkAYwBhAHQAZQAgAFwAdQAwADAAMgA3AEEAcQB1AGEAYwB1AGwAdAB1AHIAZQBcAHUAMAAwADIANwAgAHIAbwB3AC4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFIAZQBtAG8AdgBlAGQAIABhAHMAdABlAHIAaQBzAGsAcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAcAByAG8AZAB1AGMAdABpAG8AbgAgAHMAeQBzAHQAZQBtACAAbwBuAGwAeQBcAHUAMAAwADIANwAsACAAXAB1ADAAMAAyADcAcgBhAGkAbgBmAGEAbABsACAAegBvAG4AZQBcAHUAMAAwADIANwAgAGEAbgBkACAAXAB1ADAAMAAyADcAaQByAHIAaQBnAGEAdABpAG8AbgAgAG0AZQB0AGgAbwBkAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AG4AbwBuAC0AaQByAHIAaQBnAGEAdABlAGQAIABwAGEAcwB0AHUAcgBlAFwAdQAwADAAMgA3ACAAcgBvAHcAIAB3AGkAdABoACAAcwBhAG0AZQAgAEUARgAgAGYAbwByACAAbABvAHcAIABhAG4AZAAgAGgAaQBnAGgAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAIAB0AG8AIABhAGkAZAAgAGwAbwBvAGsAdQBwAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXABuAFYARQBFAFIARwAgADIAMAAyADYAOgAgAEMAaABhAHAAdABlAHIAIAAxACwAIABzAGUAYwB0AGkAbwBuACAAMQAuADgALgAyACAATABlAGEAYwBoAGkAbgBnACwAIABjAGwAaQBtAGEAdABlACAAYQBuAGQAIAByAGEAaQBuAGYAYQBsAGwAIAB6AG8AbgBlAHMAXABuAEkAUABDAEMAOgAgAE4AMgBPACAARQBNAEkAUwBTAEkATwBOAFMAIABGAFIATwBNACAATQBBAE4AQQBHAEUARAAgAFMATwBJAEwAUwAsACAAQQBOAEQAIABDAE8AMgAgAEUATQBJAFMAUwBJAE8ATgBTACAARgBSAE8ATQAgAEwASQBNAEUAIABBAE4ARAAgAFUAUgBFAEEAIABBAFAAUABMAEkAQwBBAFQASQBPAE4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAFcARQBUACAAZgBvAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuACAAdAB5AHAAZQBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBkAGkAbQBlAG4AcwBpAG8AbgBsAGUAcwBzAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAQwBoAGEAcAB0AGUAcgAgADEALAAgAHMAZQBjAHQAaQBvAG4AIAAxAC4AOAAuADIAIABMAGUAYQBjAGgAaQBuAGcALAAgAGMAbABpAG0AYQB0AGUAIABhAG4AZAAgAHIAYQBpAG4AZgBhAGwAbAAgAHoAbwBuAGUAcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEkAUABDAEMAIAAyADAAMQA5ACAAUgBlAGYAaQBuAGUAbQBlAG4AdAAgAFYAbwBsAHUAbQBlACAANAA6ACAAQwBoAGEAcAB0AGUAcgAgADEAMQA6ACAATgAyAE8AIABFAG0AaQBzAHMAaQBvAG4AcwAgAGYAcgBvAG0AIABNAGEAbgBhAGcAZQBkACAAUwBvAGkAbABzACwAIABhAG4AZAAgAEMATwAyACAARQBtAGkAcwBzAGkAbwBuAHMAIABmAHIAbwBtACAATABpAG0AZQAgAGEAbgBkACAAVQByAGUAYQAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADYALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEkAcgByAGkAZwBhAHQAaQBvAG4AIAB0AHkAcABlACAAaQByAFwAIgAsAFwAIgBGAHIAYQBjAFcARQBUAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AdAAgAGkAcgByAGkAZwBhAHQAZQBkAFwAIgAsACAAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAaQBwACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBwAHIAaQBuAGsAbABlAHIAIABpAHIAcgBpAGcAYQB0AGkAbwBuAFwAIgAsACAAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAcgBmAGEAYwBlACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATwB0AGgAZQByACAAaQByAHIAaQBnAGEAdABpAG8AbgBcACIALAAgADEAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBBAFIASQBBAFQASQBPAE4AIABGAFIATwBNACAAUwBPAFUAUgBDAEUAIABEAEEAVABBADoAIABUAGEAYgBsAGUAIABjAHIAZQBhAHQAZQBkACAAYgBhAHMAZQBkACAAbwBuACAAVgBFAEUAUgBHACAAdABlAHgAdAAgAFwAdQAwADAAMgA3AEEAcgBlAGEAcwAgAGEAcgBlACAAcwB1AGIAagBlAGMAdAAgAHQAbwAgAGwAZQBhAGMAaABpAG4AZwAgACgAaQAuAGUALgAsACAAaQBuACAAdABoAGUAIABsAGUAYQBjAGgAaQBuAGcAIAB6AG8AbgBlACkAIAB3AGgAZQBuAC4ALgAuACAAdABoAGUAIABsAGEAbgBkACAAaQBzACAAaQByAHIAaQBnAGEAdABlAGQAIAAoAGUAeABjAGUAcAB0ACAAZAByAGkAcAAgAGkAcgByAGkAZwBhAHQAaQBvAG4AKQAuAFwAdQAwADAAMgA3AFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXABuAFQAYQBiAGwAZQAgAEEALgAyAC4AMgAuADIAOgAgAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQAgACgARQBGAFAAUgBQACkAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEUAbQBpAHMAcwBpAG8AbgAgAGYAYQBjAHQAbwByACAAZgBvAHIAIAB1AHIAaQBuAGUAIABhAG4AZAAgAGQAdQBuAGcAIABkAGUAcABvAHMAaQB0AGUAZAAgAG8AbgAgAHAAYQBzAHQAdQByAGUALAAgAHIAYQBuAGcAZQAgAG8AcgAgAHAAYQBkAGQAbwBjAGsAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAawBnACAATgAyAE8AIAAtACAATgAgAC8AIABrAGcAIABOAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADIALgAyAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIABcACIARQBGAFAAUgBQAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBXAGUAdAAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA2ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAcgB5ACAAYwBsAGkAbQBhAHQAZQAgAHoAbwBuAGUAXAAiACwAIAAwAC4AMAAwADIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuACAAIABDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQAgAEQAQQBUAEEAOgAgAEMAaABhAG4AZwBlAGQAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAHMAXAB1ADAAMAAyADcAIAB0AG8AIABzAGkAbgBnAHUAbABhAHIAIABcAHUAMAAwADIANwBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAdQAwADAAMgA3ACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AbwBuAHQAaABzACAAdABvACAAUwBlAGEAcwBvAG4AcwAgAE0AYQBwAHAAaQBuAGcAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAG8AbgB0AGgAcwBUAG8AUwBlAGEAcwBvAG4AcwBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBvAG4AdABoAHMAVABvAFMAZQBhAHMAbwBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMQAzACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AbgB0AGgAXAAiACwAIABcACIAUwBlAGEAcwBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEoAYQBuAHUAYQByAHkAXAAiACwAIABcACIAUwB1AG0AbQBlAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEYAZQBiAHIAdQBhAHIAeQBcACIALAAgAFwAIgBTAHUAbQBtAGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBhAHIAYwBoAFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHAAcgBpAGwAXAAiACwAIABcACIAQQB1AHQAdQBtAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AYQB5AFwAIgAsACAAXAAiAEEAdQB0AHUAbQBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbgBlAFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBKAHUAbAB5AFwAIgAsACAAXAAiAFcAaQBuAHQAZQByAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAHUAZwB1AHMAdABcACIALAAgAFwAIgBXAGkAbgB0AGUAcgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAHAAdABlAG0AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE8AYwB0AG8AYgBlAHIAXAAiACwAIABcACIAUwBwAHIAaQBuAGcAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE4AbwB2AGUAbQBiAGUAcgBcACIALAAgAFwAIgBTAHAAcgBpAG4AZwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABlAGMAZQBtAGIAZQByAFwAIgAsACAAXAAiAFMAdQBtAG0AZQByAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIAAgAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AbwBuAHQAaABzAFQAbwBTAGUAYQBzAG8AbgBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAGEAbgB1AHIAZQAgAE0AYQBuAGEAZwBlAG0AZQBuAHQAIAATICAATQBlAHQAaABhAG4AZQAgAGMAbwBuAHYAZQByAHMAaQBvAG4AIABmAGEAYwB0AG8AcgAgAHAAZQByACAAdABlAG0AcABlAHIAYQB0AHUAcgBlACAAegBvAG4AZQAgACgAZgByAGEAYwB0AGkAbwBuACkAIAAoAE0AQwBGAGkAbQApAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgA4AC4AMQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATQBDAEYAVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAyACwAIAAxADYALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdAB1AHIAZQAgAHoAbwBuAGUAXAAiACwAIABcACIATQBBAFQAIAAoALoAQwApAFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQwBvAHYAZQByAGUAZAAgAGwAYQBnAG8AbwBuAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAUwBsAHUAcgByAHkAIAAoAHcAaQB0AGgAbwB1AHQAIABuAGEAdAB1AHIAYQBsACAAYwByAHUAcwB0ACkAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAGIAKQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABTAHQAbwByAGEAZwBlACAAXAB1ADAAMAAzAGMAMQAgAG0AbwBuAHQAaABcACIALAAgAFwAIgBEAGUAZQBwACAATABpAHQAdABlAHIAXAAiACwAIABcACIAUABvAHUAbAB0AHIAeQAgAE0AYQBuAHUAcgBlACAAKAB3AGkAdABoAC8AdwBpAHQAaABvAHUAdAAgAGwAaQB0AHQAZQByACkAXAAiACwAIABcACIAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAaQBuAHQAbwAgAHAAZQBsAGwAZQB0AGkAegBlAGQAIABmAGUAcgB0AGkAbABpAHMAZQByAFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACwAIABSAGEAbgBnAGUAIABhAG4AZAAgAFAAYQBkAGQAbwBjAGsAIAAoAGMAKQAoAGQAKQBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAXAAiAGQiMQAwAFwAIgAsACAAMAAuADYANgAsACAAMAAuADEALAAgADAALgAxACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADAAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBvAG8AbABcACIALAAgADEAMQAsACAAMAAuADYAOAAsACAAMAAuADEALAAgADAALgAxADEALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAyACwAIAAwAC4ANwAsACAAMAAuADEALAAgADAALgAxADMALAAgADAALgAwADAAMQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbwBsAFwAIgAsACAAMQAzACwAIAAwAC4ANwAxACwAIAAwAC4AMQAsACAAMAAuADEANAAsACAAMAAuADAAMAAxACwAIAAwAC4AMAAwADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwBvAGwAXAAiACwAIAAxADQALAAgADAALgA3ADMALAAgADAALgAxACwAIAAwAC4AMQA1ACwAIAAwAC4AMAAwADEALAAgADAALgAwADAANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAxADUALAAgADAALgA3ADQALAAgADAALgAxACwAIAAwAC4AMQA3ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA2ACwAIAAwAC4ANwA1ACwAIAAwAC4AMQAsACAAMAAuADEAOAAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEANwAsACAAMAAuADcANgAsACAAMAAuADEALAAgADAALgAyACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMQA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMQA4ACwAIAAwAC4ANwA3ACwAIAAwAC4AMQAsACAAMAAuADIAMgAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADEAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADEAOQAsACAAMAAuADcANwAsACAAMAAuADEALAAgADAALgAyADQALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAxADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADAALAAgADAALgA3ADgALAAgADAALgAxACwAIAAwAC4AMgA2ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgAxACwAIAAwAC4ANwA4ACwAIAAwAC4AMQAsACAAMAAuADIAOQAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIAMQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIAMgAsACAAMAAuADcAOAAsACAAMAAuADEALAAgADAALgAzADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAG0AcABlAHIAYQB0AGUAXAAiACwAIAAyADMALAAgADAALgA3ADkALAAgADAALgAxACwAIAAwAC4AMwA0ACwAIAAwAC4AMAAwADUALAAgADAALgAwADEALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgAzADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQBtAHAAZQByAGEAdABlAFwAIgAsACAAMgA0ACwAIAAwAC4ANwA5ACwAIAAwAC4AMQAsACAAMAAuADMANwAsACAAMAAuADAAMAA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAyACwAIAAwAC4AMAAzACwAIAAwAC4AMAA0ACwAIAAwAC4AMAAxADUALAAgADAALgAwADEANQAsACAAMAAsACAAMAAsACAAMAAuADAAMAA0ADcALAAgADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAGUAbQBwAGUAcgBhAHQAZQBcACIALAAgADIANQAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADEALAAgADAALgAwADAANQAsACAAMAAuADAAMQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADUAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANgAsACAAMAAuADcAOQAsACAAMAAuADEALAAgADAALgA0ADQALAAgADAALgAwADEALAAgADAALgAwADEANQAsACAAMAAuADAAMgAsACAAMAAuADAAMwAsACAAMAAuADAANAAsACAAMAAuADAAMQA1ACwAIAAwAC4AMAAxADUALAAgADAALAAgADAALAAgADAALgAwADAANAA3ACwAIAAyADYAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBhAHIAbQBcACIALAAgADIANwAsACAAMAAuADgALAAgADAALgAxACwAIAAwAC4ANAA4ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFcAYQByAG0AXAAiACwAIABcACIAZSIyADgAXAAiACwAIAAwAC4AOAAsACAAMAAuADEALAAgADAALgA1ACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxADUALAAgADAALgAwADIALAAgADAALgAwADMALAAgADAALgAwADQALAAgADAALgAwADEANQAsACAAMAAuADAAMQA1ACwAIAAwACwAIAAwACwAIAAwAC4AMAAwADQANwAsACAAMgA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwBcACIALAAgAFwAIgBEAGEAaQBsAHkAIABzAHAAcgBlAGEAZABcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoAG8AdQB0ACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIAUABhAHMAdAB1AHIAZQAgAHIAYQBuAGcAZQAgAGEAbgBkACAAcABhAGQAZABvAGMAawBcACIALAAgAFwAIgBNAEEAVAAgAHIAYQB3AFwAIgAgAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAEYAUgBPAE0AIABTAE8AVQBSAEMARQA6ACAAQQBkAGQAZQBkACAAcgBvAHcAIABvAGYAIABOAEkAUgAgAE0ATQBBACAAZABlAGYAaQBuAGkAdABpAG8AbgBzACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuACAARAB1AHAAbABpAGMAYQB0AGUAZAAgAFwAdQAwADAAMgA3AFAAbwB1AGwAdAByAHkAIAB3AGkAdABoACAAYQBuAGQAIAB3AGkAdABoAG8AdQB0ACAAbABpAHQAdABlAHIAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABzAGUAcABhAHIAYQB0AGUAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgAgAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE0AQQBUACAAcgBhAHcAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAbABsAG8AdwAgAGwAbwBvAGsAdQBwACAAbwBmACAAbgB1AG0AYgBlAHIAcwAuAFwAIgApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBPAHIAZwBhAG4AaQBjAEYAZQByAHQAaQBsAGkAcwBlAHIAQQBuAGQAQwByAG8AcABSAGUAcwBpAGQAdQBlAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAIABmAG8AcgAgAG8AcgBnAGEAbgBpAGMAIABmAGUAcgB0AGkAbABpAHMAZQByACAAYQBuAGQAIABjAHIAbwBwACAAcgBlAHMAaQBkAHUAZQBzACAAcgBlAHQAdQByAG4AZQBkACAAdABvACAAdABoAGUAIABzAG8AaQBsAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEYATgBpACAAXAB1ADAAMAAyADYAIABFAEYATgAyAE8AaQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAGsAZwAgAE4AMgBPACAALQAgAE4AIAAvACAAawBnACAATgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE8AcgBnAGEAbgBpAGMARgBlAHIAdABpAGwAaQBzAGUAcgBBAG4AZABDAHIAbwBwAFIAZQBzAGkAZAB1AGUAcwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMgAuADEALgA0AFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAXAAiAEUARgBOAGkAIABcAHUAMAAwADIANgAgAEUARgBOADIATwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVwBlAHQAIABjAGwAaQBtAGEAdABlACAAegBvAG4AZQBcACIALAAgADAALgAwADAANgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAHIAeQAgAGMAbABpAG0AYQB0AGUAIAB6AG8AbgBlAFwAIgAsACAAMAAuADAAMAA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATwByAGcAYQBuAGkAYwBGAGUAcgB0AGkAbABpAHMAZQByAEEAbgBkAEMAcgBvAHAAUgBlAHMAaQBkAHUAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAiAH0ALAB7ACIAcABhAHQAaAAiADoAIgAvAHAAcgBvAGoAZQBjAHQAcwAvAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAE4AMgBPACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUATgAyAE8AOgAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAE4AMgBPACkAXABuAEcAVwBQAE4AMgBPADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAATgAyAE8AKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBOADIATwAsACAARwBXAFAAXwBOADIATwAsAFwAbgAgACAAIAAgAEUAXwBOADIATwAgACoAIABHAFcAUABfAE4AMgBPAFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAE4AMgBPACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AE4AMgBPAH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AE4AMgBPAH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBOADIATwBcACIALABcACIATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAATgAyAE8AKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAATgAyAE8AXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABuAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABOADIATwApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgBDAG8AbgB2AGUAcgB0ACAAbQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAdABvACAAYwBhAHIAYgBvAG4AIABkAGkAbwB4AGkAZABlACAAZQBxAHUAaQB2AGEAbABlAG4AdAAgAGUAbQBpAHMAcwBpAG8AbgBzAFwAbgBFAEMASAA0ACAAQwBPADIAZQBcAG4AdAAgAEMATwAyAGUAXABuAEUAQwBIADQAOgAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgACgAdAAgAEMASAA0ACkAXABuAEcAVwBQAEMASAA0ADoAIABnAGwAbwBiAGEAbAAgAHcAYQByAG0AaQBuAGcAIABwAG8AdABlAG4AdABpAGEAbAAgAGYAbwByACAAbQBlAHQAaABhAG4AZQAgACgAdAAgAEMATwAyAC0AZQAgAC8AIAB0ACAAQwBIADQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEUAXwBDAEgANAAsACAARwBXAFAAXwBDAEgANAAsAFwAbgAgACAAIAAgAEUAXwBDAEgANAAgACoAIABHAFcAUABfAEMASAA0AFwAbgAgACAAKQBcAG4AOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBvAG4AdgBlAHIAdAAgAG0AZQB0AGgAYQBuAGUAIABlAG0AaQBzAHMAaQBvAG4AcwAgAHQAbwAgAGMAYQByAGIAbwBuACAAZABpAG8AeABpAGQAZQAgAGUAcQB1AGkAdgBhAGwAZQBuAHQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAEMASAA0ACAAQwBPADIAZQBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAdAAgAEMATwAyAGUAXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBPADIAXwBlACAAPQAgAEUAXwB7AEMASAA0AH0AIABcAFwAdABpAG0AZQBzACAARwBXAFAAXwB7AEMASAA0AH0AXAAiACkAOwBcAG4AXABuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBDAEgANABcACIALABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAKAB0ACAAQwBIADQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARwBXAFAAQwBIADQAXAAiACwAXAAiAEcAbABvAGIAYQBsACAAdwBhAHIAbQBpAG4AZwAgAHAAbwB0AGUAbgB0AGkAYQBsACAAZgBvAHIAIABtAGUAdABoAGEAbgBlACAAKAB0ACAAQwBPADIALQBlACAALwAgAHQAIABDAEgANAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7ACIAfQAsAHsAIgBwAGEAdABoACIAOgAiAC8AcAByAG8AagBlAGMAdABzAC8AQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhACIALAAiAHQAZQB4AHQAIgA6ACIALwAqAFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgBTAG8AdQByAGMAZQAgAGQAYQB0AGEAIAB0AGgAYQB0ACAAaQBzACAAYwBvAG0AbQBvAG4AIABhAGMAcgBvAHMAcwAgAGEAbABsACAAbABpAHYAZQBzAHQAbwBjAGsAIAB0AHkAcABlAHMAXABuAEUAeABjAGUAbAAgAG0AbwBkAHUAbABlACAAbgBhAG0AZQA6ACAAUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuAFMAbwB1AHIAYwBlADoAIABOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQBcAG4ATgBJAFIAXwAyADAAMgAzAF8AVgBvAGwAMQBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AFwAbgA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBcAG4ARgByAGEAYwBXAEUAVABNAE0AUwBpACAAPQAgAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcAG4AKABUAGEAYgBsAGUAIABBADUALgA1AC4AMQAwAC4AMgAgAGkAcwAgAHIAZQBmAGUAcgBlAG4AYwBlAGQAIABpAG4AIABOAEkAUgAgAGIAdQB0ACAAMQAgAGkAcwAgAHUAcwBlAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABhAHYAYQBpAGwAYQBiAGwAZQAgAGYAbwByACAAbABlAGEAYwBoAGkAbgBnACAAYQBuAGQAIAByAHUAbgBvAGYAZgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMAVwBFAFQATQBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKAAxACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXABuAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTACAAPQAgADAALgAwADIAIAAoAEcAZwAgAE4ALwBHAGcAIABhAHAAcABsAGkAZQBkACkAIAAoAEMAUwAgAEUARgAsACAAcwBvAHUAcgBjAGUAIABJAFAAQwBDACAAKAAyADAAMQA5ACkAKQAgAFwAbgBmAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAbABvAHMAdAAgAHQAaAByAG8AdQBnAGgAIABsAGUAYQBjAGgAaQBuAGcAIABhAG4AZAAgAHIAdQBuAG8AZgBmAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAE4AIABsAG8AcwB0ACAAdABoAHIAbwB1AGcAaAAgAGwAZQBhAGMAaABpAG4AZwAgAGEAbgBkACAAcgB1AG4AbwBmAGYAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATgBhAHQAaQBvAG4AYQBsACAASQBuAHYAZQBuAHQAbwByAHkAIABSAGUAcABvAHIAdAAgADIAMAAyADMAIABWAG8AbAB1AG0AZQAgADEAOgAgAEUAcQB1AGEAdABpAG8AbgBzACAAMwAuAEIALgA1AGEAXwAzACwAIAAzAC4AQgAuADUAYwBfADMALAAgADMALgBCAC4ANQBkAF8AMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAEwARQBBAEMASABfAE0AUwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA4ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AGkAbwBuACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIARQBtAGkAcwBzAGkAbwBuACAAZgBhAGMAdABvAHIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAHIAcgBpAGcAYQB0AGUAZAAgAHAAYQBzAHQAdQByAGUAXAAiACwAIAAwAC4AMAAwADUAOQA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIASQByAHIAaQBnAGEAdABlAGQAIABjAHIAbwBwAFwAIgAsACAAMAAuADAAMAA3ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAcABhAHMAdAB1AHIAZQBcACIALAAgADAALgAwADAAMQA4ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAG8AbgAtAGkAcgByAGkAZwBhAHQAZQBkACAAYwByAG8AcABcACIALAAgADAALgAwADAANAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAHUAZwBhAHIAIABjAGEAbgBlAFwAIgAsACAAMAAuADAAMQA5ADkAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAbwB0AHQAbwBuAFwAIgAsACAAMAAuADAAMAA1ADMAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEgAbwByAHQAaQBjAHUAbAB0AHUAcgBlAFwAIgAsACAAMAAuADAAMAA2ADQAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXABuAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAYQBiAGwAZQAgADUALgAxADIAIABBAGQAZABpAHQAaQBvAG4AYQBsACAAcwB5AG0AYgBvAGwAcwAgAHUAcwBlAGQAIABpAG4AIABhAGwAZwBvAHIAaQB0AGgAbQBzACAAZgBvAHIAIABtAGEAbgB1AHIAZQAgAHIAZQBsAGEAdABlAGQAIABlAG0AaQBzAHMAaQBvAG4AcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBNAE0AUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBOAGEAdABpAG8AbgBhAGwAIABJAG4AdgBlAG4AdABvAHIAeQAgAFIAZQBwAG8AcgB0ACAAMgAwADIAMwAgAFYAbwBsAHUAbQBlACAAMQA6ACAAVABhAGIAbABlACAANQAuADEAMgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAOQAsACAAMwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwB5AG0AYgBvAGwAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABtAGEAbgBhAGcAZQBtAGUAbgB0ACAAcwB5AHMAdABlAG0AXAAiACwAIABcACIAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxAFwAIgAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiACwAIABcACIAQQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgAbQA9ADEAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADIAXAAiACwAIABcACIATABpAHEAdQBpAGQAIABzAHkAcwB0AGUAbQBzAFwAIgAsACAAXAAiAEwAaQBxAHUAaQBkACAAcwB5AHMAdABlAG0AcwAgACgAbQA9ADIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADMAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAXAAiACwAIABcACIARABhAGkAbAB5ACAAcwBwAHIAZQBhAGQAIAAoAG0APQAzACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGEAXAAiACwAIABcACIAUwB1AG0AcAAgAGEAbgBkACAAZABpAHMAcABlAHIAcwBhAGwAIABzAHkAcwB0AGUAbQBcACIALAAgAFwAIgBTAHUAbQBwACAAYQBuAGQAIABkAGkAcwBwAGUAcgBzAGEAbAAgAHMAeQBzAHQAZQBtACAAKABtAD0AMwBhACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAzAGIAXAAiACwAIABcACIARAByAGEAaQBuAHMAIAB0AG8AIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAEQAcgBhAGkAbgBzACAAdABvACAAcABhAGQAZABvAGMAawAgACgAbQA9ADMAYgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIANABcACIALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAHMAdABvAHIAYQBnAGUAIAAoAG0APQA0ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA1AFwAIgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAIAAoAG0APQA1ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgA2AFwAIgAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiACwAIABcACIAQwBvAG0AcABvAHMAdABpAG4AZwAgACgAcABhAHMAcwBpAHYAZQAgAHcAaQBuAGQAcgBvAHcAKQAgACgAbQA9ADYAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADcAXAAiACwAIABcACIARABpAGcAZQBzAHQAZQByACAALwAgAGMAbwB2AGUAcgBlAGQAIABsAGEAZwBvAG8AbgBzAFwAIgAsACAAXAAiAEQAaQBnAGUAcwB0AGUAcgAgAC8AIABjAG8AdgBlAHIAZQBkACAAbABhAGcAbwBvAG4AcwAgACgAbQA9ADcAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADgAXAAiACwAIABcACIARABlAGUAcAAgAGwAaQB0AHQAZQByAFwAIgAsACAAXAAiAEQAZQBlAHAAIABsAGkAdAB0AGUAcgAgACgAbQA9ADgAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADkAXAAiACwAIABcACIAUABpAHQAIABzAHQAbwByAGEAZwBlAFwAIgAsACAAXAAiAFAAaQB0ACAAcwB0AG8AcgBhAGcAZQAgACgAbQA9ADkAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMABcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwBcACIALAAgAFwAIgBQAG8AdQBsAHQAcgB5ACAAbQBhAG4AdQByAGUAIAB3AGkAdABoACAAYgBlAGQAZABpAG4AZwAgACgAbQA9ADEAMAApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnAFwAIgAsACAAXAAiAFAAbwB1AGwAdAByAHkAIABtAGEAbgB1AHIAZQAgAHcAaQB0AGgAbwB1AHQAIABiAGUAZABkAGkAbgBnACAAKABtAD0AMQAxACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADEAYQBcACIALAAgAFwAIgBCAGUAbAB0ACAAbQBhAG4AdQByAGUAIAByAGUAbQBvAHYAYQBsAFwAIgAsACAAXAAiAEIAZQBsAHQAIABtAGEAbgB1AHIAZQAgAHIAZQBtAG8AdgBhAGwAIAAoAG0APQAxADEAYQApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAMQAxAGIAXAAiACwAIABcACIATQBhAG4AdQByAGUAIABzAHQAbwByAGUAZAAgAGkAbgAgAGgAbwB1AHMAZQBcACIALAAgAFwAIgBNAGEAbgB1AHIAZQAgAHMAdABvAHIAZQBkACAAaQBuACAAaABvAHUAcwBlACAAKABtAD0AMQAxAGIAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEAMgBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAHAAcgBvAGMAZQBzAHMAaQBuAGcAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABwAHIAbwBjAGUAcwBzAGkAbgBnACAAKABtAD0AMQAyACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgAxADMAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AIAAoAG0APQAxADMAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiADEANABcACIALAAgAFwAIgBQAGEAcwB0AHUAcgBlACAAcgBhAG4AZwBlACAAYQBuAGQAIABwAGEAZABkAG8AYwBrAFwAIgAsACAAXAAiAFAAYQBzAHQAdQByAGUAIAByAGEAbgBnAGUAIABhAG4AZAAgAHAAYQBkAGQAbwBjAGsAIAAoAG0APQAxADQAKQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGMAYQB0AHQAbABlACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQgBlAGUAZgBDAGEAdAB0AGwAZQBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBCAGUAZQBmAEMAYQB0AHQAbABlAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADkALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIABmAG8AcgAgAG0AYQBuAHUAZgBhAGMAdAB1AHIAaQBuAGcAIABiAGUAZQBmAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBhAHQAdABsAGUALAAgAGYAbwByACAAcAByAGkAbQBlACAAYgBlAGUAZgBcACIALAAgAFwAIgBOAFMAVwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEMAYQB0AHQAbABlACwAIAB3AGUAYQBuAGUAcgBzAFwAIgAsACAAXAAiAE4AVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFEATABEAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUwBBAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVABBAFMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBWAEkAQwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFcAQQBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQwBoAGkAYwBrAGUAbgBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AVgBhAGkAcgBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEMAaABpAGMAawBlAG4AcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AQwBoAGkAYwBrAGUAbgBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBDAGgAaQBjAGsAZQBuAHMAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMgAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAG8AZAB1AGMAdABcACIALAAgAFwAIgBTAG8AdQByAGMAZQAgAHIAZQBnAGkAbwBuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAQwBoAGkAYwBrAGUAbgBzAFwAIgAsACAAXAAiAEEAdQBzAHQAcgBhAGwAaQBhAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARABhAGkAcgB5ACAAYwBhAHQAdABsAGUAIABwAHIAbwBkAHUAYwB0AHMAIABmAG8AcgAgAHMAYwBvAHAAZQAgADMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBWAGEAaQByAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8ARABhAGkAcgB5AGMAYQB0AHQAbABlAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBEAGEAaQByAHkAYwBhAHQAdABsAGUAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATABpAGYAZQBjAHkAYwBsAGUAcwAuACAAKAAyADAAMgA2ACkALgAgAEcAcgBlAGUAbgBoAG8AdQBzAGUAIABHAGEAcwAgAEUAbQBpAHMAcwBpAG8AbgAgAEkAbgB0AGUAbgBzAGkAdABpAGUAcwAgAGYAbwByACAATQBhAHQAZQByAGkAYQBsACAASQBuAHAAdQB0AHMAIAB0AG8AIABBAHUAcwB0AHIAYQBsAGkAYQBuACAAQQBnAHIAaQBjAHUAbAB0AHUAcgBlACwAIABGAGkAcwBoAGUAcgBpAGUAcwAgAGEAbgBkACAARgBvAHIAZQBzAHQAcgB5AC4AIABWAGUAcgBzAGkAbwBuACAANAA4AC4AIABkAG8AaQAgADEAMAAuADUAMgA4ADEALwB6AGUAbgBvAGQAbwAuADEAOQA2ADUANgA1ADgAMABcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAEQAYQBpAHIAeQBjAGEAdAB0AGwAZQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBQAHIAbwBkAHUAYwB0AFwAIgAsACAAXAAiAFMAbwB1AHIAYwBlACAAcgBlAGcAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGEAaQByAHkAIABjAG8AdwBzAFwAIgAsACAAXAAiAFYASQBDAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBQAGkAZwBzACAAcAByAG8AZAB1AGMAdABzACAAZgBvAHIAIABzAGMAbwBwAGUAIAAzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUABpAGcAcwBfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEwAaQBmAGUAYwB5AGMAbABlAHMALgAgACgAMgAwADIANgApAC4AIABHAHIAZQBlAG4AaABvAHUAcwBlACAARwBhAHMAIABFAG0AaQBzAHMAaQBvAG4AIABJAG4AdABlAG4AcwBpAHQAaQBlAHMAIABmAG8AcgAgAE0AYQB0AGUAcgBpAGEAbAAgAEkAbgBwAHUAdABzACAAdABvACAAQQB1AHMAdAByAGEAbABpAGEAbgAgAEEAZwByAGkAYwB1AGwAdAB1AHIAZQAsACAARgBpAHMAaABlAHIAaQBlAHMAIABhAG4AZAAgAEYAbwByAGUAcwB0AHIAeQAuACAAVgBlAHIAcwBpAG8AbgAgADQAOAAuACAAZABvAGkAIAAxADAALgA1ADIAOAAxAC8AegBlAG4AbwBkAG8ALgAxADkANgA1ADYANQA4ADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBQAGkAZwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADIALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAaQBnAHMAXAAiACwAIABcACIAQQB1AHMAdAByAGEAbABpAGEAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFMAaABlAGUAcAAgAHAAcgBvAGQAdQBjAHQAcwAgAGYAbwByACAAcwBjAG8AcABlACAAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFYAYQBpAHIAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAFAAcgBvAGQAdQBjAHQAXwBTAGgAZQBlAHAAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AUAByAG8AZAB1AGMAdABfAFMAaABlAGUAcABfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBMAGkAZgBlAGMAeQBjAGwAZQBzAC4AIAAoADIAMAAyADYAKQAuACAARwByAGUAZQBuAGgAbwB1AHMAZQAgAEcAYQBzACAARQBtAGkAcwBzAGkAbwBuACAASQBuAHQAZQBuAHMAaQB0AGkAZQBzACAAZgBvAHIAIABNAGEAdABlAHIAaQBhAGwAIABJAG4AcAB1AHQAcwAgAHQAbwAgAEEAdQBzAHQAcgBhAGwAaQBhAG4AIABBAGcAcgBpAGMAdQBsAHQAdQByAGUALAAgAEYAaQBzAGgAZQByAGkAZQBzACAAYQBuAGQAIABGAG8AcgBlAHMAdAByAHkALgAgAFYAZQByAHMAaQBvAG4AIAA0ADgALgAgAGQAbwBpACAAMQAwAC4ANQAyADgAMQAvAHoAZQBuAG8AZABvAC4AMQA5ADYANQA2ADUAOAAwAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBQAHIAbwBkAHUAYwB0AF8AUwBoAGUAZQBwAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADgALAAgADIALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBvAGQAdQBjAHQAXAAiACwAIABcACIAUwBvAHUAcgBjAGUAIAByAGUAZwBpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABtAHUAdAB0AG8AbgBcACIALAAgAFwAIgBBAHUAcwB0AHIAYQBsAGkAYQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAaABlAGUAcAAsACAAZgBvAHIAIABwAHIAaQBtAGUAIABsAGEAbQBiAFwAIgAsACAAXAAiAE4AUwBXAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAUQBMAEQAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBTAEEAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBcACIALAAgAFwAIgBUAEEAUwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFwAIgAsACAAXAAiAFYASQBDAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABcACIAXAAiACwAIABcACIAVwBBAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAiACwAIgB0AGUAeAB0ACIAOgAiAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAUgBvAHcAcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAGEAbgBkAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFIATwBXACgAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwAKQAgACsAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACAALQAgADEAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwALABcAG4AIAAgAEMATwBMAFUATQBOACgAVABhAGIAbABlAEgAZQBhAGQAZQByAEMAZQBsAGwAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEQAaQBzAHAAbABhAHkAQQByAHIAYQB5AEkAbgBUAGEAYgBsAGUAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIABBAHIAcgBhAHkARABhAHQAYQAsACAAVABhAGIAbABlAGgAZQBhAGQAZQByAEMAZQBsAGwALAAgAFIAbwB3AHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBhAG4AZABBAHIAcgBhAHkALAAgAFsAQwBvAGwAdQBtAG4AcwBCAGUAdAB3AGUAZQBuAEgAZQBhAGQAZQByAEEAbgBkAEEAcgByAGEAeQBdACwAXABuACAASQBGAEUAUgBSAE8AUgAoAFwAbgAgACAAIAAgACAASQBOAEQARQBYACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFUATgBJAFEAVQBFACgAQQByAHIAYQB5AEQAYQB0AGEAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFIATwBXACgAKQAtAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAoAFQAYQBiAGwAZQBoAGUAYQBkAGUAcgBDAGUAbABsACwAIABSAG8AdwBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAYQBuAGQAQQByAHIAYQB5ACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABDAE8ATABVAE0ATgAoACkALQBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQQByAHIAYQB5AFQAYQBiAGwAZQBDAG8AbAB1AG0AbgBTAHQAYQByAHQATgB1AG0AYgBlAHIAKABUAGEAYgBsAGUAaABlAGEAZABlAHIAQwBlAGwAbAApACAAKwBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABDAG8AbAB1AG0AbgBzAEIAZQB0AHcAZQBlAG4ASABlAGEAZABlAHIAQQBuAGQAQQByAHIAYQB5ACkALAAgADEALAAgAEMAbwBsAHUAbQBuAHMAQgBlAHQAdwBlAGUAbgBIAGUAYQBkAGUAcgBBAG4AZABBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAAgACAAIAAgACkALAAgAFwAIgBcACIAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABvAG8AawB1AHAAVgBhAGwAdQBlACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABWAGEAbAB1AGUASQBuAFQAYQBiAGwAZQBOAHUAbQBiAGUAcgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABJAEYAKABJAFMATgBVAE0AQgBFAFIAKABcAG4AIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABcACIAXAAiACkAXABuACAAIAAgACAAKQAsACAAWABMAE8ATwBLAFUAUAAoAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQAsACAAMAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUAVAB3AG8AQwBvAGwAdQBtAG4AcwBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAxACwAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAyACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAFsAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAXQAsAFwAbgAgACAAIAAgAFgATABPAE8ASwBVAFAAKAAxACwAIAAoAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxAD0ATABvAG8AawB1AHAAVgBhAGwAdQBlADEAKQAqACgATABvAG8AawB1AHAAQQByAHIAYQB5ADIAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgApACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALAAgAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQAsACAAXAAiAFwAIgAsACAAVgBhAGwAdQBlAEkARgBGAGEAbABzAGUAKQApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMQAsACAATABvAG8AawB1AHAAVgBhAGwAdQBlADIALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAIABMAG8AbwBrAHUAcABBAHIAcgBhAHkAMgAsACAAUgBlAHQAdQByAG4AQQByAHIAYQB5ACwAIABbAFYAYQBsAHUAZQBJAGYARgBhAGwAcwBlAF0ALABcAG4AIAAgACAAIABJAEYARQBSAFIATwBSACgAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgATABvAG8AawB1AHAAVgBhAGwAdQBlADEALAAgAEwAbwBvAGsAdQBwAEEAcgByAGEAeQAxACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFgATABPAE8ASwBVAFAAKABMAG8AbwBrAHUAcABWAGEAbAB1AGUAMgAsACAATABvAG8AawB1AHAAQQByAHIAYQB5ADIALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApACwAIABcACIAXAAiACwAIABWAGEAbAB1AGUASQBmAEYAYQBsAHMAZQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAHAAbABpAHQAUwB0AHIAaQBuAGcASQBuAHQAbwBBAHIAcgBhAHkAXABuAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABDAGUAbABsACwAIABEAGUAbABpAG0AaQB0AGUAcgAsACAAWwBDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQBdACwAIABbAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyAF0ALABcAG4AIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSAFgATQBMACgAXABuACAAIAAgACAAIAAgACAAIABcACIAXAB1ADAAMAAzAGMAdABcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgAgAFwAdQAwADAAMgA2AFwAbgAgACAAIAAgACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABTAFUAQgBTAFQASQBUAFUAVABFACgAUwBVAEIAUwBUAEkAVABVAFQARQAoAEMAZQBsAGwALABDAGgAYQByAGEAYwB0AGUAcgBUAG8AUgBlAG0AbwB2AGUAMQAsAFwAIgBcACIAKQAsAEMAaABhAHIAYQBjAHQAZQByAFQAbwBSAGUAbQBvAHYAZQAyACwAXAAiAFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEQAZQBsAGkAbQBpAHQAZQByACwAXAAiAFwAdQAwADAAMwBjAC8AcwBcAHUAMAAwADMAZQBcAHUAMAAwADMAYwBzAFwAdQAwADAAMwBlAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgACkAIABcAHUAMAAwADIANgBcAG4AIAAgACAAIAAgACAAIAAgAFwAIgBcAHUAMAAwADMAYwAvAHMAXAB1ADAAMAAzAGUAXAB1ADAAMAAzAGMALwB0AFwAdQAwADAAMwBlAFwAIgAsAFwAbgAgACAAIAAgACAAIAAgACAAXAAiAC8ALwBzAFwAIgBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARwBlAHQAQwBsAGkAbQBhAHQAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAYQB2AGcAVABlAG0AcAAsAGEAdgBnAFIAYQBpAG4ALABmAHIAbwBzAHQARABhAHkAcwAsAGUAbABlAHYALABtAGEAcABfAHAAZQB0ACwAXABuACAAIAAgACAAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkALABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkALABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACwAXABuACAAIAAgACAAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQAsAG0AYQB4AEYAcgBvAHMAdABBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABtAGEAeABFAGwAZQB2AGEAdABpAG8AbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABtAGkAbgBQAEUAVABBAHIAcgBhAHkALABtAGEAeABQAEUAVABBAHIAcgBhAHkALABcAG4AIAAgACAAIABjAGwAaQBtAGEAdABlAFoAbwBuAGUAQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4AVABlAG0AcABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFQAZQBtAHAAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABUAGUAbQBwAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AYQB2AGcAVABlAG0AcAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFIAYQBpAG4AZgBhAGwAbABBAHIAcgBhAHkAKQBcAHUAMAAwADMAYwA9AGEAdgBnAFIAYQBpAG4AKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABSAGEAaQBuAGYAYQBsAGwAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBhAHYAZwBSAGEAaQBuACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgAbQBpAG4ARgByAG8AcwB0AEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZgByAG8AcwB0AEQAYQB5AHMAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABtAGEAeABGAHIAbwBzAHQAQQByAHIAYQB5ACkAXAB1ADAAMAAzAGUAPQBmAHIAbwBzAHQARABhAHkAcwApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AEUAbABlAHYAYQB0AGkAbwBuAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AZQBsAGUAdgApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AaQBuAFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBjAD0AbQBhAHAAXwBwAGUAdAApACoAXABuACAAIAAgACAAIAAgACAAIAAoAFYAQQBMAFUARQAoAG0AYQB4AFAARQBUAEEAcgByAGEAeQApAFwAdQAwADAAMwBlAD0AbQBhAHAAXwBwAGUAdAApACwAXABuACAAIAAgACAAIAAgACAAIABUAEEASwBFACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEYASQBMAFQARQBSACgAYwBsAGkAbQBhAHQAZQBaAG8AbgBlAEEAcgByAGEAeQAsAG0AYQBzAGsALAAgAFwAIgBOAG8AIABtAGEAdABjAGgAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAMQBcAG4AIAAgACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAEkAdABlAG0ARgByAG8AbQBNAGkAbgBNAGEAeABcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQAsACAATQBpAG4AQQByAHIAYQB5ACwAIABNAGEAeABBAHIAcgBhAHkALAAgAEkAdABlAG0AQQByAHIAYQB5ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAG0AYQBzAGsALABcAG4AIAAgACAAIAAgACAAIAAgACgAVgBBAEwAVQBFACgATQBpAG4AQQByAHIAYQB5ACkAXAB1ADAAMAAzAGMAPQBMAG8AbwBrAHUAcABWAGEAbAB1AGUAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAKABWAEEATABVAEUAKABNAGEAeABBAHIAcgBhAHkAKQBcAHUAMAAwADMAZQA9AEwAbwBvAGsAdQBwAFYAYQBsAHUAZQApACwAXABuACAAIAAgACAAIAAgACAAIABGAEkATABUAEUAUgAoAEkAdABlAG0AQQByAHIAYQB5ACwAIABtAGEAcwBrACwAIABcACIATgBvACAAbQBhAHQAYwBoAFwAIgApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIABDAHIAaQB0AGUAcgBpAGEAMQAsACAAQwByAGkAdABlAHIAaQBhADEAVAB5AHAAZQBBAHIAcgBhAHkALAAgAFEAdQBhAG4AdABpAHQAeQAsACAAWwBNAHUAbAB0AGkAcABsAGkAZQByAF0ALAAgAFsAQwByAGkAdABlAHIAaQBhADIAXQAsAFsAQwByAGkAdABlAHIAaQBhADIAQQByAHIAYQB5AF0ALABcAG4AIAAgAEwARQBUACgAXABuACAAIAAgACAAbQB1AGwAdABpAHAAbABpAGUAcgAsACAASQBGACgASQBTAE8ATQBJAFQAVABFAEQAKABNAHUAbAB0AGkAcABsAGkAZQByACkALAAxACwATQB1AGwAdABpAHAAbABpAGUAcgApACwAXABuACAAIAAgACAAcQB1AGEAbgB0AGkAdAB5ACwAIABRAHUAYQBuAHQAaQB0AHkAKgBNAHUAbAB0AGkAcABsAGkAZQByACwAXABuACAAIAAgACAAYwByAGkAdABlAHIAaQBhADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMQBUAHkAcABlAEEAcgByAGEAeQA9AEMAcgBpAHQAZQByAGkAYQAxACkALABcAG4AIAAgACAAIABjAHIAaQB0AGUAcgBpAGEAMgAsAEkARgAoAEkAUwBPAE0ASQBUAFQARQBEACgAQwByAGkAdABlAHIAaQBhADIAKQAsADEALAAtAC0AKABDAHIAaQB0AGUAcgBpAGEAMgBBAHIAcgBhAHkAPQBDAHIAaQB0AGUAcgBpAGEAMgApACkALABcAG4AIAAgACAAIABTAFUATQBQAFIATwBEAFUAQwBUACgAYwByAGkAdABlAHIAaQBhADEAKgBjAHIAaQB0AGUAcgBpAGEAMgAqAHEAdQBhAG4AdABpAHQAeQApAFwAbgAgACAAKQBcAG4AKQA7AFwAbgBcAG4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALABcAG4AIAAgACAAIAAgACAAIAAgAEEALABTAC0AMwA2ADUALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYQAsAFkARQBBAFIAKABBACkALABcAG4AIAAgACAAIAAgACAAIAAgAHkAYgAsAFkARQBBAFIAKABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAGYAaQByAHMAdABZAGUAYQByACwAeQBhACsAKABQAGUAcgBpAG8AZABFAG4AZAAoAEQAQQBUAEUAKAB5AGEALABtACwAZAApACkAXAB1ADAAMAAzAGMAIABTACkALABcAG4AIAAgACAAIAAgACAAIAAgAGwAYQBzAHQAWQBlAGEAcgAsAHkAYgAtACgARABBAFQARQAoAHkAYgAsAG0ALABkACkAXAB1ADAAMAAzAGUAIABFACkALABcAG4AIAAgACAAIAAgACAAIAAgAE0AQQBYACgAMAAsAGwAYQBzAHQAWQBlAGEAcgAtAGYAaQByAHMAdABZAGUAYQByACsAMQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAGcAZQB0AE8AdgBlAHIAbABhAHAAcABpAG4AZwBSAGUAcABvAHIAdABpAG4AZwBQAGUAcgBpAG8AZABzAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAUAByAG8AZAB1AGMAdABpAG8AbgBDAHkAYwBsAGUARQBuAGQALABSAGUAcABvAHIAdABpAG4AZwBDAHkAYwBsAGUAUwB0AGEAcgB0ACwAXABuACAAIAAgACAATABFAFQAKABcAG4AIAAgACAAIAAgACAAIAAgAFMALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBTAHQAYQByAHQALABcAG4AIAAgACAAIAAgACAAIAAgAEUALABQAHIAbwBkAHUAYwB0AGkAbwBuAEMAeQBjAGwAZQBFAG4AZAAsAFwAbgAgACAAIAAgACAAIAAgACAAbQAsAE0ATwBOAFQASAAoAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAZAAsAEQAQQBZACgAUgBlAHAAbwByAHQAaQBuAGcAQwB5AGMAbABlAFMAdABhAHIAdAApACwAIAAvACoAaABlAGwAcABlAHIAOgAgAGUAbgBkACAAZABhAHQAZQAgAGYAbwByACAAYQAgAHIAZQBwAG8AcgB0AGkAbgBnACAAcABlAHIAaQBvAGQAIABzAHQAYQByAHQAaQBuAGcAIABhAHQAIABhACAAZwBpAHYAZQBuACAAZABhAHQAZQAqAC8AXABuACAAIAAgACAAIAAgACAAIABQAGUAcgBpAG8AZABFAG4AZAAsAEwAQQBNAEIARABBACgAcwB0ACwARQBEAEEAVABFACgAcwB0ACwAMQAyACkALQAxACkALAAgAC8AKgBvAG4AbAB5ACAAbgBlAGUAZAAgAHQAbwAgAGwAbwBvAGsAIABiAGEAYwBrACAAMwA2ADUAIABkAGEAeQBzACgAbQBhAHgAIABvAHYAZQByAGwAYQBwACAAdwBpAG4AZABvAHcAKQAqAC8AXABuACAAIAAgACAAIAAgACAAIABBACwAUwAtADMANgA1ACwAXABuACAAIAAgACAAIAAgACAAIAB5AGEALABZAEUAQQBSACgAQQApACwAXABuACAAIAAgACAAIAAgACAAIAB5AGIALABZAEUAQQBSACgARQApACwAIAAvACoAaQBmACAAdABoAGUAIABhAG4AYwBoAG8AcgAgAGYAbwByACAAeQBhACAAZQBuAGQAcwAgAGIAZQBmAG8AcgBlACAAUwAsAGkAdAAgAGMAYQBuAFwAdQAwADAAMgA3AHQAIABvAHYAZQByAGwAYQBwADsAIABtAG8AdgBlACAAdABvACAAbgBlAHgAdAAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAZgBpAHIAcwB0AFkAZQBhAHIALAB5AGEAKwAoAFAAZQByAGkAbwBkAEUAbgBkACgARABBAFQARQAoAHkAYQAsAG0ALABkACkAKQBcAHUAMAAwADMAYwBTACkALAAgAC8AKgBpAGYAIAB0AGgAZQAgAGEAbgBjAGgAbwByACAAZgBvAHIAIAB5AGIAIABzAHQAYQByAHQAcwAgAGEAZgB0AGUAcgAgAEUALABpAHQAIABjAGEAbgBcAHUAMAAwADIANwB0ACAAbwB2AGUAcgBsAGEAcAA7ACAAbQBvAHYAZQAgAHQAbwAgAHAAcgBlAHYAaQBvAHUAcwAgAHkAZQBhAHIAKgAvAFwAbgAgACAAIAAgACAAIAAgACAAbABhAHMAdABZAGUAYQByACwAeQBiAC0AKABEAEEAVABFACgAeQBiACwAbQAsAGQAKQBcAHUAMAAwADMAZQBFACkALABcAG4AIAAgACAAIAAgACAAIAAgAG4ALABNAEEAWAAoADAALABsAGEAcwB0AFkAZQBhAHIALQBmAGkAcgBzAHQAWQBlAGEAcgArADEAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAeQByAHMALABTAEUAUQBVAEUATgBDAEUAKABuACwAMQAsAGYAaQByAHMAdABZAGUAYQByACwAMQApACwAXABuACAAIAAgACAAIAAgACAAIABzAHQAYQByAHQAcwAsAEQAQQBUAEUAKAB5AHIAcwAsAG0ALABkACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMALABNAEEAUAAoAHMAdABhAHIAdABzACwAUABlAHIAaQBvAGQARQBuAGQAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAdABhAGcALABJAEYAKABzAHQAYQByAHQAcwA9AFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBTAHQAYQByAHQALABcACIAIAAoAFQAaABpAHMAIAByAGUAcABvAHIAdABpAG4AZwAgAGMAeQBjAGwAZQApAFwAIgAsAFwAIgBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAcwB0AGEAcgB0AHMAVABlAHgAdAAsAFQARQBYAFQAKABzAHQAYQByAHQAcwAsAFwAIgBkAGQAIABtAG0AbQAgAHkAeQB5AHkAXAAiACkALABcAG4AIAAgACAAIAAgACAAIAAgAGUAbgBkAHMAVABlAHgAdAAsAFQARQBYAFQAKABlAG4AZABzACwAXAAiAGQAZAAgAG0AbQBtACAAeQB5AHkAeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgAbgA9ADAALABcACIAXAAiACwASABTAFQAQQBDAEsAKABzAHQAYQByAHQAcwBUAGUAeAB0ACAAXAB1ADAAMAAyADYAIABcACIAIAB0AG8AIABcACIAIABcAHUAMAAwADIANgAgAGUAbgBkAHMAVABlAHgAdAAgAFwAdQAwADAAMgA2ACAAdABhAGcAKQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEYAdQBuAGMAdABpAG8AbgBOAGEAbQBlAFwAbgA9AEwAQQBNAEIARABBACgARgB1AG4AYwB0AGkAbwBuACwAIABUAEUAWABUAEIARQBGAE8AUgBFACgARgBPAFIATQBVAEwAQQBUAEUAWABUACgARgB1AG4AYwB0AGkAbwBuACkALAAgAFwAIgAoAFwAIgApACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZAAsACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEEAcgByAGEAeQAsACAASQByAHIAaQBnAGEAdABpAG8AbgBNAGUAdABoAG8AZABBAHIAcgBhAHkALAAgAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQAsAFIAZQB0AHUAcgBuAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkACwAIABJAEYAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAD0AXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABcACIATgBvAHQAIABpAHIAcgBpAGcAYQB0AGUAZABcACIALAAgAFwAIgBBAG4AeQBcACIAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUALAAgAEkARgAoAEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAIAA9ACAAXAAiAE4AbwB0ACAAaQByAHIAaQBnAGEAdABlAGQAXAAiACwAIABSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQAsACAAXAAiAEEAbgB5AFwAIgApACwAXABuACAAIAAgACAAIAAgACAAIABYAEwATwBPAEsAVQBQACgAMQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgACgAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBBAHIAcgBhAHkAPQBQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACkAKgBcAG4AIAAgACAAIAAgACAAIAAgACAAIAAgACAAKABJAHIAcgBpAGcAYQB0AGkAbwBuAE0AZQB0AGgAbwBkAEEAcgByAGEAeQA9AEkAcgByAGkAZwBhAHQAaQBvAG4ATQBlAHQAaABvAGQAKQAqAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIAAoAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAEEAcgByAGEAeQA9AFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlACkALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkAKQBcAG4AIAAgACAAIAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBDAHIAbwBwAHAAaQBuAGcAXwBHAGUAdABGAHIAYQBjAFcARQBUAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUALABcAG4AIAAgACAAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtACwAXABuACAAIAAgACAATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABcAG4AIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwACwAXABuACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ARgByAGEAYwBXAEUAVABMAG8AbwBrAHUAcAAsAFwAbgAgACAAIAAgAEwARQBUACgAXABuACAAIAAgACAAIAAgACAAIABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlACwATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUATABvAG8AawB1AHAALABMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACgAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAFAAcgBvAGQAdQBjAHQAaQBvAG4AUwB5AHMAdABlAG0ALABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEwAbwBvAGsAdQBwACwAUAByAG8AZAB1AGMAdABpAG8AbgBTAHkAcwB0AGUAbQBGAHIAYQBjAFcARQBUAEwAbwBvAGsAdQBwAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAASQBGACgATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUARgByAGEAYwBXAEUAVAAgACsAIABQAHIAbwBkAHUAYwB0AGkAbwBuAFMAeQBzAHQAZQBtAEYAcgBhAGMAVwBFAFQAXAB1ADAAMAAzAGUAMAAsACAAMQAsACAAMAApAFwAbgAgACAAIAAgACkAKQA7AFwAbgBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAXABuACAAIAAgACAAUwB0AGEAdABlAEMAbwBtAG0AbwBuAE4AYQBtAGUAQQByAHIAYQB5ACwAIABTAHQAYQB0AGUAQQBiAGIAcgBlAHYAaQBhAHQAaQBvAG4AQQByAHIAYQB5ACwAXABuACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlACwAIABTAHQAYQB0AGUAQwBvAG0AbQBvAG4ATgBhAG0AZQBBAHIAcgBhAHkALAAgAFMAdABhAHQAZQBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgBBAHIAcgBhAHkALAAgAFwAIgBcACIAKQBcAG4AKQA7AFwAbgBcAG4AVQB0AGkAbABpAHQAeQBfAFMAbwB1AHIAYwBlAEgAeQBwAGUAcgBsAGkAbgBrAFwAbgA9AEwAQQBNAEIARABBACgAVABhAHIAZwBlAHQAQwBlAGwAbAAsAFwAbgAgACAATABFAFQAKABcAG4AIAAgACAAIABzAGgALAAgAFQARQBYAFQAQQBGAFQARQBSACgAQwBFAEwATAAoAFwAIgBmAGkAbABlAG4AYQBtAGUAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALAAgAFwAIgBdAFwAIgApACwAXABuACAAIAAgACAAYQBkAGQAcgAsACAAQwBFAEwATAAoAFwAIgBhAGQAZAByAGUAcwBzAFwAIgAsACAAVABhAHIAZwBlAHQAQwBlAGwAbAApACwAXABuACAAIAAgACAAXAAiACMAXAB1ADAAMAAyADcAXAAiACAAXAB1ADAAMAAyADYAIABzAGgAIABcAHUAMAAwADIANgAgAFwAIgBcAHUAMAAwADIANwAhAFwAIgAgAFwAdQAwADAAMgA2ACAAYQBkAGQAcgBcAG4AIAAgACkAXABuACkAOwBcAG4AXABuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawBEAGkAZgBmAGUAcgBlAG4AdABTAGgAZQBlAHQAXABuAD0ATABBAE0AQgBEAEEAKABUAGEAcgBnAGUAdABDAGUAbABsACwAXABuACAAIABMAEUAVAAoAFwAbgAgACAAIAAgAHMAaAAsACAAVABFAFgAVABBAEYAVABFAFIAKABDAEUATABMACgAXAAiAGYAaQBsAGUAbgBhAG0AZQBcACIALAAgAFQAYQByAGcAZQB0AEMAZQBsAGwAKQAsACAAXAAiAF0AXAAiACkALABcAG4AIAAgACAAIABhAGQAZAByACwAIABDAEUATABMACgAXAAiAGEAZABkAHIAZQBzAHMAXAAiACwAIABUAGEAcgBnAGUAdABDAGUAbABsACkALABcAG4AIAAgACAAIABcACIAIwBcACIAIABcAHUAMAAwADIANgAgAGEAZABkAHIAXABuACAAIAApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADEAXwAyAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMQAsACAAMgApAFwAbgApADsAXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0AFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAQQByAGcAdQBtAGUAbgB0AHMAQQByAHIAYQB5ACwAXABuACAAIAAgACAAQwBIAE8ATwBTAEUAQwBPAEwAUwAoAEEAcgBnAHUAbQBlAG4AdABzAEEAcgByAGEAeQAsACAAMwAsACAANAApAFwAbgApADsAXABuAFwAbgBDAG8AbQBtAG8AbgBfAEcAZQB0AE0AQwBGAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAFwAbgA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlACwAIABNAE0AUwAsACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsACAATQBNAFMAQQByAHIAYQB5ACwAIABSAGUAdAB1AHIAbgBBAHIAcgBhAHkALABcAG4AIAAgACAAIABYAEwATwBPAEsAVQBQACgAXABuACAAIAAgACAAIAAgACAAIABNAEUARABJAEEATgAoAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABUAGUAbQBwAGUAcgBhAHQAdQByAGUALAAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgACAAIABNAEkATgAoAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBBAHIAcgBhAHkAKQAsACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAIAAgAE0AQQBYACgAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACAAIAAgACAAKQAsAFwAbgAgACAAIAAgACAAIAAgACAAVABlAG0AcABlAHIAYQB0AHUAcgBlAEEAcgByAGEAeQAsAFwAbgAgACAAIAAgACAAIAAgACAAWABMAE8ATwBLAFUAUAAoAE0ATQBTACwAIABNAE0AUwBBAHIAcgBhAHkALAAgAFIAZQB0AHUAcgBuAEEAcgByAGEAeQApAFwAbgAgACAAIAAgACkAXABuACkAOwBcAG4AXABuAFwAbgBVAHQAaQBsAGkAdAB5AF8AUgBlAHMAdQBsAHQAcwBJAHQAZQBtAEYAcgBvAG0ARQBxAHUAYQB0AGkAbwBuAFQAaQB0AGwAZQBBAG4AZABTAG8AdQByAGMAZQBcAG4APQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAFQAaQB0AGwAZQBDAGUAbABsACwAIABTAG8AdQByAGMAZQBDAGUAbABsACwAXABuACAAIAAgACAAUwBVAEIAUwBUAEkAVABVAFQARQAoAEwARQBGAFQAKABTAG8AdQByAGMAZQBDAGUAbABsACwAIABGAEkATgBEACgAXAAiACwAXAAiACwAIABTAG8AdQByAGMAZQBDAGUAbABsACkAIAAtADEAKQAsACAAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFwAIgAsACAAXAAiAFwAIgApACAAXAB1ADAAMAAyADYAIABcACIAIABcACIAIABcAHUAMAAwADIANgAgAFQAaQB0AGwAZQBDAGUAbABsAFwAbgApADsAIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAiACwAIgB0AGUAeAB0ACIAOgAiAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXABuAEYAcgBhAGMAdABpAG8AbgAgAG8AZgAgAHYAbwBsAGEAdABpAGwAZQAgAHMAbwBsAGkAZABzACAAbABvAHMAdAAgAGkAbgAgAHQAaABlACAAcAByAGkAbQBhAHIAeQAgAE0ATQBTAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAbABvAHQAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAAdgBvAGwAYQB0AGkAbABlACAAcwBvAGwAaQBkAHMAIABsAG8AcwB0ACAAZAB1AHIAaQBuAGcAIABzAHQAbwByAGEAZwBlACAAaQBuACAAdABoAGUAIABwAHIAaQBtAGEAcgB5ACAAcwB5AHMAdABlAG0AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYAUwBMAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADUAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAFwAbgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAbwAgAGUAYQBjAGgAIAB0AGUAcgB0AGkAYQByAHkAIABzAHkAcwB0AGUAbQAgAGEAcwBzAHUAbQBlAGQAIAB0AGgAYQB0ACAAMgAgAHAAZQByACAAYwBlAG4AdAAgAGkAcwAgAHIAdQBuACAALQAgAG8AZgBmACAAZgByAG8AbQAgAHQAaABlACAAZgBlAGUAZAAgAHAAYQBkAC4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAHIAYQBjAHQAaQBvAG4AIABvAGYAIAB2AG8AbABhAHQAaQBsAGUAIABzAG8AbABpAGQAcwAgAHQAbwAgAGUAYQBjAGgAIAB0AGUAcgB0AGkAYQByAHkAIABzAHkAcwB0AGUAbQAgAGEAcwBzAHUAbQBlAGQAIAB0AGgAYQB0ACAAMgAgAHAAZQByACAAYwBlAG4AdAAgAGkAcwAgAHIAdQBuACAALQAgAG8AZgBmACAAZgByAG8AbQAgAHQAaABlACAAZgBlAGUAZAAgAHAAYQBkAC4AXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBNAFMAbQAxAFQAMwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARgByAGEAYwB0AGkAbwBuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAANAAuADEALgAyAC4AMwAgAEMATwBOAFMAVABBAE4AVABTAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAMAAuADAAMgApADsAXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXABuAEEAcwBoACAAYwBvAG4AdABlAG4AdAAgAG8AZgAgAG0AYQBuAHUAcgBlAC4AXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AKgAvAFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAHMAaAAgAGMAbwBuAHQAZQBuAHQAIABvAGYAIABtAGEAbgB1AHIAZQAuAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBWAGEAcgBpAGEAYgBsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEEAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAcgBhAGMAdABpAG8AbgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAxADYAKQA7AFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAFwAbgBNAGUAdABoAGEAbgBlACAAZQBtAGkAcwBzAGkAbwBuAHMAIABwAG8AdABlAG4AdABpAGEAbAAuAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBlAHQAaABhAG4AZQAgAGUAbQBpAHMAcwBpAG8AbgBzACAAcABvAHQAZQBuAHQAaQBhAGwALgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAGIAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBCADAAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAG0AMwAgAEMASAA0ACAALwAgAGsAZwAgAFYAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgADQALgAxAC4AMgAuADMAIABDAE8ATgBTAFQAQQBOAFQAUwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoADAALgAxADkAKQA7AFwAbgBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADEATQBNAFMATwBwAHQAaQBvAG4AcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEALAAgADEALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBTAHQAYQBnAGUAMgBNAE0AUwBPAHAAdABpAG8AbgBzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANAAsACAAMQAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATgBvACAATQBNAFMAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFMAdABhAGcAZQAzAE0ATQBTAE8AcAB0AGkAbwBuAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAxACwAIAAxACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEwAaQB2AGUAcwB0AG8AYwBrAEMAbABhAHMAcwBlAHMAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAzACwAIAAxACwAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBFAHgAcABvAHIAdAAgAG0AaQBkACAAZgBlAGQAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQB4AHAAbwByAHQAIABsAG8AbgBnACAAZgBlAGQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXABuAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADEAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAARAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgACgAZABhAHkAcwApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAEQAdQByAGEAdABpAG8AbgAgAG8AZgAgAHMAdABhAHkAIAAoAGQAYQB5AHMAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4AMQA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAHUAcgBhAHQAaQBvAG4AIABvAGYAIABzAHQAYQB5ACAAKABkAGEAeQBzACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAyACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBGAGUAZQBkAGwAbwB0ACAAdAB5AHAAZQBcACIALAAgAFwAIgBMAGUAbgBnAHQAaAAgAG8AZgAgAFMAdABhAHkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgAxAC0AOAAwACAAZABhAHkAcwBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgA4ADEALQAyADAAMAAgAGQAYQB5AHMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBmAGUAZABcACIALAAgAFwAIgAyADAAMQArACAAZABhAHkAcwBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4AMgA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABBAG4AaQBtAGEAbAAgAGMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBuAGkAbQBhAGwAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAAQQBuAGkAbQBhAGwAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AUwBvAHUAcgBjAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFYARQBFAFIARwAgADIAMAAyADYAOgAgAFQAYQBiAGwAZQAgAEEALgAxAC4AMQAuADIAOgAgAEIAZQBlAGYAIABmAGUAZQBkAGwAbwB0ACAAYwBhAHQAdABsAGUAIAAtACAAQQBuAGkAbQBhAGwAIABjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAG8AdgBlAGQAIABmAGUAZQBkAGwAbwB0ACAAdAB5AHAAZQBzACAAdABvACAAYQAgAHMAZQBwAGEAcgBhAHQAZQAgAGMAbwBsAHUAbQBuACAAdABvACAAYQBpAGQAIABsAG8AbwBrAHUAcAAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAGEAbQBlAGQAIABcAHUAMAAwADIANwBjAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAC0AIABvAHIAaQBnAGkAbgBhAGwAIABoAGEAcwAgAGgAZQBhAGQAZQByACAAXAB1ADAAMAAyADcAVQBuAGkAdABcAHUAMAAwADIANwAgAHcAaABpAGMAaAAgAGMAbwB2AGUAcgBzACAAdAB3AG8AIABjAG8AbAB1AG0AbgBzACkAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMAAsACAANwAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAXAAiACwAIABcACIAQwBoAGEAcgBhAGMAdABlAHIAaQBzAHQAaQBjAFwAIgAsACAAXAAiAFUAbgBpAHQAXAAiACwAIABcACIAMgAwADAANQAtADIAMAAwADkAXAAiACwAIABcACIAMgAwADEAMAAtADIAMAAxADQAXAAiACwAIABcACIAMgAwADEANQAtADIAMAAxADkAXAAiACwAIABcACIAMgAwADIAMAAtADIAMAAyADMAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBEAGEAeQBzACAAbwBuACAAZgBlAGUAZABcACIALAAgAFwAIgBkAGEAeQBzAFwAIgAsACAANwAwACwAIAA3ADAALAAgADcAMAAsACAANwA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBGAGUAZQBkACAAaQBuAHQAYQBrAGUAXAAiACwAIABcACIAawBnACAARABNAC8AZABhAHkAXAAiACwAIAAxADAALgAwACwAIAAxADAALgAwACwAIAAxADAALgA0ACwAIAAxADAALgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBOACAAcgBlAHQAZQBuAHQAaQBvAG4AXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0ACAAbwBmACAAaQBuAHQAYQBrAGUAXAAiACwAIAAyADEALgAxACwAIAAyADAALgA0ACwAIAAyADAALgA0ACwAIAAyADAALgA0ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIARABhAHkAcwAgAG8AbgAgAGYAZQBlAGQAXAAiACwAIABcACIAZABhAHkAcwBcACIALAAgADEAMQA1ACwAIAAxADEANQAsACAAMQAyADAALAAgADEANQAwADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAE0AaQBkAC0AZgBlAGQAXAAiACwAIABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGQAYQB5AFwAIgAsACAAMQAxAC4AMgAsACAAMQAwAC4AOAAsACAAMQAwAC4AOAAsACAAMQAwAC4AOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAE4AIAByAGUAdABlAG4AdABpAG8AbgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAIABvAGYAIABpAG4AdABhAGsAZQBcACIALAAgADEAMgAuADUALAAgADEAMgAuADcALAAgADEAMgAuADcALAAgADEAMgAuADcAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAGYAZQBkAFwAIgAsACAAXAAiAEQAYQB5AHMAIABvAG4AIABmAGUAZQBkAFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIAAyADUAMAAsACAAMgA1ADAALAAgADIANQAwACwAIAAyADUAMAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0AZgBlAGQAXAAiACwAIABcACIARgBlAGUAZAAgAGkAbgB0AGEAawBlAFwAIgAsACAAXAAiAGsAZwAgAEQATQAvAGQAYQB5AFwAIgAsACAAOQAuADAALAAgADgALgA1ACwAIAA4AC4AMgAsACAAOAAuADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATABvAG4AZwAtAGYAZQBkAFwAIgAsACAAXAAiAE4AIAByAGUAdABlAG4AdABpAG8AbgBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAIABvAGYAIABpAG4AdABhAGsAZQBcACIALAAgADYALgA2ACwAIAA3AC4AMAAsACAANwAuADAALAAgADcALgAwAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4AMwA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAGkAZQB0ACAAcAByAG8AcABlAHIAdABpAGUAcwBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAFQAaQB0AGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAGkAZQB0ACAAcAByAG8AcABlAHIAdABpAGUAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4AMwA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABEAGkAZQB0ACAAcAByAG8AcABlAHIAdABpAGUAcwBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADEALAAgAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAIABcAG4AIAAgACAAIAAgACAAIAAgAEkATgBEAEUAWAAoAHsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFYAQQBSAEkAQQBUAEkATwBOACAATwBOACAAUwBPAFUAUgBDAEUAOgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcAQwBvAG4AdgBlAHIAdABlAGQAIAB0AG8AIABmAHIAYQBjAHQAaQBvAG4AIABjAG8AbAB1AG0AbgAgAGEAbgBkACAAYwBvAG4AdgBlAHIAdABlAGQAIABOAEQARgAgAGEAbgBkACAARQB0AGgAZQByACAAZQB4AHQAcgBhAGMAdAAgAHYAYQBsAHUAZQBzACAAdABvACAAZgByAGEAYwB0AGkAbwBuAHMALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBvAHYAZQBkACAAZgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAcwAgAHQAbwAgAGEAIABzAGUAcABhAHIAYQB0AGUAIABjAG8AbAB1AG0AbgAgAHQAbwAgAGEAaQBkACAAbABvAG8AawB1AHAALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8ARABhAHQAYQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADEAMwAsACAAOAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARgBlAGUAZABsAG8AdAAgAHQAeQBwAGUAXAAiACwAIABcACIATgB1AHQAcgBpAGUAbgB0ACAAYQBuAGEAbAB5AHMAaQBzAFwAIgAsACAAXAAiAFUAbgBpAHQAXAAiACwAIABcACIAMgAwADAANQAtADIAMAAwADkAXAAiACwAIABcACIAMgAwADEAMAAtADIAMAAxADQAXAAiACwAIABcACIAMgAwADEANQAtADIAMAAxADkAXAAiACwAIABcACIAMgAwADIAMAAtADIAMAAyADMAXAAiACwAIABcACIAQwBvAG4AdgBlAHIAdABlAGQAIAB0AG8AIABmAHIAYQBjAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBEAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAbwBtAGUAcwB0AGkAYwBcACIALAAgAFwAIgBDAHIAdQBkAGUAIABwAHIAbwB0AGUAaQBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgADAALgAxADQALAAgADAALgAxADQALAAgADAALgAxADQALAAgADAALgAxADQALAAgADAALgAxADQAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjAFwAIgAsACAAXAAiAE4ARABGAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADIAMwAuADAALAAgADIAMgAuADAALAAgADIAMgAuADAALAAgADIAMgAuADAALAAgADAALgAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABvAG0AZQBzAHQAaQBjAFwAIgAsACAAXAAiAEUAdABoAGUAcgAgAEUAeAB0AHIAYQBjAHQAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAANAAuADUALAAgADQALgA1ACwAIAA0AC4AOAAsACAANAAuADgALAAgADAALgAwADQAOAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAEQAcgB5ACAAbQBhAHQAdABlAHIAIABkAGkAZwBlAHMAdABpAGIAaQBsAGkAdAB5AFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEALAAgADAALgA4ADEAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBDAHIAdQBkAGUAIABwAHIAbwB0AGUAaQBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgADAALgAxADMALAAgADAALgAxADIANQAsACAAMAAuADEAMgAsACAAMAAuADEAMgAsACAAMAAuADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAGkAZAAtAGYAZQBkAFwAIgAsACAAXAAiAE4ARABGAFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADIANAAuADAALAAgADIAMgAuADAALAAgADIAMgAuADAALAAgADIAMgAuADAALAAgADAALgAyADIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIATQBpAGQALQBmAGUAZABcACIALAAgAFwAIgBFAHQAaABlAHIAIABFAHgAdAByAGEAYwB0AFwAIgAsACAAXAAiAHAAZQByACAAYwBlAG4AdABcACIALAAgADUALgAwACwAIAA1AC4AMAAsACAANQAuADAALAAgADUALgAwACwAIAAwAC4AMAA1ADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBGAGUAZABcACIALAAgAFwAIgBEAHIAeQAgAG0AYQB0AHQAZQByACAAZABpAGcAZQBzAHQAaQBiAGkAbABpAHQAeQBcACIALAAgAFwAIgBmAHIAYQBjAHQAaQBvAG4AXAAiACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxACwAIAAwAC4AOAAxADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEwAbwBuAGcALQBGAGUAZABcACIALAAgAFwAIgBDAHIAdQBkAGUAIABwAHIAbwB0AGUAaQBuAFwAIgAsACAAXAAiAGYAcgBhAGMAdABpAG8AbgBcACIALAAgADAALgAxADMALAAgADAALgAxADIANQAsACAAMAAuADEAMgAsACAAMAAuADEAMgAsACAAMAAuADEAMgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0ARgBlAGQAXAAiACwAIABcACIATgBEAEYAXAAiACwAIABcACIAcABlAHIAIABjAGUAbgB0AFwAIgAsACAAMgA0AC4AMAAsACAAMgA0AC4AMAAsACAAMgA0AC4AMAAsACAAMgA0AC4AMAAsACAAMAAuADIANAA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBMAG8AbgBnAC0ARgBlAGQAXAAiACwAIABcACIARQB0AGgAZQByACAARQB4AHQAcgBhAGMAdABcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIAA1AC4AMAAsACAANQAuADAALAAgADUALgA1ACwAIAA1AC4ANQAsACAAMAAuADAANQA1AFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4ALwAqACAAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4ANAA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABNAEMARgBzACAAKABmAHIAYQBjAHQAaQBvAG4AKQAgACgATQBDAEYAaQBtAFQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVABpAHQAbABlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBGAGUAZQBkAGwAbwB0ACAALQAgAE0AQwBGAHMAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIABUAGEAYgBsAGUAIABBAC4AMQAuADEALgA0ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAE0AQwBGAHMAIAAoAGYAcgBhAGMAdABpAG8AbgApACAAKABNAEMARgBpAG0AVAApAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA0ACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEQAdQBwAGwAaQBjAGEAdABlAGQAIABOAFMAVwAgAHYAYQBsAHUAZQBzACAAZgBvAHIAIABBAEMAVABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAATgBUACAAYwBvAGwAdQBtAG4AIAB0AGgAYQB0ACAAZAB1AHAAbABpAGMAYQB0AGUAcwAgAFEATABEACAAdgBhAGwAdQBlAHMAIABhAHMAIABwAGUAcgAgAGEAZAB2AGkAYwBlACAAZgByAG8AbQAgAHMAbwB1AHIAYwBlACAAZABhAHQAYQAgAHAAcgBvAHYAaQBkAGUAcgAuAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABUAEEAUwAgAGMAbwBsAHUAbQBuACAAdABoAGEAdAAgAGQAdQBwAGwAaQBjAGEAdABlAHMAIABWAEkAQwAgAHYAYQBsAHUAZQBzACAAYQBzACAAcABlAHIAIABhAGQAdgBpAGMAZQAgAGYAcgBvAG0AIABzAG8AdQByAGMAZQAgAGQAYQB0AGEAIABwAHIAbwB2AGkAZABlAHIALgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAQQBkAGQAZQBkACAAXAB1ADAAMAAyADcATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAFwAdQAwADAAMgA3ACAAYwBvAGwAdQBtAG4AIAB3AGkAdABoACAATQBNAFMAIABuAGEAbQBlAHMAIAB0AGgAYQB0ACAAbQBhAHQAYwBoACAATgBJAFIAIABkAGUAZgBpAG4AaQB0AGkAbwBuAHMALgBcACIAXABuACAAIAAgACAAIAAgACAAIAB9ACwAIAByACwAIABjACkAXABuACAAIAAgACAAIAAgACkAXABuACAAIAAgACAAKQBcAG4AIAAgACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBDAEYAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAAMQAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAE4AUwBXAFwAIgAsACAAXAAiAEEAQwBUAFwAIgAsACAAXAAiAFEATABEAFwAIgAsACAAXAAiAE4AVABcACIALAAgAFwAIgBTAEEAXAAiACwAIABcACIAVgBJAEMAXAAiACwAIABcACIAVwBBAFwAIgAsACAAXAAiAFQAQQBTAFwAIgAsACAAXAAiAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAGkAbQBhAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGwAbwB0ACAAKABGAGUAZQBkAHAAYQBkACkAXAAiACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAzACwAIAAwAC4AMAAzACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIAAwAC4AMAAxACwAIABcACIARAByAHkAbABvAHQAIAAoAGYAZQBlAGQAIABwAGEAZAApAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAIAAoAFMAdABvAGMAawBwAGkAbABlACkAXAAiACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIAAwAC4AMAAyACwAIABcACIAUwBvAGwAaQBkACAAcwB0AG8AcgBhAGcAZQBcACIAOwAgAFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABQAGEAcwBzAGkAdgBlACAAVwBpAG4AZAByAG8AdwApAFwAIgAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAMAAuADAAMQAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAIABcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIARABpAHIAZQBjAHQAIABBAHAAcABsAGkAYwBhAHQAaQBvAG4AIAB0AG8AIABzAG8AaQBsAFwAIgAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAMAAsACAAXAAiAEQAaQByAGUAYwB0ACAAYQBwAHAAbABpAGMAYQB0AGkAbwBuAFwAIgA7ACAAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQByAHQAaQBhAHIAeQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIAAoAEUAZgBmAGwAdQBlAG4AdAAgAHAAbwBuAGQAKQBcACIALAAgADAALgA3ADUALAAgADAALgA3ADUALAAgADAALgA3ADcALAAgADAALgA3ADcALAAgADAALgA3ADUALAAgADAALgA3ADUALAAgADAALgA3ADcALAAgADAALgA3ADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AXABuAFwAbgAvACoAIABcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAFwAbgBUAGEAYgBsAGUAIABBAC4AMQAuADEALgA1ADoAIABCAGUAZQBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAALQAgAE4AaQB0AHIAbwB1AHMAIABvAHgAaQBkAGUAIABFAEYAcwAgACgARQBGAG0AVAApAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuACoALwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAbABvAHQAIAAtACAATgBpAHQAcgBvAHUAcwAgAG8AeABpAGQAZQAgAEUARgBzAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVQBuAGkAdABcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4ANQA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABOAGkAdAByAG8AdQBzACAAbwB4AGkAZABlACAARQBGAHMAIAAoAEUARgBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAFYAYQByAGkAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMgAsACAAMQAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVgBBAFIASQBBAFQASQBPAE4AIABPAE4AIABTAE8AVQBSAEMARQA6AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBBAGQAZABlAGQAIABcAHUAMAAwADIANwBOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AXAB1ADAAMAAyADcAIABjAG8AbAB1AG0AbgAgAHcAaQB0AGgAIABNAE0AUwAgAG4AYQBtAGUAcwAgAHQAaABhAHQAIABtAGEAdABjAGgAIABOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AcwAuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBOAGkAdAByAG8AdQBzAE8AeABpAGQAZQBFAEYAcwBfAEQAYQB0AGEAXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAA2ACwAIAA0ACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBUAHIAZQBhAHQAbQBlAG4AdAAgAHMAdABhAGcAZQAgAFQAXAAiACwAIABcACIATQBNAFMAIABtAFwAIgAsACAAXAAiAEUARgBtAFQAIAAoAGsAZwAgAE4AMgBPAC0ATgAvAGsAZwAgAE4AKQBcACIALAAgAFwAIgBOAEkAUgAgAGQAZQBmAGkAbgBpAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFAAcgBpAG0AYQByAHkAXAAiACwAIABcACIARAByAHkAIABsAG8AdAAgACgARgBlAGUAZABwAGEAZAApAFwAIgAsACAAMAAuADAAMAA1ADQALAAgAFwAIgBEAHIAeQBsAG8AdAAgACgAZgBlAGUAZAAgAHAAYQBkACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAFMAbwBsAGkAZAAgAFMAdABvAHIAYQBnAGUAIAAoAFMAdABvAGMAawBwAGkAbABlACkAXAAiACwAIAAwAC4AMAAwADUALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABQAGEAcwBzAGkAdgBlACAAVwBpAG4AZAByAG8AdwApAFwAIgAsACAAMAAuADAAMQAsACAAXAAiAEMAbwBtAHAAbwBzAHQAaQBuAGcAIAAoAHAAYQBzAHMAaQB2AGUAIAB3AGkAbgBkAHIAbwB3ACkAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFMAZQBjAG8AbgBkAGEAcgB5AFwAIgAsACAAXAAiAEQAaQByAGUAYwB0ACAAQQBwAHAAbABpAGMAYQB0AGkAbwBuACAAdABvACAAcwBvAGkAbABcACIALAAgADAALAAgAFwAIgBEAGkAcgBlAGMAdAAgAGEAcABwAGwAaQBjAGEAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVABlAHIAdABpAGEAcgB5AFwAIgAsACAAXAAiAFUAbgBjAG8AdgBlAHIAZQBkACAAYQBuAGEAZQByAG8AYgBpAGMAIABsAGEAZwBvAG8AbgAgACgARQBmAGYAbAB1AGUAbgB0ACAAUABvAG4AZAApAFwAIgAsACAAMAAsACAAXAAiAEEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBcAG4AXABuAC8AKgAgAFwAbgAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABcAG4AVABhAGIAbABlACAAQQAuADEALgAxAC4ANgA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAIAAoAEYAcgBhAGMARwBBAFMATQBtAFQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEYAZQBlAGQAbABvAHQAIAAtACAARgByAGEAYwB0AGkAbwBuACAAbwBmACAATgAgAHYAbwBsAGEAdABpAGwAaQBzAGUAZAAgAGIAeQAgAE0ATQBTACAAKABGAHIAYQBjAEcAQQBTAE0AbQBUACkAXAAiACkAOwBcAG4AXABuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFUAbgBpAHQAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFwAIgApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAVABhAGIAbABlACAAQQAuADEALgAxAC4ANgA6ACAAQgBlAGUAZgAgAGYAZQBlAGQAbABvAHQAIABjAGEAdAB0AGwAZQAgAC0AIABGAHIAYQBjAHQAaQBvAG4AIABvAGYAIABOACAAdgBvAGwAYQB0AGkAbABpAHMAZQBkACAAYgB5ACAATQBNAFMAIAAoAEYAcgBhAGMARwBBAFMATQBtAFQAKQBcACIAKQA7AFwAbgBcAG4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXABuACAAIAAgACAATQBBAEsARQBBAFIAUgBBAFkAKAAyACwAIAAxACwAIABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsACAAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBWAEEAUgBJAEEAVABJAE8ATgAgAE8ATgAgAFMATwBVAFIAQwBFADoAXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAEEAZABkAGUAZAAgAFwAdQAwADAAMgA3AE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcAHUAMAAwADIANwAgAGMAbwBsAHUAbQBuACAAdwBpAHQAaAAgAE0ATQBTACAAbgBhAG0AZQBzACAAdABoAGEAdAAgAG0AYQB0AGMAaAAgAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBzAC4AXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBEAGEAdABhAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgANgAsACAANAAsACAAXABuACAAIAAgACAAIAAgAEwAQQBNAEIARABBACgAcgAsAGMALAAgAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAVAByAGUAYQB0AG0AZQBuAHQAIABzAHQAYQBnAGUAIABUAFwAIgAsACAAXAAiAE0ATQBTACAAbQBcACIALAAgAFwAIgBGAHIAYQBjAEcAQQBTAE0AbQBUACAAKABrAGcAIABOAEgAMwAtAE4AIAArACAATgBPAHgALQBOACkALwBrAGcAIABOAFwAIgAsACAAXAAiAE4ASQBSACAAZABlAGYAaQBuAGkAdABpAG8AbgBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUAByAGkAbQBhAHIAeQBcACIALAAgAFwAIgBEAHIAeQAgAGwAbwB0ACAAKABGAGUAZQBkAHAAYQBkACkAXAAiACwAIAAwAC4ANgAsACAAXAAiAEQAcgB5AGwAbwB0ACAAKABmAGUAZQBkACAAcABhAGQAKQBcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIAUwBlAGMAbwBuAGQAYQByAHkAXAAiACwAIABcACIAUwBvAGwAaQBkACAAUwB0AG8AcgBhAGcAZQAgACgAUwB0AG8AYwBrAHAAaQBsAGUAKQBcACIALAAgADAALgAyADUALAAgAFwAIgBTAG8AbABpAGQAIABzAHQAbwByAGEAZwBlAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABQAGEAcwBzAGkAdgBlACAAVwBpAG4AZAByAG8AdwApAFwAIgAsACAAMAAuADQALAAgAFwAIgBDAG8AbQBwAG8AcwB0AGkAbgBnACAAKABwAGEAcwBzAGkAdgBlACAAdwBpAG4AZAByAG8AdwApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBTAGUAYwBvAG4AZABhAHIAeQBcACIALAAgAFwAIgBEAGkAcgBlAGMAdAAgAEEAcABwAGwAaQBjAGEAdABpAG8AbgAgAHQAbwAgAHMAbwBpAGwAXAAiACwAIAAwACwAIABcACIARABpAHIAZQBjAHQAIABhAHAAcABsAGkAYwBhAHQAaQBvAG4AXAAiADsAXABuACAAIAAgACAAIAAgACAAIAAgACAAXAAiAFQAZQByAHQAaQBhAHIAeQBcACIALAAgAFwAIgBVAG4AYwBvAHYAZQByAGUAZAAgAGEAbgBhAGUAcgBvAGIAaQBjACAAbABhAGcAbwBvAG4AIAAoAEUAZgBmAGwAdQBlAG4AdAAgAHAAbwBuAGQAKQBcACIALAAgADAALgAzADUALAAgAFwAIgBBAG4AYQBlAHIAbwBiAGkAYwAgAGwAYQBnAG8AbwBuAFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgBcAG4AIgB9ACwAewAiAHAAYQB0AGgAIgA6ACIALwBwAHIAbwBqAGUAYwB0AHMALwBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMAIgAsACIAdABlAHgAdAAiADoAIgAvACoAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuADMALgAxADoAIABFAG4AdABlAHIAaQBjACAATQBlAHQAaABhAG4AZQAgAC0AIABGAGUAZQBkAGwAbwB0ACAAQgBlAGUAZgBcAG4APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQBcAG4AMwAuADEALgAxAC4AMQAgAE0AZQB0AGgAbwBkACAAMQAgAC0AIABFAG4AdABlAHIAaQBjACAAQgBlAGUAZgAgAEYAZQBlAGQAbABvAHQAXABuAD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0APQA9AD0AXABuACoALwBcAG4AXABuAC8AKgBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgBUAG8AdABhAGwAIABhAG4AbgB1AGEAbAAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAZgByAG8AbQAgAGUAbgB0AGUAcgBpAGMAIABmAGUAcgBtAGUAbgB0AGEAdABpAG8AbgAgAGkAbgAgAGYAZQBlAGQAbABvAHQAIABiAGUAZQBmACAAYwBhAHQAdABsAGUAXABuAEUAXwBlAG4AdABlAHIAaQBjAFwAbgB0ACAAQwBIADQAXABuAEUAXwB7AGUAbgB0AGUAcgBpAGMAfQA9AFwAXABzAHUAbQBcAFwAbgBvAGwAaQBtAGkAdABzAF8AagAoAEQAXwBqAFwAXAB0AGkAbQBlAHMAIABNAF8AagBcAFwAdABpAG0AZQBzACAATgBfAGoAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ARABfAGoAIAA9ACAAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGwAbwB0ACAAKABkAGEAeQBzACkAXABuAE0AXwBqACAAPQAgAGQAYQBpAGwAeQAgAG0AZQB0AGgAYQBuAGUAIABwAHIAbwBkAHUAYwB0AGkAbwBuACAAKABrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQApAFwAbgBOAF8AagAgAD0AIABuAHUAbQBiAGUAcgBzACAAbwBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAbABvAHQAIAAoAGgAZQBhAGQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEQAXwBqACwAIABNAF8AagAsACAATgBfAGoALABcAG4AIAAgACAAIAAoAEQAXwBqACAAKgAgAE0AXwBqACAAKgAgAE4AXwBqACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAFQAbwB0AGEAbAAgAGEAbgBuAHUAYQBsACAAbQBlAHQAaABhAG4AZQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABmAHIAbwBtACAAZQBuAHQAZQByAGkAYwAgAGYAZQByAG0AZQBuAHQAYQB0AGkAbwBuACAAaQBuACAAZgBlAGUAZABsAG8AdAAgAGIAZQBlAGYAIABjAGEAdAB0AGwAZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIARQBfAGUAbgB0AGUAcgBpAGMAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgB0ACAAQwBIADQAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAVgBFAEUAUgBHACAAMgAwADIANgA6ACAAMwAuADEALgAxAC4AMQAsACAARQBxAHUAYQB0AGkAbwBuACAAKAAxACkAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBMAGEAdABlAHgARQBxAHUAYQB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBFAF8AewBlAG4AdABlAHIAaQBjAH0APQBcAFwAcwB1AG0AXABcAG4AbwBsAGkAbQBpAHQAcwBfAGoAKABEAF8AagBcAFwAdABpAG0AZQBzACAATQBfAGoAXABcAHQAaQBtAGUAcwAgAE4AXwBqACkAXABcAHQAaQBtAGUAcwAgADEAMABeAHsALQAzAH0AXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBBAHIAZwB1AG0AZQBuAHQAcwBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcAG4AIAAgACAAIABNAEEASwBFAEEAUgBSAEEAWQAoADMALAAgADQALABcAG4AIAAgACAAIAAgACAATABBAE0AQgBEAEEAKAByACwAYwAsAFwAbgAgACAAIAAgACAAIAAgACAASQBOAEQARQBYACgAewBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARABfAGoAXAAiACwAIABcACIAZAB1AHIAYQB0AGkAbwBuACAAbwBmACAAcwB0AGEAeQAgAG8AZgAgAGUAYQBjAGgAIABjAGEAdAB0AGwAZQAgAGwAbwB0AFwAIgAsACAAXAAiAGQAYQB5AHMAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBNAF8AagBcACIALAAgAFwAIgBkAGEAaQBsAHkAIABtAGUAdABoAGEAbgBlACAAcAByAG8AZAB1AGMAdABpAG8AbgBcACIALAAgAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIALAAgAFwAIgBDAGEAbABjAHUAbABhAHQAZQBkACAAZgByAG8AbQAgADMALgAxAC4AMQAuADEALAAgACgAMgApAFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAF8AagBcACIALAAgAFwAIgBuAHUAbQBiAGUAcgBzACAAbwBmACAAZgBlAGUAZABsAG8AdAAgAGMAYQB0AHQAbABlACAAaQBuACAAZQBhAGMAaAAgAGMAYQB0AHQAbABlACAAbABvAHQAXAAiACwAIABcACIAaABlAGEAZABcACIALAAgAFwAIgBJAG4AcAB1AHQAXAAiAFwAbgAgACAAIAAgACAAIAAgACAAfQAsACAAcgAsACAAYwApAFwAbgAgACAAIAAgACAAIAApAFwAbgAgACAAIAAgACkAXABuACAAIAApADsAXABuAFwAbgAvACoAXABuAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBcAG4ARABhAGkAbAB5ACAAcAByAG8AZAB1AGMAdABpAG8AbgAgAG8AZgAgAGUAbgB0AGUAcgBpAGMAIABtAGUAdABoAGEAbgBlAFwAbgBNAF8AagBcAG4AawBnACAAQwBIADQALwBoAGUAYQBkAC8AZABhAHkAXABuAE0AXwBqAD0AKAA1AC4AMQAxAFwAXAB0AGkAbQBlAHMAIABJAF8AagAtADQALgAwADAAXABcAHQAaQBtAGUAcwAgAEUARQBfAGoAKwAyAC4AMgA2AFwAXAB0AGkAbQBlAHMAIABOAEQARgBfAGoAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcAG4ASQBfAGoAIAA9ACAAZAByAHkAIABtAGEAdAB0AGUAcgAgAGkAbgB0AGEAawBlACAAKABrAGcAIABEAE0ALwBoAGUAYQBkAC8AZABhAHkAKQBcAG4ARQBFAF8AagAgAD0AIABlAHQAaABlAHIAIABlAHgAdAByAGEAYwB0ACAAYQBzACAAYQAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABvAGYAIABJAF8AagAgACgAcABlAHIAIABjAGUAbgB0ACkAXABuAE4ARABGAF8AagAgAD0AIABuAGUAdQB0AHIAYQBsACAAZABlAHQAZQByAGcAZQBuAHQAIABmAGkAYgByAGUAIABhAHMAIABhACAAcABlAHIAYwBlAG4AdABhAGcAZQAgAG8AZgAgAEkAXwBqACAAKABwAGUAcgAgAGMAZQBuAHQAKQBcAG4ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAC0ALQAtAFwAbgAqAC8AXABuAFwAbgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAEkAXwBqACwAIABFAEUAXwBqACwAIABOAEQARgBfAGoALABcAG4AIAAgACAAIAAoADUALgAxADEAIAAqACAASQBfAGoAIAAtACAANAAuADAAMAAgACoAIABFAEUAXwBqACAAKwAgADIALgAyADYAIAAqACAATgBEAEYAXwBqACkAIAAqACAAMQAwACAAXgAgAC0AMwBcAG4AIAAgACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBUAGkAdABsAGUAXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAEQAYQBpAGwAeQAgAHAAcgBvAGQAdQBjAHQAaQBvAG4AIABvAGYAIABlAG4AdABlAHIAaQBjACAAbQBlAHQAaABhAG4AZQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFYAYQByAGkAYQBiAGwAZQBcAG4AIAAgAD0ATABBAE0AQgBEAEEAKABcACIATQBfAGoAXAAiACkAOwBcAG4AXABuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0AFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBrAGcAIABDAEgANAAvAGgAZQBhAGQALwBkAGEAeQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFMAbwB1AHIAYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBWAEUARQBSAEcAIAAyADAAMgA2ADoAIAAzAC4AMQAuADEALgAxACwAIABFAHEAdQBhAHQAaQBvAG4AIAAoADIAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAIgBBAGwAbQBlAGkAZABhACAAZQB0ACAAYQBsAC4AIAAoADIAMAAyADUAKQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AXABuACAAIAA9AEwAQQBNAEIARABBACgAXAAiAE0AXwBqAD0AKAA1AC4AMQAxAFwAXAB0AGkAbQBlAHMAIABJAF8AagAtADQALgAwADAAXABcAHQAaQBtAGUAcwAgAEUARQBfAGoAKwAyAC4AMgA2AFwAXAB0AGkAbQBlAHMAIABOAEQARgBfAGoAKQBcAFwAdABpAG0AZQBzACAAMQAwAF4AewAtADMAfQBcACIAKQA7AFwAbgBcAG4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzAFwAbgAgACAAPQBMAEEATQBCAEQAQQAoAFwAbgAgACAAIAAgAE0AQQBLAEUAQQBSAFIAQQBZACgAMwAsACAANAAsAFwAbgAgACAAIAAgACAAIABMAEEATQBCAEQAQQAoAHIALABjACwAXABuACAAIAAgACAAIAAgACAAIABJAE4ARABFAFgAKAB7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBJAF8AagBcACIALAAgAFwAIgBkAHIAeQAgAG0AYQB0AHQAZQByACAAaQBuAHQAYQBrAGUAXAAiACwAIABcACIAawBnACAARABNAC8AaABlAGEAZAAvAGQAYQB5AFwAIgAsACAAXAAiAEkAbgBwAHUAdABcACIAOwBcAG4AIAAgACAAIAAgACAAIAAgACAAIABcACIARQBFAF8AagBcACIALAAgAFwAIgBlAHQAaABlAHIAIABlAHgAdAByAGEAYwB0ACAAYQBzACAAYQAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABvAGYAIABJAF8AagBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgA7AFwAbgAgACAAIAAgACAAIAAgACAAIAAgAFwAIgBOAEQARgBfAGoAXAAiACwAIABcACIAbgBlAHUAdAByAGEAbAAgAGQAZQB0AGUAcgBnAGUAbgB0ACAAZgBpAGIAcgBlACAAYQBzACAAYQAgAHAAZQByAGMAZQBuAHQAYQBnAGUAIABvAGYAIABJAF8AagBcACIALAAgAFwAIgBwAGUAcgAgAGMAZQBuAHQAXAAiACwAIABcACIASQBuAHAAdQB0AFwAIgBcAG4AIAAgACAAIAAgACAAIAAgAH0ALAAgAHIALAAgAGMAKQBcAG4AIAAgACAAIAAgACAAKQBcAG4AIAAgACAAIAApAFwAbgAgACAAKQA7AFwAbgAiAH0AXQAsACIAcAByAG8AagBlAGMAdABOAGEAbQBlAHMAIgA6AFsAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAZQBuAHMAaQB0AHkATwBmAE0AZQB0AGgAYQBuAGUAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGUAbgBzAGkAdAB5AE8AZgBNAGUAdABoAGEAbgBlAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AE4AMgBvAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBDAGcAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbwBuAHYAZQByAHQATgAyAG8ARQBsAGUAbQBlAG4AdABhAGwAVABvAE0AbwBsAGUAYwB1AGwAYQByAEMAZwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABOADIAbwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAQwBnAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBvAG4AdgBlAHIAdABHAGEAcwBFAGwAZQBtAGUAbgB0AGEAbABUAG8ATQBvAGwAZQBjAHUAbABhAHIAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAG8AbgB2AGUAcgB0AEcAYQBzAEUAbABlAG0AZQBuAHQAYQBsAFQAbwBNAG8AbABlAGMAdQBsAGEAcgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEcAVwBQAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARwBXAFAAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBBAHUAcwB0AHIAYQBsAGkAYQBuAFMAdABhAHQAZQBzAFQAZQByAHIAaQB0AG8AcgBpAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEEAdQBzAHQAcgBhAGwAaQBhAG4AUwB0AGEAdABlAHMAVABlAHIAcgBpAHQAbwByAGkAZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAEEAUwBBADQAQQByAGUAYQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBBAFMAQQA0AEEAcgBlAGEAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAQQBTAEEANABBAHIAZQBhAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFcAZQB0AEEAbgBkAEQAcgB5AFoAbwBuAGUAcwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVwBlAHQAQQBuAGQARAByAHkAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBXAGUAdABBAG4AZABEAHIAeQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBDAGwAaQBtAGEAdABlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AQwBsAGkAbQBhAHQAZQBaAG8AbgBlAHMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEMAbABpAG0AYQB0AGUAWgBvAG4AZQBzAF8AQQBwAHAAZQBuAGQAaQBjAGUAcwAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AVABlAG0AcABlAHIAYQB0AHUAcgBlAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFQAZQBtAHAAZQByAGEAdAB1AHIAZQBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8AUgBhAGkAbgBmAGEAbABsAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAFIAYQBpAG4AZgBhAGwAbABaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBSAGEAaQBuAGYAYQBsAGwAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABlAGEAYwBoAGkAbgBnAFoAbwBuAGUAcwBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAZQBhAGMAaABpAG4AZwBaAG8AbgBlAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGUAYQBjAGgAaQBuAGcAWgBvAG4AZQBzAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEQAYQB0AGEAUwBjAG8AcgBlAHMAXwBTAGMAbwBwAGUAMwBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAYgBsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARABhAHQAYQBTAGMAbwByAGUAcwBfAFMAYwBvAHAAZQAzAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBEAGEAdABhAFMAYwBvAHIAZQBzAF8AUwBjAG8AcABlADMAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAEwARQBBAEMASABfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMATABFAEEAQwBIAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAbABlAGEAYwBoAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAGwAZQBhAGMAaABfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBsAGUAYQBjAGgAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAE4AMgBPAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYATgAyAE8AXwBEAGEAdABhACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBOADIATwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAHIAYQBjAFcARQBUAEkAcgByAGkAZwBhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAFMAbwB1AHIAYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAE4ASQBSAFIAZQBmAGUAcgBlAG4AYwBlACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAcgBhAGMAVwBFAFQASQByAHIAaQBnAGEAdABpAG8AbgBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgByAGEAYwBXAEUAVABJAHIAcgBpAGcAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAEMAbwBtAG0AbwBuAF8AUwBvAHUAcgBjAGUARABhAHQAYQBfAEUARgBQAGEAcwB0AHUAcgBlAFIAYQBuAGcAZQBBAG4AZABQAGEAZABkAG8AYwBrAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBDAG8AbQBtAG8AbgBfAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBFAEYAUABhAHMAdAB1AHIAZQBSAGEAbgBnAGUAQQBuAGQAUABhAGQAZABvAGMAawBfAEQAYQB0AGEAIgAsACIAQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AQwBvAG0AbQBvAG4AXwBTAG8AdQByAGMAZQBEAGEAdABhAF8ARQBGAFAAYQBzAHQAdQByAGUAUgBhAG4AZwBlAEEAbgBkAFAAYQBkAGQAbwBjAGsAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQATgAyAE8AVABvAEMATwAyAGUAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8AVQBuAGkAdAAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AE4AMgBPAFQAbwBDAE8AMgBlAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABOADIATwBUAG8AQwBPADIAZQBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAIgAsACIAQwBvAG0AbQBvAG4AXwBFAHEAdQBhAHQAaQBvAG4AcwAuAEMAbwBtAG0AbwBuAF8AQwBvAG4AdgBlAHIAdABDAEgANABUAG8AQwBPADIAZQBfAFQAaQB0AGwAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAF8ARQBxAHUAYQB0AGkAbwBuAHMALgBDAG8AbQBtAG8AbgBfAEMAbwBuAHYAZQByAHQAQwBIADQAVABvAEMATwAyAGUAXwBOAEkAUgBSAGUAZgBlAHIAZQBuAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8ATABhAHQAZQB4AEUAcQB1AGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEUAcQB1AGEAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBDAG8AbgB2AGUAcgB0AEMASAA0AFQAbwBDAE8AMgBlAF8AQQByAGcAdQBtAGUAbgB0AHMAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBXAEUAVABNAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBGAHIAYQBjAFcARQBUAE0ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8AVABpAHQAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBVAG4AaQB0ACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8ARgByAGEAYwBMAEUAQQBDAEgAXwBNAFMAXwBTAG8AdQByAGMAZQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAEYAcgBhAGMATABFAEEAQwBIAF8ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBMAGkAdgBlAHMAdABvAGMAawBfAFMAbwB1AHIAYwBlAEQAYQB0AGEALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ATABpAHYAZQBzAHQAbwBjAGsAXwBDAG8AbQBtAG8AbgBfAFMAeQBtAGIAbwBsAHMATQBNAFMAXwBUAGkAdABsAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AVgBhAGkAcgBhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAEwAaQB2AGUAcwB0AG8AYwBrAF8AUwBvAHUAcgBjAGUARABhAHQAYQAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBMAGkAdgBlAHMAdABvAGMAawBfAEMAbwBtAG0AbwBuAF8AUwB5AG0AYgBvAGwAcwBNAE0AUwBfAFUAbgBpAHQAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8AUwBvAHUAcgBjAGUAIgAsACIAQwBvAG0AbQBvAG4ATABpAHYAZQBzAHQAbwBjAGsAXwBTAG8AdQByAGMAZQBEAGEAdABhAC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEwAaQB2AGUAcwB0AG8AYwBrAF8AQwBvAG0AbQBvAG4AXwBTAHkAbQBiAG8AbABzAE0ATQBTAF8ARABhAHQAYQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAFIAbwB3AFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBHAGUAdABBAHIAcgBhAHkAVABhAGIAbABlAEMAbwBsAHUAbQBuAFMAdABhAHIAdABOAHUAbQBiAGUAcgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgByAGEAeQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAE4AdQBtAGIAZQByACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEwAbwBvAGsAdQBwAFYAYQBsAHUAZQBJAG4AVABhAGIAbABlAFQAdwBvAEMAbwBsAHUAbQBuAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ATABvAG8AawB1AHAAVgBhAGwAdQBlAEkAbgBUAGEAYgBsAGUATwBuAGUAQwBvAGwAdQBtAG4AQQBuAGQASABlAGEAZABlAHIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwBwAGwAaQB0AFMAdAByAGkAbgBnAEkAbgB0AG8AQQByAHIAYQB5ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AVQB0AGkAbABpAHQAeQBfAEcAZQB0AEMAbABpAG0AYQB0AGUAWgBvAG4AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABJAHQAZQBtAEYAcgBvAG0ATQBpAG4ATQBhAHgAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8AUwB1AG0AUQB1AGEAbgB0AGkAdAB5AEYAcgBvAG0AQwByAGkAdABlAHIAaQBhACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAEMAeQBjAGwAZQBzACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AZwBlAHQATwB2AGUAcgBsAGEAcABwAGkAbgBnAFIAZQBwAG8AcgB0AGkAbgBnAFAAZQByAGkAbwBkAHMAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBGAHUAbgBjAHQAaQBvAG4ATgBhAG0AZQAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBMAG8AbwBrAHUAcABOADIATwBFAEYARgByAG8AbQBQAHIAbwBkAEkAcgByAGkAZwBhAHQAaQBvAG4AUgBhAGkAbgBmAGEAbABsACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AQwByAG8AcABwAGkAbgBnAF8ARwBlAHQARgByAGEAYwBXAEUAVAAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBDAG8AbgB2AGUAcgB0AFMAdABhAHQAZQBDAG8AbQBtAG8AbgBOAGEAbQBlAFQAbwBBAGIAYgByAGUAdgBpAGEAdABpAG8AbgAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBTAG8AdQByAGMAZQBIAHkAcABlAHIAbABpAG4AawAiACwAIgBDAG8AbQBtAG8AbgBfAEkAbgBwAHUAdABGAHUAbgBjAHQAaQBvAG4AcwAuAFUAdABpAGwAaQB0AHkAXwBEAGkAcwBwAGwAYQB5AEEAcgBnAHUAbQBlAG4AdABzAF8AMQBfADIAIgAsACIAQwBvAG0AbQBvAG4AXwBJAG4AcAB1AHQARgB1AG4AYwB0AGkAbwBuAHMALgBVAHQAaQBsAGkAdAB5AF8ARABpAHMAcABsAGEAeQBBAHIAZwB1AG0AZQBuAHQAcwBfADMAXwA0ACIALAAiAEMAbwBtAG0AbwBuAF8ASQBuAHAAdQB0AEYAdQBuAGMAdABpAG8AbgBzAC4AQwBvAG0AbQBvAG4AXwBHAGUAdABNAEMARgBUAGUAbQBwAGUAcgBhAHQAdQByAGUAWgBvAG4AZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AVgBTAEwAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBWAFMATABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAFYAUwBMAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0ATQBTAG0AMQBUADMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBNAFMAbQAxAFQAMwBfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAE0AUwBtADEAVAAzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAcwBoAEMAbwBuAHQAZQBuAHQAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AQQBzAGgAQwBvAG4AdABlAG4AdABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAHMAaABDAG8AbgB0AGUAbgB0AF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFQAaQB0AGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQBiAGwAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AZQB0AGgAYQBuAGUARQBtAGkAcwBzAGkAbwBuAHMAUABvAHQAZQBuAHQAaQBhAGwAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATQBlAHQAaABhAG4AZQBFAG0AaQBzAHMAaQBvAG4AcwBQAG8AdABlAG4AdABpAGEAbABfAFYAYQByAGkAYQB0AGkAbwBuACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAGUAdABoAGEAbgBlAEUAbQBpAHMAcwBpAG8AbgBzAFAAbwB0AGUAbgB0AGkAYQBsAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADEATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADIATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8AUwB0AGEAZwBlADMATQBNAFMATwBwAHQAaQBvAG4AcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATABpAHYAZQBzAHQAbwBjAGsAQwBsAGEAcwBzAGUAcwAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAHUAcgBhAHQAaQBvAG4ATwBmAFMAdABhAHkAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARAB1AHIAYQB0AGkAbwBuAE8AZgBTAHQAYQB5AF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAdQByAGEAdABpAG8AbgBPAGYAUwB0AGEAeQBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBBAG4AaQBtAGEAbABDAGgAYQByAGEAYwB0AGUAcgBpAHMAdABpAGMAcwBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEEAbgBpAG0AYQBsAEMAaABhAHIAYQBjAHQAZQByAGkAcwB0AGkAYwBzAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBVAG4AaQB0ACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBEAGkAZQB0AFAAcgBvAHAAZQByAHQAaQBlAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARABpAGUAdABQAHIAbwBwAGUAcgB0AGkAZQBzAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEQAaQBlAHQAUAByAG8AcABlAHIAdABpAGUAcwBfAEQAYQB0AGEAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBNAEMARgBfAFUAbgBpAHQAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AUwBvAHUAcgBjAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE0AQwBGAF8ARABhAHQAYQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBUAGkAdABsAGUAIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAE4AaQB0AHIAbwB1AHMATwB4AGkAZABlAEUARgBzAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBTAG8AdQByAGMAZQAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBWAGEAcgBpAGEAdABpAG8AbgAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ATgBpAHQAcgBvAHUAcwBPAHgAaQBkAGUARQBGAHMAXwBEAGEAdABhACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVABpAHQAbABlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVQBuAGkAdAAiACwAIgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdAAuAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AF8ARgByAGEAYwBOAFYAbwBsAGEAdABpAGwAaQBzAGUAZABfAFMAbwB1AHIAYwBlACIALAAiAFMAbwB1AHIAYwBlAEQAYQB0AGEAXwBGAGUAZQBkAGwAbwB0AC4AUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQAXwBGAHIAYQBjAE4AVgBvAGwAYQB0AGkAbABpAHMAZQBkAF8AVgBhAHIAaQBhAHQAaQBvAG4AIgAsACIAUwBvAHUAcgBjAGUARABhAHQAYQBfAEYAZQBlAGQAbABvAHQALgBTAG8AdQByAGMAZQBEAGEAdABhAF8ARgBlAGUAZABsAG8AdABfAEYAcgBhAGMATgBWAG8AbABhAHQAaQBsAGkAcwBlAGQAXwBEAGEAdABhACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADEAXwBUAG8AdABhAGwAQQBuAG4AdQBhAGwATQBlAHQAaABhAG4AZQBGAHIAbwBtAEUAbgB0AGUAcgBpAGMARgBlAHIAbQBlAG4AdABhAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAxAF8AVABvAHQAYQBsAEEAbgBuAHUAYQBsAE0AZQB0AGgAYQBuAGUARgByAG8AbQBFAG4AdABlAHIAaQBjAEYAZQByAG0AZQBuAHQAYQB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMQBfAFQAbwB0AGEAbABBAG4AbgB1AGEAbABNAGUAdABoAGEAbgBlAEYAcgBvAG0ARQBuAHQAZQByAGkAYwBGAGUAcgBtAGUAbgB0AGEAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAFQAaQB0AGwAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8AVgBhAHIAaQBhAGIAbABlACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBVAG4AaQB0ACIALAAiAEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBfAEYAZQBlAGQAbABvAHQAXwBFAHEAdQBhAHQAaQBvAG4AcwAuAFYARQBFAFIARwBfADMAXwAxAF8AMQBfADEAXwBfADIAXwBEAGEAaQBsAHkARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAFAAcgBvAGQAdQBjAHQAaQBvAG4AXwBTAG8AdQByAGMAZQAiACwAIgBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAXwBGAGUAZQBkAGwAbwB0AF8ARQBxAHUAYQB0AGkAbwBuAHMALgBWAEUARQBSAEcAXwAzAF8AMQBfADEAXwAxAF8AXwAyAF8ARABhAGkAbAB5AEUAbgB0AGUAcgBpAGMATQBlAHQAaABhAG4AZQBQAHIAbwBkAHUAYwB0AGkAbwBuAF8ATgBJAFIAUgBlAGYAZQByAGUAbgBjAGUAIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEwAYQB0AGUAeABFAHEAdQBhAHQAaQBvAG4AIgAsACIARQBuAHQAZQByAGkAYwBNAGUAdABoAGEAbgBlAF8ARgBlAGUAZABsAG8AdABfAEUAcQB1AGEAdABpAG8AbgBzAC4AVgBFAEUAUgBHAF8AMwBfADEAXwAxAF8AMQBfAF8AMgBfAEQAYQBpAGwAeQBFAG4AdABlAHIAaQBjAE0AZQB0AGgAYQBuAGUAUAByAG8AZAB1AGMAdABpAG8AbgBfAEEAcgBnAHUAbQBlAG4AdABzACIAXQAsACIAbABvAGMAYQBsAGUAIgA6AHsAIgBsAGkAcwB0AFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAcgBvAHcAUwBlAHAAYQByAGEAdABvAHIAIgA6ACIAOwAiACwAIgBjAG8AbAB1AG0AbgBTAGUAcABhAHIAYQB0AG8AcgAiADoAIgAsACIALAAiAHQAaABvAHUAcwBhAG4AZABzAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiACwAIgAsACIAdABoAG8AdQBzAGEAbgBkAHMAUABvAHMAaQB0AGkAbwBuAHMAIgA6AFsAMwBdACwAIgBkAGUAYwBpAG0AYQBsAFMAZQBwAGEAcgBhAHQAbwByACIAOgAiAC4AIgAsACIAZABhAHQAZQBPAHIAZABlAHIAIgA6ACIARABNAFkAIgAsACIAYwB1AHIAcgBlAG4AYwB5AFMAeQBtAGIAbwBsACIAOgAiACQAIgAsACIAaQBzAEMAdQByAHIAZQBuAGMAeQBTAHkAbQBiAG8AbABMAGUAYQBkACIAOgB0AHIAdQBlACwAIgBpAHMAQwB1AHIAcgBlAG4AYwB5AFMAZQBwAEIAeQBTAHAAYQBjAGUAIgA6AGYAYQBsAHMAZQAsACIAcgBvAHcATABlAHQAdABlAHIAIgA6ACIAUgAiACwAIgBjAG8AbAB1AG0AbgBMAGUAdAB0AGUAcgAiADoAIgBDACIALAAiAHIAYwBMAGUAZgB0AEIAcgBhAGMAawBlAHQAIgA6ACIAWwAiACwAIgByAGMAUgBpAGcAaAB0AEIAcgBhAGMAawBlAHQAIgA6ACIAXQAiACwAIgBzAHQAYQB0AGUAbQBlAG4AdABTAGUAcABhAHIAYQB0AG8AcgAiADoAIgA7ACIALAAiAGwAbwBjAGEAbABlAE4AYQBtAGUAIgA6ACIAZQBuAC0AdQBzACIAfQB9AA==</AFEJSONBlob>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CD460F9D-420A-4723-B323-396E4D19EC9B}">
   <ds:schemaRefs>
@@ -23163,6 +23169,22 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{809E3D44-A88D-4EBF-A307-6B8CE77A3361}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -23179,20 +23201,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9A9CF321-0D35-4044-BC72-33748FE2B865}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps4.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B6BE249C-20B1-4A62-BBCD-F2A46D88BCAB}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.advancedformulaenvironment.officeapps.live.com/afejsonblob/1.0"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>